<commit_message>
update: add non-duplicate Daily Brief records DCBM-119 to DCBM-121
</commit_message>
<xml_diff>
--- a/00_Master/Deep_CBM_Latest.xlsx
+++ b/00_Master/Deep_CBM_Latest.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Research\Deep_CBM_Knowledge_Base\00_Master\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3115A6B0-8F78-42DD-8E6C-B2F4C169565D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1912C42A-662A-4CDD-BDFE-1B9454C6A448}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1644" yWindow="0" windowWidth="15372" windowHeight="12240" firstSheet="1" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="完整文献矩阵" sheetId="1" r:id="rId1"/>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5767" uniqueCount="2787">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5908" uniqueCount="2879">
   <si>
     <t>序号</t>
   </si>
@@ -8984,12 +8984,303 @@
   <si>
     <t>新增13篇基于官方题录/DOI初步核验；全文精读后可继续补充定量参数与局限性。</t>
   </si>
+  <si>
+    <t>DCBM-119</t>
+  </si>
+  <si>
+    <t>ZhiDi Liu</t>
+  </si>
+  <si>
+    <t>ZhiDi Liu; Duo Wang; Binrui Yang; Jidong Tang; Chengwang Wang; Wei Wang; Xinsi Hu; Jingnan Zhang</t>
+  </si>
+  <si>
+    <t>Evaluating deep coal rock gas fracturing sweet spot intervals using PSO-ELM algorithm and petrophysical logging data</t>
+  </si>
+  <si>
+    <t>基于 PSO-ELM 算法与岩石物理测井资料的深部煤岩气压裂甜点段评价</t>
+  </si>
+  <si>
+    <t>Early access article</t>
+  </si>
+  <si>
+    <t>10.1038/s41598-026-54924-z</t>
+  </si>
+  <si>
+    <t>https://www.nature.com/articles/s41598-026-54924-z</t>
+  </si>
+  <si>
+    <t>Journal article</t>
+  </si>
+  <si>
+    <t>Ordos Basin; Daning-Jixian Block</t>
+  </si>
+  <si>
+    <t>Deep coal rock gas; No. 5 and No. 8 coal seams</t>
+  </si>
+  <si>
+    <t>深部煤岩气储层</t>
+  </si>
+  <si>
+    <t>识别深部煤岩气压裂甜点段</t>
+  </si>
+  <si>
+    <t>PSO-ELM、测井资料、10 个地质工程控制因素、甜点分级</t>
+  </si>
+  <si>
+    <t>X-11 井预测准确率超过 85%；I、II 类甜点段资源丰富</t>
+  </si>
+  <si>
+    <t>将 PSO-ELM 用于地质工程一体化压裂甜点评价</t>
+  </si>
+  <si>
+    <t>跨区块泛化需验证；机器学习可解释性需增强</t>
+  </si>
+  <si>
+    <t>可作为响应差异的地质工程背景变量参考</t>
+  </si>
+  <si>
+    <t>第二章；第三章；第五章</t>
+  </si>
+  <si>
+    <t>PSO-ELM; fracturing sweet spot; logging; geologic-engineering integration</t>
+  </si>
+  <si>
+    <t>Nature 页面、DOI、题名、作者、摘要已核验</t>
+  </si>
+  <si>
+    <t>DCBM-120</t>
+  </si>
+  <si>
+    <t>Hui Pan</t>
+  </si>
+  <si>
+    <t>Hui Pan; Wanjin Zhao; Mengbo Zhang; Run He; Guoliang Yan; Dongyang He</t>
+  </si>
+  <si>
+    <t>Prediction Methods for Gas-bearing Properties in Deep Coal Measures in the Ordos Basin</t>
+  </si>
+  <si>
+    <t>鄂尔多斯盆地深部煤系含气性预测方法</t>
+  </si>
+  <si>
+    <t>Journal of Geophysics and Engineering</t>
+  </si>
+  <si>
+    <t>gxag082</t>
+  </si>
+  <si>
+    <t>10.1093/jge/gxag082</t>
+  </si>
+  <si>
+    <t>https://academic.oup.com/jge/advance-article/doi/10.1093/jge/gxag082/8708932</t>
+  </si>
+  <si>
+    <t>Advance article / accepted manuscript</t>
+  </si>
+  <si>
+    <t>Ordos Basin</t>
+  </si>
+  <si>
+    <t>Deep coal measures; No. 8 coal seam</t>
+  </si>
+  <si>
+    <t>No. 8 seam thickness 6-16 m, average 7.8 m</t>
+  </si>
+  <si>
+    <t>建立深部煤系含气性预测方法</t>
+  </si>
+  <si>
+    <t>地质约束、岩石物理、Bayesian AVO、频变地震反演</t>
+  </si>
+  <si>
+    <t>新评价参数可增强气敏感性和岩性区分能力，提高含气性预测精度</t>
+  </si>
+  <si>
+    <t>面向煤系气的地质—岩石物理—频变反演框架</t>
+  </si>
+  <si>
+    <t>依赖高质量地震和井震标定；与生产动态关联需进一步建立</t>
+  </si>
+  <si>
+    <t>可作为地质背景变量和含气性解释依据</t>
+  </si>
+  <si>
+    <t>gas-bearing prediction; deep coal measures; Ordos Basin; seismic inversion</t>
+  </si>
+  <si>
+    <t>Oxford 页面、DOI、题名、作者、摘要已核验</t>
+  </si>
+  <si>
+    <t>DCBM-121</t>
+  </si>
+  <si>
+    <t>YANG Jiaosheng; WANG Nan; WANG Meizhu; DENG Jia; LU Xiuqin; SONG Hongqing</t>
+  </si>
+  <si>
+    <t>Productivity prediction and production performances of deep coalbed methane horizontal wells throughout full life cycle</t>
+  </si>
+  <si>
+    <t>深部煤层气水平井全生命周期产能预测与生产动态</t>
+  </si>
+  <si>
+    <t>3551-3561</t>
+  </si>
+  <si>
+    <t>10.13225/j.cnki.jccs.QH25.0479</t>
+  </si>
+  <si>
+    <t>https://www.mtxb.com.cn/en/article/doi/10.13225/j.cnki.jccs.QH25.0479</t>
+  </si>
+  <si>
+    <t>Deep CBM fractured horizontal well</t>
+  </si>
+  <si>
+    <t>建立全生命周期产能预测模型</t>
+  </si>
+  <si>
+    <t>Langmuir 等温吸附、气水两相两区流、10 年生产预测</t>
+  </si>
+  <si>
+    <t>早期游离气贡献高；后期解吸气贡献升高；10 年累产中解吸气 63.54%、游离气 36.46%</t>
+  </si>
+  <si>
+    <t>将游离气—解吸气动态贡献纳入深部煤层气水平井全生命周期预测</t>
+  </si>
+  <si>
+    <t>参数不确定性较高；需结合现场排采制度进一步验证</t>
+  </si>
+  <si>
+    <t>强相关，可解释早期响应和中长期产能关系</t>
+  </si>
+  <si>
+    <t>第二章；第四章；第五章</t>
+  </si>
+  <si>
+    <t>productivity prediction; full life cycle; free gas; desorbed gas; horizontal well</t>
+  </si>
+  <si>
+    <t>煤炭学报页面、DOI、卷期页码、摘要已核验</t>
+  </si>
+  <si>
+    <t>研究区/对象：Ordos Basin; Daning-Jixian Block；Deep coal rock gas; No. 5 and No. 8 coal seams；深度：深部煤岩气储层。</t>
+  </si>
+  <si>
+    <t>【研究目的】识别深部煤岩气压裂甜点段
+【数据/方法】PSO-ELM、测井资料、10 个地质工程控制因素、甜点分级
+【核心发现】X-11 井预测准确率超过 85%；I、II 类甜点段资源丰富
+【创新点】将 PSO-ELM 用于地质工程一体化压裂甜点评价
+【局限性】跨区块泛化需验证；机器学习可解释性需增强
+【与你课题的关系】可作为响应差异的地质工程背景变量参考</t>
+  </si>
+  <si>
+    <t>研究区/对象：Ordos Basin；Deep coal measures; No. 8 coal seam；深度：No. 8 seam thickness 6-16 m, average 7.8 m。</t>
+  </si>
+  <si>
+    <t>【研究目的】建立深部煤系含气性预测方法
+【数据/方法】地质约束、岩石物理、Bayesian AVO、频变地震反演
+【核心发现】新评价参数可增强气敏感性和岩性区分能力，提高含气性预测精度
+【创新点】面向煤系气的地质—岩石物理—频变反演框架
+【局限性】依赖高质量地震和井震标定；与生产动态关联需进一步建立
+【与你课题的关系】可作为地质背景变量和含气性解释依据</t>
+  </si>
+  <si>
+    <t>研究区/对象：Ordos Basin; Daning-Jixian Block；Deep CBM fractured horizontal well；深度：深部煤层气储层。</t>
+  </si>
+  <si>
+    <t>【研究目的】建立全生命周期产能预测模型
+【数据/方法】Langmuir 等温吸附、气水两相两区流、10 年生产预测
+【核心发现】早期游离气贡献高；后期解吸气贡献升高；10 年累产中解吸气 63.54%、游离气 36.46%
+【创新点】将游离气—解吸气动态贡献纳入深部煤层气水平井全生命周期预测
+【局限性】参数不确定性较高；需结合现场排采制度进一步验证
+【与你课题的关系】强相关，可解释早期响应和中长期产能关系</t>
+  </si>
+  <si>
+    <t>2026-07-09 Daily Brief corrected update</t>
+  </si>
+  <si>
+    <t>Added DCBM-119 to DCBM-121</t>
+  </si>
+  <si>
+    <t>Skipped duplicate candidate</t>
+  </si>
+  <si>
+    <t>flowback characteristics, existing DCBM-028</t>
+  </si>
+  <si>
+    <t>Master record count</t>
+  </si>
+  <si>
+    <t>118 -&gt; 121</t>
+  </si>
+  <si>
+    <t>Daily Brief</t>
+  </si>
+  <si>
+    <t>09_Daily_Brief/2026-07-09/Deep_CBM_daily_brief_20260709.md</t>
+  </si>
+  <si>
+    <t>原DCBM-119</t>
+  </si>
+  <si>
+    <t>10.3389/feart.2026.1772109 / Evaluation of development effectiveness of deep coalbed methane based on flowback characteristics-a case study of the Daning-Jixian block</t>
+  </si>
+  <si>
+    <t>DOI完全一致；英文题名一致；中文题名一致</t>
+  </si>
+  <si>
+    <t>跳过</t>
+  </si>
+  <si>
+    <t>原DCBM-120</t>
+  </si>
+  <si>
+    <t>10.1038/s41598-026-54924-z / Evaluating deep coal rock gas fracturing sweet spot intervals using PSO-ELM algorithm and petrophysical logging data</t>
+  </si>
+  <si>
+    <t>不重复</t>
+  </si>
+  <si>
+    <t>DOI、英文题名、中文题名、作者年份均未检出</t>
+  </si>
+  <si>
+    <t>原DCBM-121</t>
+  </si>
+  <si>
+    <t>10.1093/jge/gxag082 / Prediction Methods for Gas-bearing Properties in Deep Coal Measures in the Ordos Basin</t>
+  </si>
+  <si>
+    <t>原DCBM-122</t>
+  </si>
+  <si>
+    <t>10.13225/j.cnki.jccs.QH25.0479 / Productivity prediction and production performances of deep coalbed methane horizontal wells throughout full life cycle</t>
+  </si>
+  <si>
+    <t>Daily Brief corrected</t>
+  </si>
+  <si>
+    <t>PASS</t>
+  </si>
+  <si>
+    <t>Added records</t>
+  </si>
+  <si>
+    <t>DCBM-119 to DCBM-121</t>
+  </si>
+  <si>
+    <t>Skipped duplicate</t>
+  </si>
+  <si>
+    <t>Original DCBM-119 already exists as DCBM-028</t>
+  </si>
+  <si>
+    <t>Duplicate DOI/title check</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <sz val="11"/>
       <name val="Carlito"/>
@@ -9009,6 +9300,12 @@
       <name val="宋体"/>
       <family val="3"/>
       <charset val="134"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Carlito"/>
     </font>
   </fonts>
   <fills count="8">
@@ -9065,11 +9362,12 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="1" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -9091,10 +9389,14 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="6" borderId="1" xfId="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="7" borderId="1" xfId="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="2" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="2">
+  <cellStyles count="3">
     <cellStyle name="Normal" xfId="1" xr:uid="{00000000-0005-0000-0000-000000000000}"/>
     <cellStyle name="常规" xfId="0" builtinId="0"/>
+    <cellStyle name="超链接" xfId="2" builtinId="8"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -9309,7 +9611,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AA119"/>
+  <dimension ref="A1:AA122"/>
   <sheetFormatPr defaultRowHeight="13.8"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
@@ -19150,11 +19452,257 @@
         <v>2217</v>
       </c>
     </row>
+    <row r="120" spans="1:27" ht="41.4">
+      <c r="A120" s="1">
+        <v>119</v>
+      </c>
+      <c r="B120" s="1" t="s">
+        <v>2787</v>
+      </c>
+      <c r="C120" s="1" t="s">
+        <v>2788</v>
+      </c>
+      <c r="D120" s="1" t="s">
+        <v>2789</v>
+      </c>
+      <c r="E120" s="1">
+        <v>2026</v>
+      </c>
+      <c r="F120" s="1" t="s">
+        <v>2790</v>
+      </c>
+      <c r="G120" s="1" t="s">
+        <v>2791</v>
+      </c>
+      <c r="H120" s="1" t="s">
+        <v>638</v>
+      </c>
+      <c r="I120" s="1"/>
+      <c r="J120" s="1"/>
+      <c r="K120" s="1" t="s">
+        <v>2792</v>
+      </c>
+      <c r="L120" s="1" t="s">
+        <v>2793</v>
+      </c>
+      <c r="M120" s="9" t="s">
+        <v>2794</v>
+      </c>
+      <c r="N120" s="1" t="s">
+        <v>2795</v>
+      </c>
+      <c r="O120" s="1" t="s">
+        <v>2796</v>
+      </c>
+      <c r="P120" s="1" t="s">
+        <v>2797</v>
+      </c>
+      <c r="Q120" s="1" t="s">
+        <v>2798</v>
+      </c>
+      <c r="R120" s="1" t="s">
+        <v>2799</v>
+      </c>
+      <c r="S120" s="1" t="s">
+        <v>2800</v>
+      </c>
+      <c r="T120" s="1" t="s">
+        <v>2801</v>
+      </c>
+      <c r="U120" s="1" t="s">
+        <v>2802</v>
+      </c>
+      <c r="V120" s="1" t="s">
+        <v>2803</v>
+      </c>
+      <c r="W120" s="1" t="s">
+        <v>2804</v>
+      </c>
+      <c r="X120" s="1" t="s">
+        <v>2805</v>
+      </c>
+      <c r="Y120" s="1" t="s">
+        <v>2806</v>
+      </c>
+      <c r="Z120" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="AA120" s="1" t="s">
+        <v>2807</v>
+      </c>
+    </row>
+    <row r="121" spans="1:27" ht="41.4">
+      <c r="A121" s="1">
+        <v>120</v>
+      </c>
+      <c r="B121" s="1" t="s">
+        <v>2808</v>
+      </c>
+      <c r="C121" s="1" t="s">
+        <v>2809</v>
+      </c>
+      <c r="D121" s="1" t="s">
+        <v>2810</v>
+      </c>
+      <c r="E121" s="1">
+        <v>2026</v>
+      </c>
+      <c r="F121" s="1" t="s">
+        <v>2811</v>
+      </c>
+      <c r="G121" s="1" t="s">
+        <v>2812</v>
+      </c>
+      <c r="H121" s="1" t="s">
+        <v>2813</v>
+      </c>
+      <c r="I121" s="1"/>
+      <c r="J121" s="1"/>
+      <c r="K121" s="1" t="s">
+        <v>2814</v>
+      </c>
+      <c r="L121" s="1" t="s">
+        <v>2815</v>
+      </c>
+      <c r="M121" s="9" t="s">
+        <v>2816</v>
+      </c>
+      <c r="N121" s="1" t="s">
+        <v>2817</v>
+      </c>
+      <c r="O121" s="1" t="s">
+        <v>2818</v>
+      </c>
+      <c r="P121" s="1" t="s">
+        <v>2819</v>
+      </c>
+      <c r="Q121" s="1" t="s">
+        <v>2820</v>
+      </c>
+      <c r="R121" s="1" t="s">
+        <v>2821</v>
+      </c>
+      <c r="S121" s="1" t="s">
+        <v>2822</v>
+      </c>
+      <c r="T121" s="1" t="s">
+        <v>2823</v>
+      </c>
+      <c r="U121" s="1" t="s">
+        <v>2824</v>
+      </c>
+      <c r="V121" s="1" t="s">
+        <v>2825</v>
+      </c>
+      <c r="W121" s="1" t="s">
+        <v>2826</v>
+      </c>
+      <c r="X121" s="1" t="s">
+        <v>2805</v>
+      </c>
+      <c r="Y121" s="1" t="s">
+        <v>2827</v>
+      </c>
+      <c r="Z121" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="AA121" s="1" t="s">
+        <v>2828</v>
+      </c>
+    </row>
+    <row r="122" spans="1:27" ht="41.4">
+      <c r="A122" s="1">
+        <v>121</v>
+      </c>
+      <c r="B122" s="1" t="s">
+        <v>2829</v>
+      </c>
+      <c r="C122" s="1" t="s">
+        <v>1477</v>
+      </c>
+      <c r="D122" s="1" t="s">
+        <v>2830</v>
+      </c>
+      <c r="E122" s="1">
+        <v>2026</v>
+      </c>
+      <c r="F122" s="1" t="s">
+        <v>2831</v>
+      </c>
+      <c r="G122" s="1" t="s">
+        <v>2832</v>
+      </c>
+      <c r="H122" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="I122" s="1">
+        <v>51</v>
+      </c>
+      <c r="J122" s="1">
+        <v>6</v>
+      </c>
+      <c r="K122" s="1" t="s">
+        <v>2833</v>
+      </c>
+      <c r="L122" s="1" t="s">
+        <v>2834</v>
+      </c>
+      <c r="M122" s="9" t="s">
+        <v>2835</v>
+      </c>
+      <c r="N122" s="1" t="s">
+        <v>2795</v>
+      </c>
+      <c r="O122" s="1" t="s">
+        <v>2796</v>
+      </c>
+      <c r="P122" s="1" t="s">
+        <v>2836</v>
+      </c>
+      <c r="Q122" s="1" t="s">
+        <v>341</v>
+      </c>
+      <c r="R122" s="1" t="s">
+        <v>2837</v>
+      </c>
+      <c r="S122" s="1" t="s">
+        <v>2838</v>
+      </c>
+      <c r="T122" s="1" t="s">
+        <v>2839</v>
+      </c>
+      <c r="U122" s="1" t="s">
+        <v>2840</v>
+      </c>
+      <c r="V122" s="1" t="s">
+        <v>2841</v>
+      </c>
+      <c r="W122" s="1" t="s">
+        <v>2842</v>
+      </c>
+      <c r="X122" s="1" t="s">
+        <v>2843</v>
+      </c>
+      <c r="Y122" s="1" t="s">
+        <v>2844</v>
+      </c>
+      <c r="Z122" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="AA122" s="1" t="s">
+        <v>2845</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>
+  <hyperlinks>
+    <hyperlink ref="M120" r:id="rId1" xr:uid="{CC16D580-FDCE-4E16-95A4-6D8C719BCB74}"/>
+    <hyperlink ref="M121" r:id="rId2" xr:uid="{61B660BB-0451-434D-861F-5A2A7A017BCD}"/>
+    <hyperlink ref="M122" r:id="rId3" xr:uid="{BBC8EAEE-6B77-43F7-8540-3A99CD9FC4B3}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
-    <tablePart r:id="rId1"/>
+    <tablePart r:id="rId4"/>
   </tableParts>
 </worksheet>
 </file>
@@ -22427,7 +22975,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
-  <dimension ref="A1:N119"/>
+  <dimension ref="A1:N122"/>
   <sheetFormatPr defaultRowHeight="13.8"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -27680,6 +28228,120 @@
         <v>2515</v>
       </c>
     </row>
+    <row r="120" spans="1:14" ht="82.8">
+      <c r="A120" s="1" t="s">
+        <v>2787</v>
+      </c>
+      <c r="B120" s="1">
+        <v>2026</v>
+      </c>
+      <c r="C120" s="1" t="s">
+        <v>2791</v>
+      </c>
+      <c r="D120" s="1" t="s">
+        <v>2846</v>
+      </c>
+      <c r="E120" s="1" t="s">
+        <v>2847</v>
+      </c>
+      <c r="F120" s="1" t="s">
+        <v>2799</v>
+      </c>
+      <c r="G120" s="1" t="s">
+        <v>2800</v>
+      </c>
+      <c r="H120" s="1" t="s">
+        <v>2801</v>
+      </c>
+      <c r="I120" s="1" t="s">
+        <v>2802</v>
+      </c>
+      <c r="J120" s="1" t="s">
+        <v>2803</v>
+      </c>
+      <c r="K120" s="1"/>
+      <c r="L120" s="1"/>
+      <c r="M120" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="N120" s="1"/>
+    </row>
+    <row r="121" spans="1:14" ht="82.8">
+      <c r="A121" s="1" t="s">
+        <v>2808</v>
+      </c>
+      <c r="B121" s="1">
+        <v>2026</v>
+      </c>
+      <c r="C121" s="1" t="s">
+        <v>2812</v>
+      </c>
+      <c r="D121" s="1" t="s">
+        <v>2848</v>
+      </c>
+      <c r="E121" s="1" t="s">
+        <v>2849</v>
+      </c>
+      <c r="F121" s="1" t="s">
+        <v>2821</v>
+      </c>
+      <c r="G121" s="1" t="s">
+        <v>2822</v>
+      </c>
+      <c r="H121" s="1" t="s">
+        <v>2823</v>
+      </c>
+      <c r="I121" s="1" t="s">
+        <v>2824</v>
+      </c>
+      <c r="J121" s="1" t="s">
+        <v>2825</v>
+      </c>
+      <c r="K121" s="1"/>
+      <c r="L121" s="1"/>
+      <c r="M121" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="N121" s="1"/>
+    </row>
+    <row r="122" spans="1:14" ht="82.8">
+      <c r="A122" s="1" t="s">
+        <v>2829</v>
+      </c>
+      <c r="B122" s="1">
+        <v>2026</v>
+      </c>
+      <c r="C122" s="1" t="s">
+        <v>2832</v>
+      </c>
+      <c r="D122" s="1" t="s">
+        <v>2850</v>
+      </c>
+      <c r="E122" s="1" t="s">
+        <v>2851</v>
+      </c>
+      <c r="F122" s="1" t="s">
+        <v>2837</v>
+      </c>
+      <c r="G122" s="1" t="s">
+        <v>2838</v>
+      </c>
+      <c r="H122" s="1" t="s">
+        <v>2839</v>
+      </c>
+      <c r="I122" s="1" t="s">
+        <v>2840</v>
+      </c>
+      <c r="J122" s="1" t="s">
+        <v>2841</v>
+      </c>
+      <c r="K122" s="1"/>
+      <c r="L122" s="1"/>
+      <c r="M122" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="N122" s="1"/>
+    </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -27688,7 +28350,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:B11"/>
   <sheetFormatPr defaultRowHeight="13.8"/>
   <cols>
     <col min="1" max="2" width="50" customWidth="1"/>
@@ -27750,6 +28412,38 @@
         <v>2778</v>
       </c>
     </row>
+    <row r="8" spans="1:2">
+      <c r="A8" t="s">
+        <v>2852</v>
+      </c>
+      <c r="B8" t="s">
+        <v>2853</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2">
+      <c r="A9" t="s">
+        <v>2854</v>
+      </c>
+      <c r="B9" t="s">
+        <v>2855</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2">
+      <c r="A10" t="s">
+        <v>2856</v>
+      </c>
+      <c r="B10" t="s">
+        <v>2857</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2">
+      <c r="A11" t="s">
+        <v>2858</v>
+      </c>
+      <c r="B11" t="s">
+        <v>2859</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -27758,7 +28452,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
-  <dimension ref="A1:F17"/>
+  <dimension ref="A1:F21"/>
   <sheetFormatPr defaultRowHeight="13.8"/>
   <sheetData>
     <row r="1" spans="1:6" ht="27.6">
@@ -28099,6 +28793,86 @@
       </c>
       <c r="F17" s="1" t="s">
         <v>2765</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" ht="303.60000000000002">
+      <c r="A18" s="1" t="s">
+        <v>2860</v>
+      </c>
+      <c r="B18" s="1" t="s">
+        <v>2861</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>2757</v>
+      </c>
+      <c r="D18" s="1" t="s">
+        <v>2862</v>
+      </c>
+      <c r="E18" s="1" t="s">
+        <v>610</v>
+      </c>
+      <c r="F18" s="1" t="s">
+        <v>2863</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" ht="276">
+      <c r="A19" s="1" t="s">
+        <v>2864</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>2865</v>
+      </c>
+      <c r="C19" s="1" t="s">
+        <v>2866</v>
+      </c>
+      <c r="D19" s="1" t="s">
+        <v>2867</v>
+      </c>
+      <c r="E19" s="1" t="s">
+        <v>2787</v>
+      </c>
+      <c r="F19" s="1" t="s">
+        <v>2762</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" ht="193.2">
+      <c r="A20" s="1" t="s">
+        <v>2868</v>
+      </c>
+      <c r="B20" s="1" t="s">
+        <v>2869</v>
+      </c>
+      <c r="C20" s="1" t="s">
+        <v>2866</v>
+      </c>
+      <c r="D20" s="1" t="s">
+        <v>2867</v>
+      </c>
+      <c r="E20" s="1" t="s">
+        <v>2808</v>
+      </c>
+      <c r="F20" s="1" t="s">
+        <v>2762</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" ht="276">
+      <c r="A21" s="1" t="s">
+        <v>2870</v>
+      </c>
+      <c r="B21" s="1" t="s">
+        <v>2871</v>
+      </c>
+      <c r="C21" s="1" t="s">
+        <v>2866</v>
+      </c>
+      <c r="D21" s="1" t="s">
+        <v>2867</v>
+      </c>
+      <c r="E21" s="1" t="s">
+        <v>2829</v>
+      </c>
+      <c r="F21" s="1" t="s">
+        <v>2762</v>
       </c>
     </row>
   </sheetData>
@@ -28109,7 +28883,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0B00-000000000000}">
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:B11"/>
   <sheetFormatPr defaultRowHeight="13.8"/>
   <cols>
     <col min="1" max="2" width="42" customWidth="1"/>
@@ -28163,6 +28937,46 @@
         <v>2786</v>
       </c>
     </row>
+    <row r="7" spans="1:2">
+      <c r="A7" t="s">
+        <v>2872</v>
+      </c>
+      <c r="B7" t="s">
+        <v>2873</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2">
+      <c r="A8" t="s">
+        <v>2874</v>
+      </c>
+      <c r="B8" t="s">
+        <v>2875</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2">
+      <c r="A9" t="s">
+        <v>2876</v>
+      </c>
+      <c r="B9" t="s">
+        <v>2877</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2">
+      <c r="A10" t="s">
+        <v>2856</v>
+      </c>
+      <c r="B10" t="s">
+        <v>2857</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2">
+      <c r="A11" t="s">
+        <v>2878</v>
+      </c>
+      <c r="B11" t="s">
+        <v>2873</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
update: process Deep CBM daily brief 2026-07-24
- Added 2 new records: DCBM-135, DCBM-136
- DCBM-135: Qiang Guo — Seismic rock-physics inversion for deep CBM (J. Applied Geophysics)
- DCBM-136: Q. Zhang — North China CBM geochemistry and microbial methanogenesis (Fuel, 2027)
- 0 duplicates; all fields filled from RIS + prose
- Master: 134 -> 136, ID continuous, zero duplicates
- Protected dirs unmodified
</commit_message>
<xml_diff>
--- a/00_Master/Deep_CBM_Latest.xlsx
+++ b/00_Master/Deep_CBM_Latest.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView activeTab="5" autoFilterDateGrouping="1" firstSheet="0" minimized="0" showHorizontalScroll="1" showSheetTabs="1" showVerticalScroll="1" tabRatio="600" visibility="visible" windowHeight="12456" windowWidth="23256" xWindow="-108" yWindow="-108"/>
+    <workbookView activeTab="4" autoFilterDateGrouping="1" firstSheet="0" minimized="0" showHorizontalScroll="1" showSheetTabs="1" showVerticalScroll="1" tabRatio="600" visibility="visible" windowHeight="16776" windowWidth="30936" xWindow="-108" yWindow="-108"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="完整文献矩阵" sheetId="1" state="visible" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="3147">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="3198">
   <si>
     <t>序号</t>
   </si>
@@ -8326,6 +8326,135 @@
     <t>Nanoconfinement; coalbed methane; 吸附; 游离气; 纳米限域; 孔隙结构; 吸附热力学</t>
   </si>
   <si>
+    <t>DCBM-135</t>
+  </si>
+  <si>
+    <t>Guo, Qiang</t>
+  </si>
+  <si>
+    <t>Guo, Qiang; Chen, Yang; Huang, Yaping; Ba, Jing</t>
+  </si>
+  <si>
+    <t>Seismic rock-physics inversion for petrophysical parameters in deep coalbed methane reservoirs with complex pore structures</t>
+  </si>
+  <si>
+    <t>复杂孔隙结构深部煤层气储层岩石物理参数地震反演</t>
+  </si>
+  <si>
+    <t>Journal of Applied Geophysics</t>
+  </si>
+  <si>
+    <t>251</t>
+  </si>
+  <si>
+    <t>106338</t>
+  </si>
+  <si>
+    <t>10.1016/j.jappgeo.2026.106338</t>
+  </si>
+  <si>
+    <t>https://www.sciencedirect.com/science/article/abs/pii/S0926985126002478</t>
+  </si>
+  <si>
+    <t>鄂尔多斯盆地东缘；石炭系本溪组</t>
+  </si>
+  <si>
+    <t>深部煤层气储层（双重孔隙体系，埋深1500-2300 m）</t>
+  </si>
+  <si>
+    <t>1500-2300 m；平均厚度约12 m</t>
+  </si>
+  <si>
+    <t>构建考虑空间变化孔隙纵横比的岩石物理-地震反演框架，联合反演深部煤层储层物性参数</t>
+  </si>
+  <si>
+    <t>两口井测井资料；煤层及围岩岩石物理建模；空间可变孔隙纵横比；Taylor展开线性化正演；高斯混合模型多峰岩相统计；贝叶斯线性反演；总孔隙度/黏土体积分数/孔隙纵横比联合预测；二维地震剖面验证</t>
+  </si>
+  <si>
+    <t>固定孔隙纵横比难以描述深部煤层复杂双孔隙结构；空间变化孔隙纵横比可改善储层物性反演；高斯混合先验可处理多峰统计分布；实际二维地震资料可辅助识别含气煤层和储层物性变化</t>
+  </si>
+  <si>
+    <t>将孔隙几何参数与常规储层物性参数联合反演；空间变化孔隙纵横比表征深部煤层双孔隙复杂性；高斯混合统计先验与贝叶斯岩石物理反演结合</t>
+  </si>
+  <si>
+    <t>对初始模型和先验信息依赖较高；两口井和单一二维剖面限制泛化；等效孔隙纵横比是复杂孔裂隙体系的简化；地震反演只能提供间接储层证据</t>
+  </si>
+  <si>
+    <t>储层非均质性；裂缝-基质双重孔隙；多源资料融合的必要性；后续引入地震/测井和孔裂隙参数的理由</t>
+  </si>
+  <si>
+    <t>引言：深部煤储层复杂孔裂隙及预测难点；方法讨论：多源储层参数与地震反演；讨论：储层非均质性作为动态差异的替代解释；局限：间接地球物理证据不能替代生产因果验证</t>
+  </si>
+  <si>
+    <t>seismic inversion; rock physics; pore aspect ratio; deep coalbed methane; Bayesian inversion; Ordos Basin</t>
+  </si>
+  <si>
+    <t>出版商题名/作者/DOI/卷和文章号已核验</t>
+  </si>
+  <si>
+    <t>DCBM-136</t>
+  </si>
+  <si>
+    <t>Zhang, Q.</t>
+  </si>
+  <si>
+    <t>Zhang, Q.; Li, Y.; Tang, S.; Zhang, P.; Zhang, S.; Xi, Z.</t>
+  </si>
+  <si>
+    <t>2027 (online 2026)</t>
+  </si>
+  <si>
+    <t>Geochemical evolution and microbial controls on methanogenic potential in North China coalbed methane reservoirs: Implications for CBM bioengineering</t>
+  </si>
+  <si>
+    <t>华北煤层气藏地球化学演化与产甲烷潜力的微生物控制：对煤层气生物工程的启示</t>
+  </si>
+  <si>
+    <t>428</t>
+  </si>
+  <si>
+    <t>140384</t>
+  </si>
+  <si>
+    <t>10.1016/j.fuel.2026.140384</t>
+  </si>
+  <si>
+    <t>https://www.sciencedirect.com/science/article/abs/pii/S0016236126021393</t>
+  </si>
+  <si>
+    <t>华北4个煤层气区：沁水盆地南部、宁武盆地南部、鄂尔多斯盆地东缘神府区块、临兴区块</t>
+  </si>
+  <si>
+    <t>煤层气藏（69口生产井；不同埋深/煤阶/水动力条件）</t>
+  </si>
+  <si>
+    <t>研究华北煤层气藏地球化学演化与产甲烷潜力的微生物控制机制，评估煤层气生物工程潜力</t>
+  </si>
+  <si>
+    <t>69口生产井采样；产出气组分与甲烷碳氢同位素；产出水主要离子和水化学；溶解无机碳及其同位素；微生物群落分析；产甲烷功能基因；区域水动力封闭和盐度对比</t>
+  </si>
+  <si>
+    <t>4个研究区以热成因甲烷为主；沁水南部存在局部次生微生物改造信号；神府和临兴产出水盐度更高/Na-Cl富集/水动力封闭更强；沁水南部产甲烷菌多样性和功能基因更丰富；神府整体产甲烷功能基因丰度较低；水化学条件是限制微生物增产适用性的关键因素</t>
+  </si>
+  <si>
+    <t>联合气体/产出水/同位素/微生物群落和功能基因；在热成因气背景下识别局部次生生物成因改造；将区域水化学差异与微生物增产适用性直接联系；为晚期/低产井微生物增产筛选提供约束框架</t>
+  </si>
+  <si>
+    <t>微生物深入分析主要集中在沁水南部和神府/区域覆盖不完全对称；产出水微生物不一定完全代表原位煤基质微生物群落；69口井均为生产井/长期排采可能已改变原始水化学和微生物状态；产甲烷功能基因表明潜力不等同于现场增产效果</t>
+  </si>
+  <si>
+    <t>产出水化学和水动力封闭；区块差异及保存条件；长期排采后流体环境演化；生物成因与热成因气的区分；不能仅凭气水动态推断气源或微生物作用</t>
+  </si>
+  <si>
+    <t>引言：华北煤层气水化学和气源背景；讨论：产出水/盐度/封闭和区域差异；局限：生产动态不能直接识别气源或微生物机制；展望：低产/晚期井微生物增产的筛选与验证</t>
+  </si>
+  <si>
+    <t>CBM bioengineering; microbial methanogenesis; hydrogeochemistry; North China; Fuel; microbial community</t>
+  </si>
+  <si>
+    <t>出版商题名/DOI/卷期/摘要和研究设计已核验；作者缩写待Crossref补全</t>
+  </si>
+  <si>
     <t>指标</t>
   </si>
   <si>
@@ -8350,7 +8479,7 @@
     <t>当前主表版本</t>
   </si>
   <si>
-    <t>v1_134_daily_brief_update_2026-07-23</t>
+    <t>v1_136_daily_brief_update_2026-07-24</t>
   </si>
   <si>
     <t>Deep_CBM_complete_literature_matrix_v1_105.xlsx</t>
@@ -9925,6 +10054,18 @@
 【与你课题的关系】早期游离气贡献和相态评价边界。</t>
   </si>
   <si>
+    <t>【局限性】间接地球物理证据不能替代生产因果验证。</t>
+  </si>
+  <si>
+    <t>间接地球物理证据不能替代生产因果验证。</t>
+  </si>
+  <si>
+    <t>【局限性】生产动态不能直接识别气源或微生物机制；</t>
+  </si>
+  <si>
+    <t>生产动态不能直接识别气源或微生物机制；</t>
+  </si>
+  <si>
     <t>日期</t>
   </si>
   <si>
@@ -10000,6 +10141,12 @@
     <t>新增: DCBM-125, DCBM-126, DCBM-127, DCBM-128, DCBM-129, DCBM-130, DCBM-131, DCBM-132, DCBM-133, DCBM-134, DCBM-135, DCBM-136, DCBM-137; 跳过重复: 0; 主库记录数更新为 12 → (待QC确认)</t>
   </si>
   <si>
+    <t>2026-07-24 Daily Brief Update</t>
+  </si>
+  <si>
+    <t>新增: DCBM-135, DCBM-136; 跳过重复: 0; 主库记录数更新为 13 → (待QC确认)</t>
+  </si>
+  <si>
     <t>候选原编号</t>
   </si>
   <si>
@@ -10139,6 +10286,12 @@
   </si>
   <si>
     <t>新增 10 篇, 跳过重复 0 篇, 待 validate 确认</t>
+  </si>
+  <si>
+    <t>Daily Brief Update 2026-07-24</t>
+  </si>
+  <si>
+    <t>新增 2 篇, 跳过重复 0 篇, 待 validate 确认</t>
   </si>
 </sst>
 </file>
@@ -10278,7 +10431,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" displayName="DeepCBMComplete105" headerRowCount="1" id="1" name="DeepCBMComplete105" ref="A1:AA106">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" displayName="DeepCBMComplete105" headerRowCount="1" id="1" name="DeepCBMComplete105" ref="A1:AA135">
   <tableColumns count="27">
     <tableColumn id="1" name="序号"/>
     <tableColumn id="2" name="文献ID"/>
@@ -10313,7 +10466,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" displayName="DeepCBMWebIndex105" headerRowCount="1" id="2" name="DeepCBMWebIndex105" ref="A1:H106">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" displayName="DeepCBMWebIndex105" headerRowCount="1" id="2" name="DeepCBMWebIndex105" ref="A1:H134">
   <tableColumns count="8">
     <tableColumn id="1" name="序号"/>
     <tableColumn id="2" name="文献ID"/>
@@ -10481,7 +10634,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA135"/>
+  <dimension ref="A1:AA137"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="13.8" outlineLevelCol="0"/>
   <cols>
     <col customWidth="1" max="1" min="1" width="8"/>
@@ -20563,7 +20716,7 @@
         <v>2516</v>
       </c>
     </row>
-    <row r="123" spans="1:27">
+    <row customHeight="1" ht="96.59999999999999" r="123" spans="1:27">
       <c r="A123" s="10" t="n">
         <v>122</v>
       </c>
@@ -20721,7 +20874,7 @@
         <v>2537</v>
       </c>
     </row>
-    <row r="125" spans="1:27">
+    <row customHeight="1" ht="69" r="125" spans="1:27">
       <c r="A125" s="10" t="n">
         <v>124</v>
       </c>
@@ -20966,7 +21119,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="128" spans="1:27">
+    <row customHeight="1" ht="41.4" r="128" spans="1:27">
       <c r="A128" s="10" t="n">
         <v>127</v>
       </c>
@@ -21043,7 +21196,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="129" spans="1:27">
+    <row customHeight="1" ht="69" r="129" spans="1:27">
       <c r="A129" s="10" t="n">
         <v>128</v>
       </c>
@@ -21194,7 +21347,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="131" spans="1:27">
+    <row customHeight="1" ht="55.2" r="131" spans="1:27">
       <c r="A131" s="10" t="n">
         <v>130</v>
       </c>
@@ -21437,7 +21590,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="134" spans="1:27">
+    <row customHeight="1" ht="41.4" r="134" spans="1:27">
       <c r="A134" s="10" t="n">
         <v>133</v>
       </c>
@@ -21599,6 +21752,167 @@
       </c>
       <c r="AA135" t="s">
         <v>100</v>
+      </c>
+    </row>
+    <row r="136" spans="1:27">
+      <c r="A136" t="n">
+        <v>135</v>
+      </c>
+      <c r="B136" t="s">
+        <v>2761</v>
+      </c>
+      <c r="C136" t="s">
+        <v>2762</v>
+      </c>
+      <c r="D136" t="s">
+        <v>2763</v>
+      </c>
+      <c r="E136" t="s">
+        <v>31</v>
+      </c>
+      <c r="F136" t="s">
+        <v>2764</v>
+      </c>
+      <c r="G136" t="s">
+        <v>2765</v>
+      </c>
+      <c r="H136" t="s">
+        <v>2766</v>
+      </c>
+      <c r="I136" t="s">
+        <v>2767</v>
+      </c>
+      <c r="J136" t="s"/>
+      <c r="K136" t="s">
+        <v>2768</v>
+      </c>
+      <c r="L136" t="s">
+        <v>2769</v>
+      </c>
+      <c r="M136" t="s">
+        <v>2770</v>
+      </c>
+      <c r="N136" t="s">
+        <v>2466</v>
+      </c>
+      <c r="O136" t="s">
+        <v>2771</v>
+      </c>
+      <c r="P136" t="s">
+        <v>2772</v>
+      </c>
+      <c r="Q136" t="s">
+        <v>2773</v>
+      </c>
+      <c r="R136" t="s">
+        <v>2774</v>
+      </c>
+      <c r="S136" t="s">
+        <v>2775</v>
+      </c>
+      <c r="T136" t="s">
+        <v>2776</v>
+      </c>
+      <c r="U136" t="s">
+        <v>2777</v>
+      </c>
+      <c r="V136" t="s">
+        <v>2778</v>
+      </c>
+      <c r="W136" t="s">
+        <v>2779</v>
+      </c>
+      <c r="X136" t="s">
+        <v>2780</v>
+      </c>
+      <c r="Y136" t="s">
+        <v>2781</v>
+      </c>
+      <c r="Z136" t="s">
+        <v>145</v>
+      </c>
+      <c r="AA136" t="s">
+        <v>2782</v>
+      </c>
+    </row>
+    <row r="137" spans="1:27">
+      <c r="A137" t="n">
+        <v>136</v>
+      </c>
+      <c r="B137" t="s">
+        <v>2783</v>
+      </c>
+      <c r="C137" t="s">
+        <v>2784</v>
+      </c>
+      <c r="D137" t="s">
+        <v>2785</v>
+      </c>
+      <c r="E137" t="s">
+        <v>2786</v>
+      </c>
+      <c r="F137" t="s">
+        <v>2787</v>
+      </c>
+      <c r="G137" t="s">
+        <v>2788</v>
+      </c>
+      <c r="H137" t="s">
+        <v>1122</v>
+      </c>
+      <c r="I137" t="s">
+        <v>2789</v>
+      </c>
+      <c r="J137" t="s">
+        <v>2746</v>
+      </c>
+      <c r="K137" t="s">
+        <v>2790</v>
+      </c>
+      <c r="L137" t="s">
+        <v>2791</v>
+      </c>
+      <c r="M137" t="s">
+        <v>2792</v>
+      </c>
+      <c r="N137" t="s">
+        <v>2466</v>
+      </c>
+      <c r="O137" t="s">
+        <v>2793</v>
+      </c>
+      <c r="P137" t="s">
+        <v>2794</v>
+      </c>
+      <c r="R137" t="s">
+        <v>2795</v>
+      </c>
+      <c r="S137" t="s">
+        <v>2796</v>
+      </c>
+      <c r="T137" t="s">
+        <v>2797</v>
+      </c>
+      <c r="U137" t="s">
+        <v>2798</v>
+      </c>
+      <c r="V137" t="s">
+        <v>2799</v>
+      </c>
+      <c r="W137" t="s">
+        <v>2800</v>
+      </c>
+      <c r="X137" t="s">
+        <v>2801</v>
+      </c>
+      <c r="Y137" t="s">
+        <v>2802</v>
+      </c>
+      <c r="Z137" t="s">
+        <v>145</v>
+      </c>
+      <c r="AA137" t="s">
+        <v>2803</v>
       </c>
     </row>
   </sheetData>
@@ -21628,13 +21942,13 @@
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" s="2" t="s">
-        <v>2761</v>
+        <v>2804</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>2762</v>
+        <v>2805</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>2763</v>
+        <v>2806</v>
       </c>
       <c r="D1" s="2" t="n"/>
       <c r="E1" s="2" t="n"/>
@@ -21642,13 +21956,13 @@
     </row>
     <row r="2" spans="1:6">
       <c r="A2" s="3" t="s">
-        <v>2764</v>
+        <v>2807</v>
       </c>
       <c r="B2" s="3" t="n">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>2765</v>
+        <v>2808</v>
       </c>
       <c r="D2" s="3" t="n"/>
       <c r="E2" s="3" t="n"/>
@@ -21656,13 +21970,13 @@
     </row>
     <row customHeight="1" ht="27.6" r="3" spans="1:6">
       <c r="A3" s="3" t="s">
-        <v>2766</v>
+        <v>2809</v>
       </c>
       <c r="B3" s="3" t="n">
         <v>21</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>2767</v>
+        <v>2810</v>
       </c>
       <c r="D3" s="3" t="n"/>
       <c r="E3" s="3" t="n"/>
@@ -21670,13 +21984,13 @@
     </row>
     <row customHeight="1" ht="27.6" r="4" spans="1:6">
       <c r="A4" s="3" t="s">
-        <v>2768</v>
+        <v>2811</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>2769</v>
+        <v>2812</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>2770</v>
+        <v>2813</v>
       </c>
       <c r="D4" s="3" t="n"/>
       <c r="E4" s="3" t="n"/>
@@ -21684,13 +21998,13 @@
     </row>
     <row customHeight="1" ht="27.6" r="5" spans="1:6">
       <c r="A5" s="3" t="s">
-        <v>2771</v>
+        <v>2814</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>2772</v>
+        <v>2815</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>2773</v>
+        <v>2816</v>
       </c>
       <c r="D5" s="3" t="n"/>
       <c r="E5" s="3" t="n"/>
@@ -21698,13 +22012,13 @@
     </row>
     <row customHeight="1" ht="27.6" r="6" spans="1:6">
       <c r="A6" s="3" t="s">
-        <v>2774</v>
+        <v>2817</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>2775</v>
+        <v>2818</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>2776</v>
+        <v>2819</v>
       </c>
       <c r="D6" s="3" t="n"/>
       <c r="E6" s="3" t="n"/>
@@ -21715,14 +22029,14 @@
         <v>4</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>2777</v>
+        <v>2820</v>
       </c>
       <c r="C7" s="3" t="n"/>
       <c r="D7" s="3" t="s">
         <v>13</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>2777</v>
+        <v>2820</v>
       </c>
       <c r="F7" s="3" t="n"/>
     </row>
@@ -21760,7 +22074,7 @@
     </row>
     <row r="10" spans="1:6">
       <c r="A10" s="3" t="s">
-        <v>2778</v>
+        <v>2821</v>
       </c>
       <c r="B10" s="3" t="n">
         <v>1</v>
@@ -21776,7 +22090,7 @@
     </row>
     <row r="11" spans="1:6">
       <c r="A11" s="3" t="s">
-        <v>2779</v>
+        <v>2822</v>
       </c>
       <c r="B11" s="3" t="n">
         <v>1</v>
@@ -21792,7 +22106,7 @@
     </row>
     <row r="12" spans="1:6">
       <c r="A12" s="3" t="s">
-        <v>2780</v>
+        <v>2823</v>
       </c>
       <c r="B12" s="3" t="n">
         <v>1</v>
@@ -21881,7 +22195,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H134"/>
+  <dimension ref="A1:H136"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="13.8" outlineLevelCol="0"/>
   <cols>
     <col customWidth="1" max="1" min="1" width="8"/>
@@ -24647,7 +24961,7 @@
         <v>2217</v>
       </c>
     </row>
-    <row r="107" spans="1:8">
+    <row customHeight="1" ht="41.4" r="107" spans="1:8">
       <c r="A107" s="12" t="n">
         <v>106</v>
       </c>
@@ -24673,7 +24987,7 @@
         <v>2217</v>
       </c>
     </row>
-    <row r="108" spans="1:8">
+    <row customHeight="1" ht="27.6" r="108" spans="1:8">
       <c r="A108" s="12" t="n">
         <v>107</v>
       </c>
@@ -24699,7 +25013,7 @@
         <v>2217</v>
       </c>
     </row>
-    <row r="109" spans="1:8">
+    <row customHeight="1" ht="27.6" r="109" spans="1:8">
       <c r="A109" s="12" t="n">
         <v>108</v>
       </c>
@@ -24723,7 +25037,7 @@
         <v>2217</v>
       </c>
     </row>
-    <row r="110" spans="1:8">
+    <row customHeight="1" ht="27.6" r="110" spans="1:8">
       <c r="A110" s="12" t="n">
         <v>109</v>
       </c>
@@ -24749,7 +25063,7 @@
         <v>2217</v>
       </c>
     </row>
-    <row r="111" spans="1:8">
+    <row customHeight="1" ht="41.4" r="111" spans="1:8">
       <c r="A111" s="12" t="n">
         <v>110</v>
       </c>
@@ -24775,7 +25089,7 @@
         <v>2217</v>
       </c>
     </row>
-    <row r="112" spans="1:8">
+    <row customHeight="1" ht="27.6" r="112" spans="1:8">
       <c r="A112" s="12" t="n">
         <v>111</v>
       </c>
@@ -24801,7 +25115,7 @@
         <v>2217</v>
       </c>
     </row>
-    <row r="113" spans="1:8">
+    <row customHeight="1" ht="27.6" r="113" spans="1:8">
       <c r="A113" s="12" t="n">
         <v>112</v>
       </c>
@@ -24825,7 +25139,7 @@
         <v>2217</v>
       </c>
     </row>
-    <row r="114" spans="1:8">
+    <row customHeight="1" ht="27.6" r="114" spans="1:8">
       <c r="A114" s="12" t="n">
         <v>113</v>
       </c>
@@ -24849,7 +25163,7 @@
         <v>2217</v>
       </c>
     </row>
-    <row r="115" spans="1:8">
+    <row customHeight="1" ht="41.4" r="115" spans="1:8">
       <c r="A115" s="12" t="n">
         <v>114</v>
       </c>
@@ -24875,7 +25189,7 @@
         <v>2217</v>
       </c>
     </row>
-    <row r="116" spans="1:8">
+    <row customHeight="1" ht="27.6" r="116" spans="1:8">
       <c r="A116" s="12" t="n">
         <v>115</v>
       </c>
@@ -24899,7 +25213,7 @@
         <v>2217</v>
       </c>
     </row>
-    <row r="117" spans="1:8">
+    <row customHeight="1" ht="27.6" r="117" spans="1:8">
       <c r="A117" s="12" t="n">
         <v>116</v>
       </c>
@@ -24925,7 +25239,7 @@
         <v>2217</v>
       </c>
     </row>
-    <row r="118" spans="1:8">
+    <row customHeight="1" ht="27.6" r="118" spans="1:8">
       <c r="A118" s="12" t="n">
         <v>117</v>
       </c>
@@ -24951,7 +25265,7 @@
         <v>2217</v>
       </c>
     </row>
-    <row r="119" spans="1:8">
+    <row customHeight="1" ht="27.6" r="119" spans="1:8">
       <c r="A119" s="12" t="n">
         <v>118</v>
       </c>
@@ -25362,6 +25676,28 @@
       </c>
       <c r="H134" t="s">
         <v>100</v>
+      </c>
+    </row>
+    <row r="135" spans="1:8">
+      <c r="A135" t="n">
+        <v>135</v>
+      </c>
+      <c r="B135" t="s">
+        <v>2761</v>
+      </c>
+      <c r="F135" t="s">
+        <v>2769</v>
+      </c>
+    </row>
+    <row r="136" spans="1:8">
+      <c r="A136" t="n">
+        <v>136</v>
+      </c>
+      <c r="B136" t="s">
+        <v>2783</v>
+      </c>
+      <c r="F136" t="s">
+        <v>2791</v>
       </c>
     </row>
   </sheetData>
@@ -25387,10 +25723,10 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="2" t="s">
-        <v>2781</v>
+        <v>2824</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>2763</v>
+        <v>2806</v>
       </c>
     </row>
     <row r="2" spans="1:2">
@@ -25398,7 +25734,7 @@
         <v>0</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>2782</v>
+        <v>2825</v>
       </c>
     </row>
     <row r="3" spans="1:2">
@@ -25406,7 +25742,7 @@
         <v>1</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>2783</v>
+        <v>2826</v>
       </c>
     </row>
     <row r="4" spans="1:2">
@@ -25414,7 +25750,7 @@
         <v>2</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>2784</v>
+        <v>2827</v>
       </c>
     </row>
     <row r="5" spans="1:2">
@@ -25422,7 +25758,7 @@
         <v>3</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>2785</v>
+        <v>2828</v>
       </c>
     </row>
     <row r="6" spans="1:2">
@@ -25430,7 +25766,7 @@
         <v>4</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>2786</v>
+        <v>2829</v>
       </c>
     </row>
     <row r="7" spans="1:2">
@@ -25438,7 +25774,7 @@
         <v>5</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>2787</v>
+        <v>2830</v>
       </c>
     </row>
     <row r="8" spans="1:2">
@@ -25446,7 +25782,7 @@
         <v>6</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>2788</v>
+        <v>2831</v>
       </c>
     </row>
     <row r="9" spans="1:2">
@@ -25454,15 +25790,15 @@
         <v>7</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>2789</v>
+        <v>2832</v>
       </c>
     </row>
     <row r="10" spans="1:2">
       <c r="A10" s="3" t="s">
-        <v>2790</v>
+        <v>2833</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>2791</v>
+        <v>2834</v>
       </c>
     </row>
     <row r="11" spans="1:2">
@@ -25470,7 +25806,7 @@
         <v>11</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>2792</v>
+        <v>2835</v>
       </c>
     </row>
     <row r="12" spans="1:2">
@@ -25478,7 +25814,7 @@
         <v>12</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>2793</v>
+        <v>2836</v>
       </c>
     </row>
     <row r="13" spans="1:2">
@@ -25486,7 +25822,7 @@
         <v>13</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>2794</v>
+        <v>2837</v>
       </c>
     </row>
     <row r="14" spans="1:2">
@@ -25494,7 +25830,7 @@
         <v>14</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>2795</v>
+        <v>2838</v>
       </c>
     </row>
     <row r="15" spans="1:2">
@@ -25502,7 +25838,7 @@
         <v>15</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>2796</v>
+        <v>2839</v>
       </c>
     </row>
     <row r="16" spans="1:2">
@@ -25510,7 +25846,7 @@
         <v>16</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>2797</v>
+        <v>2840</v>
       </c>
     </row>
     <row r="17" spans="1:2">
@@ -25518,7 +25854,7 @@
         <v>17</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>2798</v>
+        <v>2841</v>
       </c>
     </row>
     <row r="18" spans="1:2">
@@ -25526,7 +25862,7 @@
         <v>18</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>2799</v>
+        <v>2842</v>
       </c>
     </row>
     <row r="19" spans="1:2">
@@ -25534,7 +25870,7 @@
         <v>19</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>2800</v>
+        <v>2843</v>
       </c>
     </row>
     <row r="20" spans="1:2">
@@ -25542,7 +25878,7 @@
         <v>20</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>2801</v>
+        <v>2844</v>
       </c>
     </row>
     <row r="21" spans="1:2">
@@ -25550,7 +25886,7 @@
         <v>21</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>2802</v>
+        <v>2845</v>
       </c>
     </row>
     <row r="22" spans="1:2">
@@ -25558,7 +25894,7 @@
         <v>22</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>2803</v>
+        <v>2846</v>
       </c>
     </row>
     <row r="23" spans="1:2">
@@ -25566,7 +25902,7 @@
         <v>23</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>2804</v>
+        <v>2847</v>
       </c>
     </row>
     <row r="24" spans="1:2">
@@ -25574,7 +25910,7 @@
         <v>24</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>2805</v>
+        <v>2848</v>
       </c>
     </row>
     <row r="25" spans="1:2">
@@ -25582,7 +25918,7 @@
         <v>25</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>2806</v>
+        <v>2849</v>
       </c>
     </row>
     <row r="26" spans="1:2">
@@ -25590,7 +25926,7 @@
         <v>26</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>2807</v>
+        <v>2850</v>
       </c>
     </row>
   </sheetData>
@@ -25604,7 +25940,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N135"/>
+  <dimension ref="A1:N137"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="13.8" outlineLevelCol="0"/>
   <cols>
     <col customWidth="1" max="1" min="1" width="12"/>
@@ -25629,22 +25965,22 @@
         <v>4</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>2808</v>
+        <v>2851</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>2809</v>
+        <v>2852</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>2810</v>
+        <v>2853</v>
       </c>
       <c r="F1" s="5" t="s">
         <v>17</v>
       </c>
       <c r="G1" s="5" t="s">
-        <v>2811</v>
+        <v>2854</v>
       </c>
       <c r="H1" s="5" t="s">
-        <v>2812</v>
+        <v>2855</v>
       </c>
       <c r="I1" s="5" t="s">
         <v>20</v>
@@ -25653,16 +25989,16 @@
         <v>21</v>
       </c>
       <c r="K1" s="5" t="s">
-        <v>2813</v>
+        <v>2856</v>
       </c>
       <c r="L1" s="5" t="s">
-        <v>2814</v>
+        <v>2857</v>
       </c>
       <c r="M1" s="5" t="s">
         <v>25</v>
       </c>
       <c r="N1" s="5" t="s">
-        <v>2815</v>
+        <v>2858</v>
       </c>
     </row>
     <row customHeight="1" ht="110.4" r="2" spans="1:14">
@@ -25676,10 +26012,10 @@
         <v>33</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>2816</v>
+        <v>2859</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>2817</v>
+        <v>2860</v>
       </c>
       <c r="F2" s="1" t="s">
         <v>44</v>
@@ -25706,7 +26042,7 @@
         <v>52</v>
       </c>
       <c r="N2" s="1" t="s">
-        <v>2818</v>
+        <v>2861</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="3" spans="1:14">
@@ -25720,10 +26056,10 @@
         <v>59</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>2819</v>
+        <v>2862</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>2820</v>
+        <v>2863</v>
       </c>
       <c r="F3" s="1" t="s">
         <v>68</v>
@@ -25750,7 +26086,7 @@
         <v>52</v>
       </c>
       <c r="N3" s="1" t="s">
-        <v>2818</v>
+        <v>2861</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="4" spans="1:14">
@@ -25764,10 +26100,10 @@
         <v>83</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>2821</v>
+        <v>2864</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>2822</v>
+        <v>2865</v>
       </c>
       <c r="F4" s="1" t="s">
         <v>92</v>
@@ -25794,7 +26130,7 @@
         <v>52</v>
       </c>
       <c r="N4" s="1" t="s">
-        <v>2818</v>
+        <v>2861</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="5" spans="1:14">
@@ -25808,10 +26144,10 @@
         <v>106</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>2823</v>
+        <v>2866</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>2824</v>
+        <v>2867</v>
       </c>
       <c r="F5" s="1" t="s">
         <v>115</v>
@@ -25838,7 +26174,7 @@
         <v>52</v>
       </c>
       <c r="N5" s="1" t="s">
-        <v>2818</v>
+        <v>2861</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="6" spans="1:14">
@@ -25852,10 +26188,10 @@
         <v>128</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>2825</v>
+        <v>2868</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>2826</v>
+        <v>2869</v>
       </c>
       <c r="F6" s="1" t="s">
         <v>137</v>
@@ -25882,7 +26218,7 @@
         <v>145</v>
       </c>
       <c r="N6" s="1" t="s">
-        <v>2818</v>
+        <v>2861</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="7" spans="1:14">
@@ -25896,10 +26232,10 @@
         <v>152</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>2827</v>
+        <v>2870</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>2828</v>
+        <v>2871</v>
       </c>
       <c r="F7" s="1" t="s">
         <v>160</v>
@@ -25926,7 +26262,7 @@
         <v>145</v>
       </c>
       <c r="N7" s="1" t="s">
-        <v>2818</v>
+        <v>2861</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="8" spans="1:14">
@@ -25940,10 +26276,10 @@
         <v>174</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>2829</v>
+        <v>2872</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>2830</v>
+        <v>2873</v>
       </c>
       <c r="F8" s="1" t="s">
         <v>181</v>
@@ -25970,7 +26306,7 @@
         <v>189</v>
       </c>
       <c r="N8" s="1" t="s">
-        <v>2818</v>
+        <v>2861</v>
       </c>
     </row>
     <row customHeight="1" ht="82.8" r="9" spans="1:14">
@@ -25984,10 +26320,10 @@
         <v>195</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>2831</v>
+        <v>2874</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>2832</v>
+        <v>2875</v>
       </c>
       <c r="F9" s="1" t="s">
         <v>201</v>
@@ -26014,7 +26350,7 @@
         <v>145</v>
       </c>
       <c r="N9" s="1" t="s">
-        <v>2818</v>
+        <v>2861</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="10" spans="1:14">
@@ -26028,10 +26364,10 @@
         <v>214</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>2833</v>
+        <v>2876</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>2834</v>
+        <v>2877</v>
       </c>
       <c r="F10" s="1" t="s">
         <v>220</v>
@@ -26058,7 +26394,7 @@
         <v>52</v>
       </c>
       <c r="N10" s="1" t="s">
-        <v>2818</v>
+        <v>2861</v>
       </c>
     </row>
     <row customHeight="1" ht="82.8" r="11" spans="1:14">
@@ -26072,10 +26408,10 @@
         <v>233</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>2835</v>
+        <v>2878</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>2836</v>
+        <v>2879</v>
       </c>
       <c r="F11" s="1" t="s">
         <v>239</v>
@@ -26102,7 +26438,7 @@
         <v>189</v>
       </c>
       <c r="N11" s="1" t="s">
-        <v>2818</v>
+        <v>2861</v>
       </c>
     </row>
     <row customHeight="1" ht="82.8" r="12" spans="1:14">
@@ -26116,10 +26452,10 @@
         <v>252</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>2837</v>
+        <v>2880</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>2838</v>
+        <v>2881</v>
       </c>
       <c r="F12" s="1" t="s">
         <v>258</v>
@@ -26146,7 +26482,7 @@
         <v>145</v>
       </c>
       <c r="N12" s="1" t="s">
-        <v>2818</v>
+        <v>2861</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="13" spans="1:14">
@@ -26160,10 +26496,10 @@
         <v>272</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>2839</v>
+        <v>2882</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>2840</v>
+        <v>2883</v>
       </c>
       <c r="F13" s="1" t="s">
         <v>278</v>
@@ -26190,7 +26526,7 @@
         <v>52</v>
       </c>
       <c r="N13" s="1" t="s">
-        <v>2818</v>
+        <v>2861</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="14" spans="1:14">
@@ -26204,10 +26540,10 @@
         <v>291</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>2841</v>
+        <v>2884</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>2842</v>
+        <v>2885</v>
       </c>
       <c r="F14" s="1" t="s">
         <v>300</v>
@@ -26234,7 +26570,7 @@
         <v>145</v>
       </c>
       <c r="N14" s="1" t="s">
-        <v>2818</v>
+        <v>2861</v>
       </c>
     </row>
     <row customHeight="1" ht="82.8" r="15" spans="1:14">
@@ -26248,10 +26584,10 @@
         <v>313</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>2843</v>
+        <v>2886</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>2844</v>
+        <v>2887</v>
       </c>
       <c r="F15" s="1" t="s">
         <v>321</v>
@@ -26278,7 +26614,7 @@
         <v>52</v>
       </c>
       <c r="N15" s="1" t="s">
-        <v>2818</v>
+        <v>2861</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="16" spans="1:14">
@@ -26292,10 +26628,10 @@
         <v>334</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>2845</v>
+        <v>2888</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>2846</v>
+        <v>2889</v>
       </c>
       <c r="F16" s="1" t="s">
         <v>343</v>
@@ -26322,7 +26658,7 @@
         <v>52</v>
       </c>
       <c r="N16" s="1" t="s">
-        <v>2818</v>
+        <v>2861</v>
       </c>
     </row>
     <row customHeight="1" ht="82.8" r="17" spans="1:14">
@@ -26336,10 +26672,10 @@
         <v>356</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>2847</v>
+        <v>2890</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>2848</v>
+        <v>2891</v>
       </c>
       <c r="F17" s="1" t="s">
         <v>363</v>
@@ -26366,7 +26702,7 @@
         <v>52</v>
       </c>
       <c r="N17" s="1" t="s">
-        <v>2818</v>
+        <v>2861</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="18" spans="1:14">
@@ -26380,10 +26716,10 @@
         <v>376</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>2849</v>
+        <v>2892</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>2850</v>
+        <v>2893</v>
       </c>
       <c r="F18" s="1" t="s">
         <v>383</v>
@@ -26410,7 +26746,7 @@
         <v>145</v>
       </c>
       <c r="N18" s="1" t="s">
-        <v>2818</v>
+        <v>2861</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="19" spans="1:14">
@@ -26424,10 +26760,10 @@
         <v>397</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>2851</v>
+        <v>2894</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>2852</v>
+        <v>2895</v>
       </c>
       <c r="F19" s="1" t="s">
         <v>404</v>
@@ -26454,7 +26790,7 @@
         <v>145</v>
       </c>
       <c r="N19" s="1" t="s">
-        <v>2818</v>
+        <v>2861</v>
       </c>
     </row>
     <row customHeight="1" ht="82.8" r="20" spans="1:14">
@@ -26468,10 +26804,10 @@
         <v>418</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>2853</v>
+        <v>2896</v>
       </c>
       <c r="E20" s="1" t="s">
-        <v>2854</v>
+        <v>2897</v>
       </c>
       <c r="F20" s="1" t="s">
         <v>427</v>
@@ -26498,7 +26834,7 @@
         <v>145</v>
       </c>
       <c r="N20" s="1" t="s">
-        <v>2818</v>
+        <v>2861</v>
       </c>
     </row>
     <row customHeight="1" ht="82.8" r="21" spans="1:14">
@@ -26512,10 +26848,10 @@
         <v>441</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>2855</v>
+        <v>2898</v>
       </c>
       <c r="E21" s="1" t="s">
-        <v>2856</v>
+        <v>2899</v>
       </c>
       <c r="F21" s="1" t="s">
         <v>448</v>
@@ -26542,7 +26878,7 @@
         <v>145</v>
       </c>
       <c r="N21" s="1" t="s">
-        <v>2818</v>
+        <v>2861</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="22" spans="1:14">
@@ -26556,10 +26892,10 @@
         <v>462</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>2857</v>
+        <v>2900</v>
       </c>
       <c r="E22" s="1" t="s">
-        <v>2858</v>
+        <v>2901</v>
       </c>
       <c r="F22" s="1" t="s">
         <v>467</v>
@@ -26586,7 +26922,7 @@
         <v>52</v>
       </c>
       <c r="N22" s="1" t="s">
-        <v>2818</v>
+        <v>2861</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="23" spans="1:14">
@@ -26600,10 +26936,10 @@
         <v>481</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>2859</v>
+        <v>2902</v>
       </c>
       <c r="E23" s="1" t="s">
-        <v>2860</v>
+        <v>2903</v>
       </c>
       <c r="F23" s="1" t="s">
         <v>489</v>
@@ -26630,7 +26966,7 @@
         <v>145</v>
       </c>
       <c r="N23" s="1" t="s">
-        <v>2818</v>
+        <v>2861</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="24" spans="1:14">
@@ -26644,10 +26980,10 @@
         <v>503</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>2861</v>
+        <v>2904</v>
       </c>
       <c r="E24" s="1" t="s">
-        <v>2862</v>
+        <v>2905</v>
       </c>
       <c r="F24" s="1" t="s">
         <v>511</v>
@@ -26674,7 +27010,7 @@
         <v>52</v>
       </c>
       <c r="N24" s="1" t="s">
-        <v>2818</v>
+        <v>2861</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="25" spans="1:14">
@@ -26688,10 +27024,10 @@
         <v>524</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>2863</v>
+        <v>2906</v>
       </c>
       <c r="E25" s="1" t="s">
-        <v>2864</v>
+        <v>2907</v>
       </c>
       <c r="F25" s="1" t="s">
         <v>532</v>
@@ -26718,7 +27054,7 @@
         <v>145</v>
       </c>
       <c r="N25" s="1" t="s">
-        <v>2818</v>
+        <v>2861</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="26" spans="1:14">
@@ -26732,10 +27068,10 @@
         <v>546</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>2865</v>
+        <v>2908</v>
       </c>
       <c r="E26" s="1" t="s">
-        <v>2866</v>
+        <v>2909</v>
       </c>
       <c r="F26" s="1" t="s">
         <v>554</v>
@@ -26762,7 +27098,7 @@
         <v>52</v>
       </c>
       <c r="N26" s="1" t="s">
-        <v>2818</v>
+        <v>2861</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="27" spans="1:14">
@@ -26776,10 +27112,10 @@
         <v>568</v>
       </c>
       <c r="D27" s="1" t="s">
-        <v>2867</v>
+        <v>2910</v>
       </c>
       <c r="E27" s="1" t="s">
-        <v>2868</v>
+        <v>2911</v>
       </c>
       <c r="F27" s="1" t="s">
         <v>577</v>
@@ -26806,7 +27142,7 @@
         <v>52</v>
       </c>
       <c r="N27" s="1" t="s">
-        <v>2818</v>
+        <v>2861</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="28" spans="1:14">
@@ -26820,10 +27156,10 @@
         <v>591</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>2869</v>
+        <v>2912</v>
       </c>
       <c r="E28" s="1" t="s">
-        <v>2870</v>
+        <v>2913</v>
       </c>
       <c r="F28" s="1" t="s">
         <v>600</v>
@@ -26850,7 +27186,7 @@
         <v>52</v>
       </c>
       <c r="N28" s="1" t="s">
-        <v>2818</v>
+        <v>2861</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="29" spans="1:14">
@@ -26864,10 +27200,10 @@
         <v>614</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>2871</v>
+        <v>2914</v>
       </c>
       <c r="E29" s="1" t="s">
-        <v>2872</v>
+        <v>2915</v>
       </c>
       <c r="F29" s="1" t="s">
         <v>623</v>
@@ -26894,7 +27230,7 @@
         <v>52</v>
       </c>
       <c r="N29" s="1" t="s">
-        <v>2818</v>
+        <v>2861</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="30" spans="1:14">
@@ -26908,10 +27244,10 @@
         <v>637</v>
       </c>
       <c r="D30" s="1" t="s">
-        <v>2873</v>
+        <v>2916</v>
       </c>
       <c r="E30" s="1" t="s">
-        <v>2874</v>
+        <v>2917</v>
       </c>
       <c r="F30" s="1" t="s">
         <v>646</v>
@@ -26938,7 +27274,7 @@
         <v>52</v>
       </c>
       <c r="N30" s="1" t="s">
-        <v>2818</v>
+        <v>2861</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="31" spans="1:14">
@@ -26952,10 +27288,10 @@
         <v>659</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>2875</v>
+        <v>2918</v>
       </c>
       <c r="E31" s="1" t="s">
-        <v>2876</v>
+        <v>2919</v>
       </c>
       <c r="F31" s="1" t="s">
         <v>668</v>
@@ -26982,7 +27318,7 @@
         <v>52</v>
       </c>
       <c r="N31" s="1" t="s">
-        <v>2818</v>
+        <v>2861</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="32" spans="1:14">
@@ -26996,10 +27332,10 @@
         <v>682</v>
       </c>
       <c r="D32" s="1" t="s">
-        <v>2877</v>
+        <v>2920</v>
       </c>
       <c r="E32" s="1" t="s">
-        <v>2878</v>
+        <v>2921</v>
       </c>
       <c r="F32" s="1" t="s">
         <v>689</v>
@@ -27026,7 +27362,7 @@
         <v>52</v>
       </c>
       <c r="N32" s="1" t="s">
-        <v>2818</v>
+        <v>2861</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="33" spans="1:14">
@@ -27040,10 +27376,10 @@
         <v>702</v>
       </c>
       <c r="D33" s="1" t="s">
-        <v>2879</v>
+        <v>2922</v>
       </c>
       <c r="E33" s="1" t="s">
-        <v>2880</v>
+        <v>2923</v>
       </c>
       <c r="F33" s="1" t="s">
         <v>709</v>
@@ -27070,7 +27406,7 @@
         <v>145</v>
       </c>
       <c r="N33" s="1" t="s">
-        <v>2818</v>
+        <v>2861</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="34" spans="1:14">
@@ -27084,10 +27420,10 @@
         <v>722</v>
       </c>
       <c r="D34" s="1" t="s">
-        <v>2881</v>
+        <v>2924</v>
       </c>
       <c r="E34" s="1" t="s">
-        <v>2882</v>
+        <v>2925</v>
       </c>
       <c r="F34" s="1" t="s">
         <v>731</v>
@@ -27114,7 +27450,7 @@
         <v>52</v>
       </c>
       <c r="N34" s="1" t="s">
-        <v>2818</v>
+        <v>2861</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="35" spans="1:14">
@@ -27128,10 +27464,10 @@
         <v>744</v>
       </c>
       <c r="D35" s="1" t="s">
-        <v>2883</v>
+        <v>2926</v>
       </c>
       <c r="E35" s="1" t="s">
-        <v>2884</v>
+        <v>2927</v>
       </c>
       <c r="F35" s="1" t="s">
         <v>751</v>
@@ -27158,7 +27494,7 @@
         <v>52</v>
       </c>
       <c r="N35" s="1" t="s">
-        <v>2818</v>
+        <v>2861</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="36" spans="1:14">
@@ -27172,10 +27508,10 @@
         <v>764</v>
       </c>
       <c r="D36" s="1" t="s">
-        <v>2885</v>
+        <v>2928</v>
       </c>
       <c r="E36" s="1" t="s">
-        <v>2886</v>
+        <v>2929</v>
       </c>
       <c r="F36" s="1" t="s">
         <v>772</v>
@@ -27202,7 +27538,7 @@
         <v>145</v>
       </c>
       <c r="N36" s="1" t="s">
-        <v>2818</v>
+        <v>2861</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="37" spans="1:14">
@@ -27216,10 +27552,10 @@
         <v>785</v>
       </c>
       <c r="D37" s="1" t="s">
-        <v>2887</v>
+        <v>2930</v>
       </c>
       <c r="E37" s="1" t="s">
-        <v>2888</v>
+        <v>2931</v>
       </c>
       <c r="F37" s="1" t="s">
         <v>792</v>
@@ -27246,7 +27582,7 @@
         <v>145</v>
       </c>
       <c r="N37" s="1" t="s">
-        <v>2818</v>
+        <v>2861</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="38" spans="1:14">
@@ -27260,10 +27596,10 @@
         <v>806</v>
       </c>
       <c r="D38" s="1" t="s">
-        <v>2889</v>
+        <v>2932</v>
       </c>
       <c r="E38" s="1" t="s">
-        <v>2890</v>
+        <v>2933</v>
       </c>
       <c r="F38" s="1" t="s">
         <v>814</v>
@@ -27290,7 +27626,7 @@
         <v>145</v>
       </c>
       <c r="N38" s="1" t="s">
-        <v>2818</v>
+        <v>2861</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="39" spans="1:14">
@@ -27304,10 +27640,10 @@
         <v>827</v>
       </c>
       <c r="D39" s="1" t="s">
-        <v>2891</v>
+        <v>2934</v>
       </c>
       <c r="E39" s="1" t="s">
-        <v>2892</v>
+        <v>2935</v>
       </c>
       <c r="F39" s="1" t="s">
         <v>834</v>
@@ -27334,7 +27670,7 @@
         <v>145</v>
       </c>
       <c r="N39" s="1" t="s">
-        <v>2818</v>
+        <v>2861</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="40" spans="1:14">
@@ -27348,10 +27684,10 @@
         <v>848</v>
       </c>
       <c r="D40" s="1" t="s">
-        <v>2893</v>
+        <v>2936</v>
       </c>
       <c r="E40" s="1" t="s">
-        <v>2894</v>
+        <v>2937</v>
       </c>
       <c r="F40" s="1" t="s">
         <v>856</v>
@@ -27378,7 +27714,7 @@
         <v>52</v>
       </c>
       <c r="N40" s="1" t="s">
-        <v>2818</v>
+        <v>2861</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="41" spans="1:14">
@@ -27392,10 +27728,10 @@
         <v>870</v>
       </c>
       <c r="D41" s="1" t="s">
-        <v>2895</v>
+        <v>2938</v>
       </c>
       <c r="E41" s="1" t="s">
-        <v>2896</v>
+        <v>2939</v>
       </c>
       <c r="F41" s="1" t="s">
         <v>878</v>
@@ -27422,7 +27758,7 @@
         <v>52</v>
       </c>
       <c r="N41" s="1" t="s">
-        <v>2818</v>
+        <v>2861</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="42" spans="1:14">
@@ -27436,10 +27772,10 @@
         <v>891</v>
       </c>
       <c r="D42" s="1" t="s">
-        <v>2897</v>
+        <v>2940</v>
       </c>
       <c r="E42" s="1" t="s">
-        <v>2898</v>
+        <v>2941</v>
       </c>
       <c r="F42" s="1" t="s">
         <v>901</v>
@@ -27466,7 +27802,7 @@
         <v>52</v>
       </c>
       <c r="N42" s="1" t="s">
-        <v>2818</v>
+        <v>2861</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="43" spans="1:14">
@@ -27480,10 +27816,10 @@
         <v>914</v>
       </c>
       <c r="D43" s="1" t="s">
-        <v>2899</v>
+        <v>2942</v>
       </c>
       <c r="E43" s="1" t="s">
-        <v>2900</v>
+        <v>2943</v>
       </c>
       <c r="F43" s="1" t="s">
         <v>921</v>
@@ -27510,7 +27846,7 @@
         <v>52</v>
       </c>
       <c r="N43" s="1" t="s">
-        <v>2818</v>
+        <v>2861</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="44" spans="1:14">
@@ -27524,10 +27860,10 @@
         <v>933</v>
       </c>
       <c r="D44" s="1" t="s">
-        <v>2901</v>
+        <v>2944</v>
       </c>
       <c r="E44" s="1" t="s">
-        <v>2902</v>
+        <v>2945</v>
       </c>
       <c r="F44" s="1" t="s">
         <v>940</v>
@@ -27554,7 +27890,7 @@
         <v>52</v>
       </c>
       <c r="N44" s="1" t="s">
-        <v>2818</v>
+        <v>2861</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="45" spans="1:14">
@@ -27568,10 +27904,10 @@
         <v>953</v>
       </c>
       <c r="D45" s="1" t="s">
-        <v>2903</v>
+        <v>2946</v>
       </c>
       <c r="E45" s="1" t="s">
-        <v>2904</v>
+        <v>2947</v>
       </c>
       <c r="F45" s="1" t="s">
         <v>959</v>
@@ -27598,7 +27934,7 @@
         <v>52</v>
       </c>
       <c r="N45" s="1" t="s">
-        <v>2818</v>
+        <v>2861</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="46" spans="1:14">
@@ -27612,10 +27948,10 @@
         <v>972</v>
       </c>
       <c r="D46" s="1" t="s">
-        <v>2905</v>
+        <v>2948</v>
       </c>
       <c r="E46" s="1" t="s">
-        <v>2906</v>
+        <v>2949</v>
       </c>
       <c r="F46" s="1" t="s">
         <v>978</v>
@@ -27642,7 +27978,7 @@
         <v>52</v>
       </c>
       <c r="N46" s="1" t="s">
-        <v>2818</v>
+        <v>2861</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="47" spans="1:14">
@@ -27656,10 +27992,10 @@
         <v>990</v>
       </c>
       <c r="D47" s="1" t="s">
-        <v>2907</v>
+        <v>2950</v>
       </c>
       <c r="E47" s="1" t="s">
-        <v>2908</v>
+        <v>2951</v>
       </c>
       <c r="F47" s="1" t="s">
         <v>997</v>
@@ -27686,7 +28022,7 @@
         <v>52</v>
       </c>
       <c r="N47" s="1" t="s">
-        <v>2818</v>
+        <v>2861</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="48" spans="1:14">
@@ -27700,10 +28036,10 @@
         <v>1010</v>
       </c>
       <c r="D48" s="1" t="s">
-        <v>2909</v>
+        <v>2952</v>
       </c>
       <c r="E48" s="1" t="s">
-        <v>2910</v>
+        <v>2953</v>
       </c>
       <c r="F48" s="1" t="s">
         <v>1018</v>
@@ -27730,7 +28066,7 @@
         <v>52</v>
       </c>
       <c r="N48" s="1" t="s">
-        <v>2818</v>
+        <v>2861</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="49" spans="1:14">
@@ -27744,10 +28080,10 @@
         <v>1030</v>
       </c>
       <c r="D49" s="1" t="s">
-        <v>2911</v>
+        <v>2954</v>
       </c>
       <c r="E49" s="1" t="s">
-        <v>2912</v>
+        <v>2955</v>
       </c>
       <c r="F49" s="1" t="s">
         <v>1037</v>
@@ -27774,7 +28110,7 @@
         <v>52</v>
       </c>
       <c r="N49" s="1" t="s">
-        <v>2818</v>
+        <v>2861</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="50" spans="1:14">
@@ -27788,10 +28124,10 @@
         <v>1049</v>
       </c>
       <c r="D50" s="1" t="s">
-        <v>2913</v>
+        <v>2956</v>
       </c>
       <c r="E50" s="1" t="s">
-        <v>2914</v>
+        <v>2957</v>
       </c>
       <c r="F50" s="1" t="s">
         <v>1055</v>
@@ -27818,7 +28154,7 @@
         <v>189</v>
       </c>
       <c r="N50" s="1" t="s">
-        <v>2818</v>
+        <v>2861</v>
       </c>
     </row>
     <row customHeight="1" ht="82.8" r="51" spans="1:14">
@@ -27832,10 +28168,10 @@
         <v>1067</v>
       </c>
       <c r="D51" s="1" t="s">
-        <v>2915</v>
+        <v>2958</v>
       </c>
       <c r="E51" s="1" t="s">
-        <v>2916</v>
+        <v>2959</v>
       </c>
       <c r="F51" s="1" t="s">
         <v>1072</v>
@@ -27862,7 +28198,7 @@
         <v>52</v>
       </c>
       <c r="N51" s="1" t="s">
-        <v>2818</v>
+        <v>2861</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="52" spans="1:14">
@@ -27876,10 +28212,10 @@
         <v>1084</v>
       </c>
       <c r="D52" s="1" t="s">
-        <v>2917</v>
+        <v>2960</v>
       </c>
       <c r="E52" s="1" t="s">
-        <v>2918</v>
+        <v>2961</v>
       </c>
       <c r="F52" s="1" t="s">
         <v>1091</v>
@@ -27906,7 +28242,7 @@
         <v>189</v>
       </c>
       <c r="N52" s="1" t="s">
-        <v>2818</v>
+        <v>2861</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="53" spans="1:14">
@@ -27920,10 +28256,10 @@
         <v>1104</v>
       </c>
       <c r="D53" s="1" t="s">
-        <v>2919</v>
+        <v>2962</v>
       </c>
       <c r="E53" s="1" t="s">
-        <v>2920</v>
+        <v>2963</v>
       </c>
       <c r="F53" s="1" t="s">
         <v>1109</v>
@@ -27950,7 +28286,7 @@
         <v>145</v>
       </c>
       <c r="N53" s="1" t="s">
-        <v>2818</v>
+        <v>2861</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="54" spans="1:14">
@@ -27964,10 +28300,10 @@
         <v>1121</v>
       </c>
       <c r="D54" s="1" t="s">
-        <v>2921</v>
+        <v>2964</v>
       </c>
       <c r="E54" s="1" t="s">
-        <v>2922</v>
+        <v>2965</v>
       </c>
       <c r="F54" s="1" t="s">
         <v>1131</v>
@@ -27994,7 +28330,7 @@
         <v>52</v>
       </c>
       <c r="N54" s="1" t="s">
-        <v>2818</v>
+        <v>2861</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="55" spans="1:14">
@@ -28008,10 +28344,10 @@
         <v>1144</v>
       </c>
       <c r="D55" s="1" t="s">
-        <v>2923</v>
+        <v>2966</v>
       </c>
       <c r="E55" s="1" t="s">
-        <v>2924</v>
+        <v>2967</v>
       </c>
       <c r="F55" s="1" t="s">
         <v>1151</v>
@@ -28038,7 +28374,7 @@
         <v>52</v>
       </c>
       <c r="N55" s="1" t="s">
-        <v>2818</v>
+        <v>2861</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="56" spans="1:14">
@@ -28052,10 +28388,10 @@
         <v>1165</v>
       </c>
       <c r="D56" s="1" t="s">
-        <v>2925</v>
+        <v>2968</v>
       </c>
       <c r="E56" s="1" t="s">
-        <v>2926</v>
+        <v>2969</v>
       </c>
       <c r="F56" s="1" t="s">
         <v>1173</v>
@@ -28082,7 +28418,7 @@
         <v>52</v>
       </c>
       <c r="N56" s="1" t="s">
-        <v>2818</v>
+        <v>2861</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="57" spans="1:14">
@@ -28096,10 +28432,10 @@
         <v>1187</v>
       </c>
       <c r="D57" s="1" t="s">
-        <v>2927</v>
+        <v>2970</v>
       </c>
       <c r="E57" s="1" t="s">
-        <v>2928</v>
+        <v>2971</v>
       </c>
       <c r="F57" s="1" t="s">
         <v>1195</v>
@@ -28126,7 +28462,7 @@
         <v>189</v>
       </c>
       <c r="N57" s="1" t="s">
-        <v>2818</v>
+        <v>2861</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="58" spans="1:14">
@@ -28140,10 +28476,10 @@
         <v>1209</v>
       </c>
       <c r="D58" s="1" t="s">
-        <v>2929</v>
+        <v>2972</v>
       </c>
       <c r="E58" s="1" t="s">
-        <v>2930</v>
+        <v>2973</v>
       </c>
       <c r="F58" s="1" t="s">
         <v>1217</v>
@@ -28170,7 +28506,7 @@
         <v>189</v>
       </c>
       <c r="N58" s="1" t="s">
-        <v>2818</v>
+        <v>2861</v>
       </c>
     </row>
     <row customHeight="1" ht="82.8" r="59" spans="1:14">
@@ -28184,10 +28520,10 @@
         <v>1231</v>
       </c>
       <c r="D59" s="1" t="s">
-        <v>2931</v>
+        <v>2974</v>
       </c>
       <c r="E59" s="1" t="s">
-        <v>2932</v>
+        <v>2975</v>
       </c>
       <c r="F59" s="1" t="s">
         <v>1239</v>
@@ -28214,7 +28550,7 @@
         <v>189</v>
       </c>
       <c r="N59" s="1" t="s">
-        <v>2818</v>
+        <v>2861</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="60" spans="1:14">
@@ -28228,10 +28564,10 @@
         <v>1252</v>
       </c>
       <c r="D60" s="1" t="s">
-        <v>2933</v>
+        <v>2976</v>
       </c>
       <c r="E60" s="1" t="s">
-        <v>2934</v>
+        <v>2977</v>
       </c>
       <c r="F60" s="1" t="s">
         <v>1261</v>
@@ -28258,7 +28594,7 @@
         <v>52</v>
       </c>
       <c r="N60" s="1" t="s">
-        <v>2818</v>
+        <v>2861</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="61" spans="1:14">
@@ -28272,10 +28608,10 @@
         <v>1275</v>
       </c>
       <c r="D61" s="1" t="s">
-        <v>2935</v>
+        <v>2978</v>
       </c>
       <c r="E61" s="1" t="s">
-        <v>2936</v>
+        <v>2979</v>
       </c>
       <c r="F61" s="1" t="s">
         <v>1283</v>
@@ -28302,7 +28638,7 @@
         <v>52</v>
       </c>
       <c r="N61" s="1" t="s">
-        <v>2818</v>
+        <v>2861</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="62" spans="1:14">
@@ -28316,10 +28652,10 @@
         <v>1297</v>
       </c>
       <c r="D62" s="1" t="s">
-        <v>2937</v>
+        <v>2980</v>
       </c>
       <c r="E62" s="1" t="s">
-        <v>2938</v>
+        <v>2981</v>
       </c>
       <c r="F62" s="1" t="s">
         <v>1305</v>
@@ -28346,7 +28682,7 @@
         <v>145</v>
       </c>
       <c r="N62" s="1" t="s">
-        <v>2818</v>
+        <v>2861</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="63" spans="1:14">
@@ -28360,10 +28696,10 @@
         <v>1319</v>
       </c>
       <c r="D63" s="1" t="s">
-        <v>2939</v>
+        <v>2982</v>
       </c>
       <c r="E63" s="1" t="s">
-        <v>2940</v>
+        <v>2983</v>
       </c>
       <c r="F63" s="1" t="s">
         <v>1327</v>
@@ -28390,7 +28726,7 @@
         <v>189</v>
       </c>
       <c r="N63" s="1" t="s">
-        <v>2818</v>
+        <v>2861</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="64" spans="1:14">
@@ -28404,10 +28740,10 @@
         <v>1341</v>
       </c>
       <c r="D64" s="1" t="s">
-        <v>2941</v>
+        <v>2984</v>
       </c>
       <c r="E64" s="1" t="s">
-        <v>2942</v>
+        <v>2985</v>
       </c>
       <c r="F64" s="1" t="s">
         <v>1348</v>
@@ -28434,7 +28770,7 @@
         <v>52</v>
       </c>
       <c r="N64" s="1" t="s">
-        <v>2818</v>
+        <v>2861</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="65" spans="1:14">
@@ -28448,10 +28784,10 @@
         <v>1361</v>
       </c>
       <c r="D65" s="1" t="s">
-        <v>2943</v>
+        <v>2986</v>
       </c>
       <c r="E65" s="1" t="s">
-        <v>2944</v>
+        <v>2987</v>
       </c>
       <c r="F65" s="1" t="s">
         <v>1368</v>
@@ -28478,7 +28814,7 @@
         <v>52</v>
       </c>
       <c r="N65" s="1" t="s">
-        <v>2818</v>
+        <v>2861</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="66" spans="1:14">
@@ -28492,10 +28828,10 @@
         <v>1382</v>
       </c>
       <c r="D66" s="1" t="s">
-        <v>2945</v>
+        <v>2988</v>
       </c>
       <c r="E66" s="1" t="s">
-        <v>2946</v>
+        <v>2989</v>
       </c>
       <c r="F66" s="1" t="s">
         <v>1389</v>
@@ -28522,7 +28858,7 @@
         <v>52</v>
       </c>
       <c r="N66" s="1" t="s">
-        <v>2818</v>
+        <v>2861</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="67" spans="1:14">
@@ -28536,10 +28872,10 @@
         <v>1403</v>
       </c>
       <c r="D67" s="1" t="s">
-        <v>2947</v>
+        <v>2990</v>
       </c>
       <c r="E67" s="1" t="s">
-        <v>2948</v>
+        <v>2991</v>
       </c>
       <c r="F67" s="1" t="s">
         <v>1408</v>
@@ -28566,7 +28902,7 @@
         <v>52</v>
       </c>
       <c r="N67" s="1" t="s">
-        <v>2818</v>
+        <v>2861</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="68" spans="1:14">
@@ -28580,10 +28916,10 @@
         <v>1421</v>
       </c>
       <c r="D68" s="1" t="s">
-        <v>2949</v>
+        <v>2992</v>
       </c>
       <c r="E68" s="1" t="s">
-        <v>2950</v>
+        <v>2993</v>
       </c>
       <c r="F68" s="1" t="s">
         <v>1428</v>
@@ -28610,7 +28946,7 @@
         <v>52</v>
       </c>
       <c r="N68" s="1" t="s">
-        <v>2818</v>
+        <v>2861</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="69" spans="1:14">
@@ -28624,10 +28960,10 @@
         <v>1442</v>
       </c>
       <c r="D69" s="1" t="s">
-        <v>2951</v>
+        <v>2994</v>
       </c>
       <c r="E69" s="1" t="s">
-        <v>2952</v>
+        <v>2995</v>
       </c>
       <c r="F69" s="1" t="s">
         <v>1448</v>
@@ -28654,7 +28990,7 @@
         <v>52</v>
       </c>
       <c r="N69" s="1" t="s">
-        <v>2818</v>
+        <v>2861</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="70" spans="1:14">
@@ -28668,10 +29004,10 @@
         <v>1460</v>
       </c>
       <c r="D70" s="1" t="s">
-        <v>2953</v>
+        <v>2996</v>
       </c>
       <c r="E70" s="1" t="s">
-        <v>2954</v>
+        <v>2997</v>
       </c>
       <c r="F70" s="1" t="s">
         <v>1466</v>
@@ -28698,7 +29034,7 @@
         <v>52</v>
       </c>
       <c r="N70" s="1" t="s">
-        <v>2818</v>
+        <v>2861</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="71" spans="1:14">
@@ -28712,10 +29048,10 @@
         <v>1480</v>
       </c>
       <c r="D71" s="1" t="s">
-        <v>2955</v>
+        <v>2998</v>
       </c>
       <c r="E71" s="1" t="s">
-        <v>2956</v>
+        <v>2999</v>
       </c>
       <c r="F71" s="1" t="s">
         <v>1486</v>
@@ -28742,7 +29078,7 @@
         <v>52</v>
       </c>
       <c r="N71" s="1" t="s">
-        <v>2818</v>
+        <v>2861</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="72" spans="1:14">
@@ -28756,10 +29092,10 @@
         <v>1499</v>
       </c>
       <c r="D72" s="1" t="s">
-        <v>2957</v>
+        <v>3000</v>
       </c>
       <c r="E72" s="1" t="s">
-        <v>2958</v>
+        <v>3001</v>
       </c>
       <c r="F72" s="1" t="s">
         <v>1505</v>
@@ -28786,7 +29122,7 @@
         <v>52</v>
       </c>
       <c r="N72" s="1" t="s">
-        <v>2818</v>
+        <v>2861</v>
       </c>
     </row>
     <row customHeight="1" ht="82.8" r="73" spans="1:14">
@@ -28800,10 +29136,10 @@
         <v>1518</v>
       </c>
       <c r="D73" s="1" t="s">
-        <v>2959</v>
+        <v>3002</v>
       </c>
       <c r="E73" s="1" t="s">
-        <v>2960</v>
+        <v>3003</v>
       </c>
       <c r="F73" s="1" t="s">
         <v>1524</v>
@@ -28830,7 +29166,7 @@
         <v>145</v>
       </c>
       <c r="N73" s="1" t="s">
-        <v>2818</v>
+        <v>2861</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="74" spans="1:14">
@@ -28844,10 +29180,10 @@
         <v>1537</v>
       </c>
       <c r="D74" s="1" t="s">
-        <v>2961</v>
+        <v>3004</v>
       </c>
       <c r="E74" s="1" t="s">
-        <v>2962</v>
+        <v>3005</v>
       </c>
       <c r="F74" s="1" t="s">
         <v>1544</v>
@@ -28874,7 +29210,7 @@
         <v>52</v>
       </c>
       <c r="N74" s="1" t="s">
-        <v>2818</v>
+        <v>2861</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="75" spans="1:14">
@@ -28888,10 +29224,10 @@
         <v>1556</v>
       </c>
       <c r="D75" s="1" t="s">
-        <v>2963</v>
+        <v>3006</v>
       </c>
       <c r="E75" s="1" t="s">
-        <v>2964</v>
+        <v>3007</v>
       </c>
       <c r="F75" s="1" t="s">
         <v>1563</v>
@@ -28918,7 +29254,7 @@
         <v>52</v>
       </c>
       <c r="N75" s="1" t="s">
-        <v>2818</v>
+        <v>2861</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="76" spans="1:14">
@@ -28932,10 +29268,10 @@
         <v>1576</v>
       </c>
       <c r="D76" s="1" t="s">
-        <v>2965</v>
+        <v>3008</v>
       </c>
       <c r="E76" s="1" t="s">
-        <v>2966</v>
+        <v>3009</v>
       </c>
       <c r="F76" s="1" t="s">
         <v>1583</v>
@@ -28962,7 +29298,7 @@
         <v>52</v>
       </c>
       <c r="N76" s="1" t="s">
-        <v>2818</v>
+        <v>2861</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="77" spans="1:14">
@@ -28976,10 +29312,10 @@
         <v>1596</v>
       </c>
       <c r="D77" s="1" t="s">
-        <v>2967</v>
+        <v>3010</v>
       </c>
       <c r="E77" s="1" t="s">
-        <v>2968</v>
+        <v>3011</v>
       </c>
       <c r="F77" s="1" t="s">
         <v>1602</v>
@@ -29006,7 +29342,7 @@
         <v>52</v>
       </c>
       <c r="N77" s="1" t="s">
-        <v>2818</v>
+        <v>2861</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="78" spans="1:14">
@@ -29020,10 +29356,10 @@
         <v>1615</v>
       </c>
       <c r="D78" s="1" t="s">
-        <v>2969</v>
+        <v>3012</v>
       </c>
       <c r="E78" s="1" t="s">
-        <v>2970</v>
+        <v>3013</v>
       </c>
       <c r="F78" s="1" t="s">
         <v>1621</v>
@@ -29050,7 +29386,7 @@
         <v>52</v>
       </c>
       <c r="N78" s="1" t="s">
-        <v>2818</v>
+        <v>2861</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="79" spans="1:14">
@@ -29064,10 +29400,10 @@
         <v>1634</v>
       </c>
       <c r="D79" s="1" t="s">
-        <v>2971</v>
+        <v>3014</v>
       </c>
       <c r="E79" s="1" t="s">
-        <v>2972</v>
+        <v>3015</v>
       </c>
       <c r="F79" s="1" t="s">
         <v>1643</v>
@@ -29094,7 +29430,7 @@
         <v>145</v>
       </c>
       <c r="N79" s="1" t="s">
-        <v>2818</v>
+        <v>2861</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="80" spans="1:14">
@@ -29108,10 +29444,10 @@
         <v>1657</v>
       </c>
       <c r="D80" s="1" t="s">
-        <v>2973</v>
+        <v>3016</v>
       </c>
       <c r="E80" s="1" t="s">
-        <v>2974</v>
+        <v>3017</v>
       </c>
       <c r="F80" s="1" t="s">
         <v>1665</v>
@@ -29138,7 +29474,7 @@
         <v>189</v>
       </c>
       <c r="N80" s="1" t="s">
-        <v>2818</v>
+        <v>2861</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="81" spans="1:14">
@@ -29152,10 +29488,10 @@
         <v>1678</v>
       </c>
       <c r="D81" s="1" t="s">
-        <v>2975</v>
+        <v>3018</v>
       </c>
       <c r="E81" s="1" t="s">
-        <v>2976</v>
+        <v>3019</v>
       </c>
       <c r="F81" s="1" t="s">
         <v>1686</v>
@@ -29182,7 +29518,7 @@
         <v>52</v>
       </c>
       <c r="N81" s="1" t="s">
-        <v>2818</v>
+        <v>2861</v>
       </c>
     </row>
     <row customHeight="1" ht="82.8" r="82" spans="1:14">
@@ -29196,10 +29532,10 @@
         <v>1700</v>
       </c>
       <c r="D82" s="1" t="s">
-        <v>2977</v>
+        <v>3020</v>
       </c>
       <c r="E82" s="1" t="s">
-        <v>2978</v>
+        <v>3021</v>
       </c>
       <c r="F82" s="1" t="s">
         <v>1708</v>
@@ -29226,7 +29562,7 @@
         <v>145</v>
       </c>
       <c r="N82" s="1" t="s">
-        <v>2818</v>
+        <v>2861</v>
       </c>
     </row>
     <row customHeight="1" ht="82.8" r="83" spans="1:14">
@@ -29240,10 +29576,10 @@
         <v>1721</v>
       </c>
       <c r="D83" s="1" t="s">
-        <v>2979</v>
+        <v>3022</v>
       </c>
       <c r="E83" s="1" t="s">
-        <v>2980</v>
+        <v>3023</v>
       </c>
       <c r="F83" s="1" t="s">
         <v>1730</v>
@@ -29270,7 +29606,7 @@
         <v>52</v>
       </c>
       <c r="N83" s="1" t="s">
-        <v>2818</v>
+        <v>2861</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="84" spans="1:14">
@@ -29284,10 +29620,10 @@
         <v>1744</v>
       </c>
       <c r="D84" s="1" t="s">
-        <v>2981</v>
+        <v>3024</v>
       </c>
       <c r="E84" s="1" t="s">
-        <v>2982</v>
+        <v>3025</v>
       </c>
       <c r="F84" s="1" t="s">
         <v>1751</v>
@@ -29314,7 +29650,7 @@
         <v>52</v>
       </c>
       <c r="N84" s="1" t="s">
-        <v>2818</v>
+        <v>2861</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="85" spans="1:14">
@@ -29328,10 +29664,10 @@
         <v>1765</v>
       </c>
       <c r="D85" s="1" t="s">
-        <v>2983</v>
+        <v>3026</v>
       </c>
       <c r="E85" s="1" t="s">
-        <v>2984</v>
+        <v>3027</v>
       </c>
       <c r="F85" s="1" t="s">
         <v>1773</v>
@@ -29358,7 +29694,7 @@
         <v>145</v>
       </c>
       <c r="N85" s="1" t="s">
-        <v>2818</v>
+        <v>2861</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="86" spans="1:14">
@@ -29372,10 +29708,10 @@
         <v>1785</v>
       </c>
       <c r="D86" s="1" t="s">
-        <v>2985</v>
+        <v>3028</v>
       </c>
       <c r="E86" s="1" t="s">
-        <v>2986</v>
+        <v>3029</v>
       </c>
       <c r="F86" s="1" t="s">
         <v>1793</v>
@@ -29402,7 +29738,7 @@
         <v>52</v>
       </c>
       <c r="N86" s="1" t="s">
-        <v>2818</v>
+        <v>2861</v>
       </c>
     </row>
     <row customHeight="1" ht="110.4" r="87" spans="1:14">
@@ -29416,10 +29752,10 @@
         <v>1806</v>
       </c>
       <c r="D87" s="1" t="s">
-        <v>2987</v>
+        <v>3030</v>
       </c>
       <c r="E87" s="1" t="s">
-        <v>2988</v>
+        <v>3031</v>
       </c>
       <c r="F87" s="1" t="s">
         <v>1813</v>
@@ -29446,7 +29782,7 @@
         <v>145</v>
       </c>
       <c r="N87" s="1" t="s">
-        <v>2818</v>
+        <v>2861</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="88" spans="1:14">
@@ -29460,10 +29796,10 @@
         <v>1826</v>
       </c>
       <c r="D88" s="1" t="s">
-        <v>2989</v>
+        <v>3032</v>
       </c>
       <c r="E88" s="1" t="s">
-        <v>2990</v>
+        <v>3033</v>
       </c>
       <c r="F88" s="1" t="s">
         <v>1834</v>
@@ -29490,7 +29826,7 @@
         <v>52</v>
       </c>
       <c r="N88" s="1" t="s">
-        <v>2818</v>
+        <v>2861</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="89" spans="1:14">
@@ -29504,10 +29840,10 @@
         <v>1846</v>
       </c>
       <c r="D89" s="1" t="s">
-        <v>2991</v>
+        <v>3034</v>
       </c>
       <c r="E89" s="1" t="s">
-        <v>2992</v>
+        <v>3035</v>
       </c>
       <c r="F89" s="1" t="s">
         <v>1854</v>
@@ -29534,7 +29870,7 @@
         <v>52</v>
       </c>
       <c r="N89" s="1" t="s">
-        <v>2818</v>
+        <v>2861</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="90" spans="1:14">
@@ -29548,10 +29884,10 @@
         <v>1866</v>
       </c>
       <c r="D90" s="1" t="s">
-        <v>2993</v>
+        <v>3036</v>
       </c>
       <c r="E90" s="1" t="s">
-        <v>2994</v>
+        <v>3037</v>
       </c>
       <c r="F90" s="1" t="s">
         <v>1873</v>
@@ -29578,7 +29914,7 @@
         <v>52</v>
       </c>
       <c r="N90" s="1" t="s">
-        <v>2818</v>
+        <v>2861</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="91" spans="1:14">
@@ -29592,10 +29928,10 @@
         <v>1884</v>
       </c>
       <c r="D91" s="1" t="s">
-        <v>2995</v>
+        <v>3038</v>
       </c>
       <c r="E91" s="1" t="s">
-        <v>2996</v>
+        <v>3039</v>
       </c>
       <c r="F91" s="1" t="s">
         <v>1892</v>
@@ -29622,7 +29958,7 @@
         <v>145</v>
       </c>
       <c r="N91" s="1" t="s">
-        <v>2818</v>
+        <v>2861</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="92" spans="1:14">
@@ -29636,10 +29972,10 @@
         <v>1904</v>
       </c>
       <c r="D92" s="1" t="s">
-        <v>2997</v>
+        <v>3040</v>
       </c>
       <c r="E92" s="1" t="s">
-        <v>2998</v>
+        <v>3041</v>
       </c>
       <c r="F92" s="1" t="s">
         <v>1912</v>
@@ -29666,7 +30002,7 @@
         <v>189</v>
       </c>
       <c r="N92" s="1" t="s">
-        <v>2818</v>
+        <v>2861</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="93" spans="1:14">
@@ -29680,10 +30016,10 @@
         <v>1923</v>
       </c>
       <c r="D93" s="1" t="s">
-        <v>2999</v>
+        <v>3042</v>
       </c>
       <c r="E93" s="1" t="s">
-        <v>3000</v>
+        <v>3043</v>
       </c>
       <c r="F93" s="1" t="s">
         <v>1931</v>
@@ -29710,7 +30046,7 @@
         <v>52</v>
       </c>
       <c r="N93" s="1" t="s">
-        <v>2818</v>
+        <v>2861</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="94" spans="1:14">
@@ -29724,10 +30060,10 @@
         <v>1943</v>
       </c>
       <c r="D94" s="1" t="s">
-        <v>3001</v>
+        <v>3044</v>
       </c>
       <c r="E94" s="1" t="s">
-        <v>3002</v>
+        <v>3045</v>
       </c>
       <c r="F94" s="1" t="s">
         <v>1950</v>
@@ -29754,7 +30090,7 @@
         <v>52</v>
       </c>
       <c r="N94" s="1" t="s">
-        <v>2818</v>
+        <v>2861</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="95" spans="1:14">
@@ -29768,10 +30104,10 @@
         <v>1961</v>
       </c>
       <c r="D95" s="1" t="s">
-        <v>3003</v>
+        <v>3046</v>
       </c>
       <c r="E95" s="1" t="s">
-        <v>3004</v>
+        <v>3047</v>
       </c>
       <c r="F95" s="1" t="s">
         <v>1968</v>
@@ -29798,7 +30134,7 @@
         <v>52</v>
       </c>
       <c r="N95" s="1" t="s">
-        <v>2818</v>
+        <v>2861</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="96" spans="1:14">
@@ -29812,10 +30148,10 @@
         <v>1980</v>
       </c>
       <c r="D96" s="1" t="s">
-        <v>3005</v>
+        <v>3048</v>
       </c>
       <c r="E96" s="1" t="s">
-        <v>3006</v>
+        <v>3049</v>
       </c>
       <c r="F96" s="1" t="s">
         <v>1988</v>
@@ -29842,7 +30178,7 @@
         <v>52</v>
       </c>
       <c r="N96" s="1" t="s">
-        <v>2818</v>
+        <v>2861</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="97" spans="1:14">
@@ -29856,10 +30192,10 @@
         <v>2000</v>
       </c>
       <c r="D97" s="1" t="s">
-        <v>3007</v>
+        <v>3050</v>
       </c>
       <c r="E97" s="1" t="s">
-        <v>3008</v>
+        <v>3051</v>
       </c>
       <c r="F97" s="1" t="s">
         <v>2006</v>
@@ -29886,7 +30222,7 @@
         <v>52</v>
       </c>
       <c r="N97" s="1" t="s">
-        <v>2818</v>
+        <v>2861</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="98" spans="1:14">
@@ -29900,10 +30236,10 @@
         <v>2019</v>
       </c>
       <c r="D98" s="1" t="s">
-        <v>3009</v>
+        <v>3052</v>
       </c>
       <c r="E98" s="1" t="s">
-        <v>3010</v>
+        <v>3053</v>
       </c>
       <c r="F98" s="1" t="s">
         <v>2028</v>
@@ -29930,7 +30266,7 @@
         <v>145</v>
       </c>
       <c r="N98" s="1" t="s">
-        <v>2818</v>
+        <v>2861</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="99" spans="1:14">
@@ -29944,10 +30280,10 @@
         <v>2041</v>
       </c>
       <c r="D99" s="1" t="s">
-        <v>3011</v>
+        <v>3054</v>
       </c>
       <c r="E99" s="1" t="s">
-        <v>3012</v>
+        <v>3055</v>
       </c>
       <c r="F99" s="1" t="s">
         <v>2049</v>
@@ -29974,7 +30310,7 @@
         <v>145</v>
       </c>
       <c r="N99" s="1" t="s">
-        <v>2818</v>
+        <v>2861</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="100" spans="1:14">
@@ -29988,10 +30324,10 @@
         <v>2062</v>
       </c>
       <c r="D100" s="1" t="s">
-        <v>3013</v>
+        <v>3056</v>
       </c>
       <c r="E100" s="1" t="s">
-        <v>3014</v>
+        <v>3057</v>
       </c>
       <c r="F100" s="1" t="s">
         <v>2069</v>
@@ -30018,7 +30354,7 @@
         <v>145</v>
       </c>
       <c r="N100" s="1" t="s">
-        <v>2818</v>
+        <v>2861</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="101" spans="1:14">
@@ -30032,10 +30368,10 @@
         <v>2082</v>
       </c>
       <c r="D101" s="1" t="s">
-        <v>3015</v>
+        <v>3058</v>
       </c>
       <c r="E101" s="1" t="s">
-        <v>3016</v>
+        <v>3059</v>
       </c>
       <c r="F101" s="1" t="s">
         <v>2090</v>
@@ -30062,7 +30398,7 @@
         <v>52</v>
       </c>
       <c r="N101" s="1" t="s">
-        <v>2818</v>
+        <v>2861</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="102" spans="1:14">
@@ -30076,10 +30412,10 @@
         <v>2102</v>
       </c>
       <c r="D102" s="1" t="s">
-        <v>3017</v>
+        <v>3060</v>
       </c>
       <c r="E102" s="1" t="s">
-        <v>3018</v>
+        <v>3061</v>
       </c>
       <c r="F102" s="1" t="s">
         <v>2110</v>
@@ -30106,7 +30442,7 @@
         <v>145</v>
       </c>
       <c r="N102" s="1" t="s">
-        <v>2818</v>
+        <v>2861</v>
       </c>
     </row>
     <row customHeight="1" ht="82.8" r="103" spans="1:14">
@@ -30120,10 +30456,10 @@
         <v>2122</v>
       </c>
       <c r="D103" s="1" t="s">
-        <v>3019</v>
+        <v>3062</v>
       </c>
       <c r="E103" s="1" t="s">
-        <v>3020</v>
+        <v>3063</v>
       </c>
       <c r="F103" s="1" t="s">
         <v>2129</v>
@@ -30150,7 +30486,7 @@
         <v>145</v>
       </c>
       <c r="N103" s="1" t="s">
-        <v>2818</v>
+        <v>2861</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="104" spans="1:14">
@@ -30164,10 +30500,10 @@
         <v>2142</v>
       </c>
       <c r="D104" s="1" t="s">
-        <v>3021</v>
+        <v>3064</v>
       </c>
       <c r="E104" s="1" t="s">
-        <v>3022</v>
+        <v>3065</v>
       </c>
       <c r="F104" s="1" t="s">
         <v>2149</v>
@@ -30194,7 +30530,7 @@
         <v>145</v>
       </c>
       <c r="N104" s="1" t="s">
-        <v>2818</v>
+        <v>2861</v>
       </c>
     </row>
     <row customHeight="1" ht="82.8" r="105" spans="1:14">
@@ -30208,10 +30544,10 @@
         <v>2161</v>
       </c>
       <c r="D105" s="1" t="s">
-        <v>3023</v>
+        <v>3066</v>
       </c>
       <c r="E105" s="1" t="s">
-        <v>3024</v>
+        <v>3067</v>
       </c>
       <c r="F105" s="1" t="s">
         <v>2168</v>
@@ -30238,7 +30574,7 @@
         <v>145</v>
       </c>
       <c r="N105" s="1" t="s">
-        <v>2818</v>
+        <v>2861</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="106" spans="1:14">
@@ -30252,10 +30588,10 @@
         <v>2181</v>
       </c>
       <c r="D106" s="1" t="s">
-        <v>3025</v>
+        <v>3068</v>
       </c>
       <c r="E106" s="1" t="s">
-        <v>3026</v>
+        <v>3069</v>
       </c>
       <c r="F106" s="1" t="s">
         <v>2187</v>
@@ -30282,7 +30618,7 @@
         <v>189</v>
       </c>
       <c r="N106" s="1" t="s">
-        <v>2818</v>
+        <v>2861</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="107" spans="1:14">
@@ -30296,10 +30632,10 @@
         <v>2201</v>
       </c>
       <c r="D107" s="1" t="s">
-        <v>3027</v>
+        <v>3070</v>
       </c>
       <c r="E107" s="1" t="s">
-        <v>3028</v>
+        <v>3071</v>
       </c>
       <c r="F107" s="1" t="s">
         <v>2209</v>
@@ -30326,7 +30662,7 @@
         <v>145</v>
       </c>
       <c r="N107" s="1" t="s">
-        <v>2818</v>
+        <v>2861</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="108" spans="1:14">
@@ -30340,10 +30676,10 @@
         <v>2222</v>
       </c>
       <c r="D108" s="1" t="s">
-        <v>3029</v>
+        <v>3072</v>
       </c>
       <c r="E108" s="1" t="s">
-        <v>3030</v>
+        <v>3073</v>
       </c>
       <c r="F108" s="1" t="s">
         <v>2228</v>
@@ -30370,7 +30706,7 @@
         <v>52</v>
       </c>
       <c r="N108" s="1" t="s">
-        <v>2818</v>
+        <v>2861</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="109" spans="1:14">
@@ -30384,10 +30720,10 @@
         <v>2241</v>
       </c>
       <c r="D109" s="1" t="s">
-        <v>3031</v>
+        <v>3074</v>
       </c>
       <c r="E109" s="1" t="s">
-        <v>3032</v>
+        <v>3075</v>
       </c>
       <c r="F109" s="1" t="s">
         <v>2247</v>
@@ -30414,7 +30750,7 @@
         <v>52</v>
       </c>
       <c r="N109" s="1" t="s">
-        <v>2818</v>
+        <v>2861</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="110" spans="1:14">
@@ -30428,10 +30764,10 @@
         <v>2259</v>
       </c>
       <c r="D110" s="1" t="s">
-        <v>3033</v>
+        <v>3076</v>
       </c>
       <c r="E110" s="1" t="s">
-        <v>3034</v>
+        <v>3077</v>
       </c>
       <c r="F110" s="1" t="s">
         <v>2268</v>
@@ -30458,7 +30794,7 @@
         <v>145</v>
       </c>
       <c r="N110" s="1" t="s">
-        <v>2818</v>
+        <v>2861</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="111" spans="1:14">
@@ -30472,10 +30808,10 @@
         <v>2281</v>
       </c>
       <c r="D111" s="1" t="s">
-        <v>3035</v>
+        <v>3078</v>
       </c>
       <c r="E111" s="1" t="s">
-        <v>3036</v>
+        <v>3079</v>
       </c>
       <c r="F111" s="1" t="s">
         <v>2289</v>
@@ -30502,7 +30838,7 @@
         <v>52</v>
       </c>
       <c r="N111" s="1" t="s">
-        <v>2818</v>
+        <v>2861</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="112" spans="1:14">
@@ -30516,10 +30852,10 @@
         <v>2302</v>
       </c>
       <c r="D112" s="1" t="s">
-        <v>3037</v>
+        <v>3080</v>
       </c>
       <c r="E112" s="1" t="s">
-        <v>3038</v>
+        <v>3081</v>
       </c>
       <c r="F112" s="1" t="s">
         <v>2311</v>
@@ -30546,7 +30882,7 @@
         <v>145</v>
       </c>
       <c r="N112" s="1" t="s">
-        <v>2818</v>
+        <v>2861</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="113" spans="1:14">
@@ -30560,10 +30896,10 @@
         <v>2324</v>
       </c>
       <c r="D113" s="1" t="s">
-        <v>3039</v>
+        <v>3082</v>
       </c>
       <c r="E113" s="1" t="s">
-        <v>3040</v>
+        <v>3083</v>
       </c>
       <c r="F113" s="1" t="s">
         <v>2331</v>
@@ -30590,7 +30926,7 @@
         <v>145</v>
       </c>
       <c r="N113" s="1" t="s">
-        <v>2818</v>
+        <v>2861</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="114" spans="1:14">
@@ -30604,10 +30940,10 @@
         <v>2343</v>
       </c>
       <c r="D114" s="1" t="s">
-        <v>3041</v>
+        <v>3084</v>
       </c>
       <c r="E114" s="1" t="s">
-        <v>3042</v>
+        <v>3085</v>
       </c>
       <c r="F114" s="1" t="s">
         <v>2350</v>
@@ -30634,7 +30970,7 @@
         <v>145</v>
       </c>
       <c r="N114" s="1" t="s">
-        <v>2818</v>
+        <v>2861</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="115" spans="1:14">
@@ -30648,10 +30984,10 @@
         <v>2362</v>
       </c>
       <c r="D115" s="1" t="s">
-        <v>3043</v>
+        <v>3086</v>
       </c>
       <c r="E115" s="1" t="s">
-        <v>3044</v>
+        <v>3087</v>
       </c>
       <c r="F115" s="1" t="s">
         <v>2369</v>
@@ -30678,7 +31014,7 @@
         <v>52</v>
       </c>
       <c r="N115" s="1" t="s">
-        <v>2818</v>
+        <v>2861</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="116" spans="1:14">
@@ -30692,10 +31028,10 @@
         <v>2381</v>
       </c>
       <c r="D116" s="1" t="s">
-        <v>3045</v>
+        <v>3088</v>
       </c>
       <c r="E116" s="1" t="s">
-        <v>3046</v>
+        <v>3089</v>
       </c>
       <c r="F116" s="1" t="s">
         <v>2389</v>
@@ -30722,7 +31058,7 @@
         <v>145</v>
       </c>
       <c r="N116" s="1" t="s">
-        <v>2818</v>
+        <v>2861</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="117" spans="1:14">
@@ -30736,10 +31072,10 @@
         <v>2401</v>
       </c>
       <c r="D117" s="1" t="s">
-        <v>3047</v>
+        <v>3090</v>
       </c>
       <c r="E117" s="1" t="s">
-        <v>3048</v>
+        <v>3091</v>
       </c>
       <c r="F117" s="1" t="s">
         <v>2410</v>
@@ -30766,7 +31102,7 @@
         <v>145</v>
       </c>
       <c r="N117" s="1" t="s">
-        <v>2818</v>
+        <v>2861</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="118" spans="1:14">
@@ -30780,10 +31116,10 @@
         <v>2423</v>
       </c>
       <c r="D118" s="1" t="s">
-        <v>3049</v>
+        <v>3092</v>
       </c>
       <c r="E118" s="1" t="s">
-        <v>3050</v>
+        <v>3093</v>
       </c>
       <c r="F118" s="1" t="s">
         <v>2431</v>
@@ -30810,7 +31146,7 @@
         <v>145</v>
       </c>
       <c r="N118" s="1" t="s">
-        <v>2818</v>
+        <v>2861</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="119" spans="1:14">
@@ -30824,10 +31160,10 @@
         <v>2443</v>
       </c>
       <c r="D119" s="1" t="s">
-        <v>3051</v>
+        <v>3094</v>
       </c>
       <c r="E119" s="1" t="s">
-        <v>3052</v>
+        <v>3095</v>
       </c>
       <c r="F119" s="1" t="s">
         <v>2450</v>
@@ -30854,7 +31190,7 @@
         <v>52</v>
       </c>
       <c r="N119" s="1" t="s">
-        <v>2818</v>
+        <v>2861</v>
       </c>
     </row>
     <row customHeight="1" ht="82.8" r="120" spans="1:14">
@@ -30868,10 +31204,10 @@
         <v>2462</v>
       </c>
       <c r="D120" s="1" t="s">
-        <v>3053</v>
+        <v>3096</v>
       </c>
       <c r="E120" s="1" t="s">
-        <v>3054</v>
+        <v>3097</v>
       </c>
       <c r="F120" s="1" t="s">
         <v>2470</v>
@@ -30906,10 +31242,10 @@
         <v>2483</v>
       </c>
       <c r="D121" s="1" t="s">
-        <v>3055</v>
+        <v>3098</v>
       </c>
       <c r="E121" s="1" t="s">
-        <v>3056</v>
+        <v>3099</v>
       </c>
       <c r="F121" s="1" t="s">
         <v>2492</v>
@@ -30944,10 +31280,10 @@
         <v>2503</v>
       </c>
       <c r="D122" s="1" t="s">
-        <v>3057</v>
+        <v>3100</v>
       </c>
       <c r="E122" s="1" t="s">
-        <v>3058</v>
+        <v>3101</v>
       </c>
       <c r="F122" s="1" t="s">
         <v>2508</v>
@@ -30982,10 +31318,10 @@
         <v>2521</v>
       </c>
       <c r="D123" t="s">
-        <v>3059</v>
+        <v>3102</v>
       </c>
       <c r="E123" t="s">
-        <v>3060</v>
+        <v>3103</v>
       </c>
       <c r="F123" t="s">
         <v>2528</v>
@@ -31012,7 +31348,7 @@
         <v>52</v>
       </c>
       <c r="N123" t="s">
-        <v>3061</v>
+        <v>3104</v>
       </c>
     </row>
     <row r="124" spans="1:14">
@@ -31029,7 +31365,7 @@
         <v>2546</v>
       </c>
       <c r="E124" t="s">
-        <v>3062</v>
+        <v>3105</v>
       </c>
       <c r="F124" t="s">
         <v>2547</v>
@@ -31056,7 +31392,7 @@
         <v>52</v>
       </c>
       <c r="N124" t="s">
-        <v>3061</v>
+        <v>3104</v>
       </c>
     </row>
     <row r="125" spans="1:14">
@@ -31073,7 +31409,7 @@
         <v>2564</v>
       </c>
       <c r="E125" t="s">
-        <v>3063</v>
+        <v>3106</v>
       </c>
       <c r="F125" t="s">
         <v>2565</v>
@@ -31100,7 +31436,7 @@
         <v>189</v>
       </c>
       <c r="N125" t="s">
-        <v>3061</v>
+        <v>3104</v>
       </c>
     </row>
     <row r="126" spans="1:14">
@@ -31117,7 +31453,7 @@
         <v>2582</v>
       </c>
       <c r="E126" t="s">
-        <v>3064</v>
+        <v>3107</v>
       </c>
       <c r="G126" t="s">
         <v>2586</v>
@@ -31135,10 +31471,10 @@
         <v>2590</v>
       </c>
       <c r="M126" t="s">
-        <v>3065</v>
+        <v>3108</v>
       </c>
       <c r="N126" t="s">
-        <v>3061</v>
+        <v>3104</v>
       </c>
     </row>
     <row r="127" spans="1:14">
@@ -31155,7 +31491,7 @@
         <v>2601</v>
       </c>
       <c r="E127" t="s">
-        <v>3066</v>
+        <v>3109</v>
       </c>
       <c r="G127" t="s">
         <v>2604</v>
@@ -31176,7 +31512,7 @@
         <v>52</v>
       </c>
       <c r="N127" t="s">
-        <v>3061</v>
+        <v>3104</v>
       </c>
     </row>
     <row r="128" spans="1:14">
@@ -31187,7 +31523,7 @@
         <v>2614</v>
       </c>
       <c r="E128" t="s">
-        <v>3067</v>
+        <v>3110</v>
       </c>
       <c r="G128" t="s">
         <v>2621</v>
@@ -31205,10 +31541,10 @@
         <v>2625</v>
       </c>
       <c r="M128" t="s">
-        <v>3065</v>
+        <v>3108</v>
       </c>
       <c r="N128" t="s">
-        <v>3061</v>
+        <v>3104</v>
       </c>
     </row>
     <row r="129" spans="1:14">
@@ -31219,7 +31555,7 @@
         <v>2632</v>
       </c>
       <c r="E129" t="s">
-        <v>3068</v>
+        <v>3111</v>
       </c>
       <c r="G129" t="s">
         <v>2639</v>
@@ -31237,7 +31573,7 @@
         <v>52</v>
       </c>
       <c r="N129" t="s">
-        <v>3061</v>
+        <v>3104</v>
       </c>
     </row>
     <row r="130" spans="1:14">
@@ -31248,7 +31584,7 @@
         <v>2650</v>
       </c>
       <c r="E130" t="s">
-        <v>3069</v>
+        <v>3112</v>
       </c>
       <c r="G130" t="s">
         <v>2658</v>
@@ -31269,7 +31605,7 @@
         <v>52</v>
       </c>
       <c r="N130" t="s">
-        <v>3061</v>
+        <v>3104</v>
       </c>
     </row>
     <row r="131" spans="1:14">
@@ -31283,7 +31619,7 @@
         <v>2673</v>
       </c>
       <c r="E131" t="s">
-        <v>3070</v>
+        <v>3113</v>
       </c>
       <c r="G131" t="s">
         <v>2676</v>
@@ -31301,7 +31637,7 @@
         <v>52</v>
       </c>
       <c r="N131" t="s">
-        <v>3061</v>
+        <v>3104</v>
       </c>
     </row>
     <row r="132" spans="1:14">
@@ -31312,7 +31648,7 @@
         <v>2687</v>
       </c>
       <c r="E132" t="s">
-        <v>3071</v>
+        <v>3114</v>
       </c>
       <c r="G132" t="s">
         <v>2695</v>
@@ -31333,7 +31669,7 @@
         <v>52</v>
       </c>
       <c r="N132" t="s">
-        <v>3061</v>
+        <v>3104</v>
       </c>
     </row>
     <row r="133" spans="1:14">
@@ -31347,7 +31683,7 @@
         <v>2705</v>
       </c>
       <c r="E133" t="s">
-        <v>3072</v>
+        <v>3115</v>
       </c>
       <c r="I133" t="s">
         <v>2714</v>
@@ -31362,7 +31698,7 @@
         <v>52</v>
       </c>
       <c r="N133" t="s">
-        <v>3061</v>
+        <v>3104</v>
       </c>
     </row>
     <row r="134" spans="1:14">
@@ -31373,7 +31709,7 @@
         <v>2722</v>
       </c>
       <c r="E134" t="s">
-        <v>3073</v>
+        <v>3116</v>
       </c>
       <c r="I134" t="s">
         <v>2733</v>
@@ -31385,7 +31721,7 @@
         <v>52</v>
       </c>
       <c r="N134" t="s">
-        <v>3061</v>
+        <v>3104</v>
       </c>
     </row>
     <row r="135" spans="1:14">
@@ -31396,7 +31732,7 @@
         <v>2744</v>
       </c>
       <c r="E135" t="s">
-        <v>3074</v>
+        <v>3117</v>
       </c>
       <c r="G135" t="s">
         <v>2754</v>
@@ -31417,7 +31753,47 @@
         <v>52</v>
       </c>
       <c r="N135" t="s">
-        <v>3061</v>
+        <v>3104</v>
+      </c>
+    </row>
+    <row r="136" spans="1:14">
+      <c r="A136" t="s">
+        <v>2761</v>
+      </c>
+      <c r="C136" t="s">
+        <v>2765</v>
+      </c>
+      <c r="E136" t="s">
+        <v>3118</v>
+      </c>
+      <c r="J136" t="s">
+        <v>3119</v>
+      </c>
+      <c r="M136" t="s">
+        <v>52</v>
+      </c>
+      <c r="N136" t="s">
+        <v>3104</v>
+      </c>
+    </row>
+    <row r="137" spans="1:14">
+      <c r="A137" t="s">
+        <v>2783</v>
+      </c>
+      <c r="C137" t="s">
+        <v>2788</v>
+      </c>
+      <c r="E137" t="s">
+        <v>3120</v>
+      </c>
+      <c r="J137" t="s">
+        <v>3121</v>
+      </c>
+      <c r="M137" t="s">
+        <v>52</v>
+      </c>
+      <c r="N137" t="s">
+        <v>3104</v>
       </c>
     </row>
   </sheetData>
@@ -31431,7 +31807,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B13"/>
+  <dimension ref="A1:B14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="13.8" outlineLevelCol="0"/>
   <cols>
     <col customWidth="1" max="2" min="1" width="50"/>
@@ -31439,106 +31815,114 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="7" t="s">
-        <v>3075</v>
+        <v>3122</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>3076</v>
+        <v>3123</v>
       </c>
     </row>
     <row r="2" spans="1:2">
       <c r="A2" t="s">
-        <v>3077</v>
+        <v>3124</v>
       </c>
       <c r="B2" t="s">
-        <v>2770</v>
+        <v>2813</v>
       </c>
     </row>
     <row r="3" spans="1:2">
       <c r="A3" t="s">
-        <v>3078</v>
+        <v>3125</v>
       </c>
       <c r="B3" t="s">
-        <v>3079</v>
+        <v>3126</v>
       </c>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" t="s">
-        <v>3080</v>
+        <v>3127</v>
       </c>
       <c r="B4" t="s">
-        <v>3081</v>
+        <v>3128</v>
       </c>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" t="s">
-        <v>3082</v>
+        <v>3129</v>
       </c>
       <c r="B5" t="s">
-        <v>3083</v>
+        <v>3130</v>
       </c>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" t="s">
-        <v>3084</v>
+        <v>3131</v>
       </c>
       <c r="B6" t="s">
-        <v>3085</v>
+        <v>3132</v>
       </c>
     </row>
     <row r="7" spans="1:2">
       <c r="A7" t="s">
-        <v>3086</v>
+        <v>3133</v>
       </c>
       <c r="B7" t="s">
-        <v>3087</v>
+        <v>3134</v>
       </c>
     </row>
     <row r="8" spans="1:2">
       <c r="A8" t="s">
-        <v>3088</v>
+        <v>3135</v>
       </c>
       <c r="B8" t="s">
-        <v>3089</v>
+        <v>3136</v>
       </c>
     </row>
     <row r="9" spans="1:2">
       <c r="A9" t="s">
-        <v>3090</v>
+        <v>3137</v>
       </c>
       <c r="B9" t="s">
-        <v>3091</v>
+        <v>3138</v>
       </c>
     </row>
     <row r="10" spans="1:2">
       <c r="A10" t="s">
-        <v>3092</v>
+        <v>3139</v>
       </c>
       <c r="B10" t="s">
-        <v>3093</v>
+        <v>3140</v>
       </c>
     </row>
     <row r="11" spans="1:2">
       <c r="A11" t="s">
-        <v>3094</v>
+        <v>3141</v>
       </c>
       <c r="B11" t="s">
-        <v>3095</v>
+        <v>3142</v>
       </c>
     </row>
     <row r="12" spans="1:2">
       <c r="A12" t="s">
-        <v>3096</v>
+        <v>3143</v>
       </c>
       <c r="B12" t="s">
-        <v>3097</v>
+        <v>3144</v>
       </c>
     </row>
     <row r="13" spans="1:2">
       <c r="A13" t="s">
-        <v>3098</v>
+        <v>3145</v>
       </c>
       <c r="B13" t="s">
-        <v>3099</v>
+        <v>3146</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2">
+      <c r="A14" t="s">
+        <v>3147</v>
+      </c>
+      <c r="B14" t="s">
+        <v>3148</v>
       </c>
     </row>
   </sheetData>
@@ -31557,82 +31941,82 @@
   <sheetData>
     <row customHeight="1" ht="27.6" r="1" spans="1:6">
       <c r="A1" s="6" t="s">
-        <v>3100</v>
+        <v>3149</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>3101</v>
+        <v>3150</v>
       </c>
       <c r="C1" s="6" t="s">
-        <v>3102</v>
+        <v>3151</v>
       </c>
       <c r="D1" s="6" t="s">
-        <v>3103</v>
+        <v>3152</v>
       </c>
       <c r="E1" s="6" t="s">
-        <v>3104</v>
+        <v>3153</v>
       </c>
       <c r="F1" s="6" t="s">
-        <v>3105</v>
+        <v>3154</v>
       </c>
     </row>
     <row customHeight="1" ht="55.2" r="2" spans="1:6">
       <c r="A2" s="1" t="s">
-        <v>3106</v>
+        <v>3155</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>38</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>3107</v>
+        <v>3156</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>3108</v>
+        <v>3157</v>
       </c>
       <c r="E2" s="1" t="s">
         <v>28</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>3109</v>
+        <v>3158</v>
       </c>
     </row>
     <row customHeight="1" ht="55.2" r="3" spans="1:6">
       <c r="A3" s="1" t="s">
-        <v>3110</v>
+        <v>3159</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>1681</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>3107</v>
+        <v>3156</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>3108</v>
+        <v>3157</v>
       </c>
       <c r="E3" s="1" t="s">
         <v>1674</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>3109</v>
+        <v>3158</v>
       </c>
     </row>
     <row customHeight="1" ht="55.2" r="4" spans="1:6">
       <c r="A4" s="1" t="s">
-        <v>3111</v>
+        <v>3160</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>1167</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>3107</v>
+        <v>3156</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>3108</v>
+        <v>3157</v>
       </c>
       <c r="E4" s="1" t="s">
         <v>1161</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>3109</v>
+        <v>3158</v>
       </c>
     </row>
     <row customHeight="1" ht="82.8" r="5" spans="1:6">
@@ -31643,16 +32027,16 @@
         <v>2204</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>3112</v>
+        <v>3161</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>3113</v>
+        <v>3162</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>3114</v>
+        <v>3163</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>3115</v>
+        <v>3164</v>
       </c>
     </row>
     <row customHeight="1" ht="82.8" r="6" spans="1:6">
@@ -31663,16 +32047,16 @@
         <v>2223</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>3112</v>
+        <v>3161</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>3113</v>
+        <v>3162</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>3114</v>
+        <v>3163</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>3115</v>
+        <v>3164</v>
       </c>
     </row>
     <row customHeight="1" ht="82.8" r="7" spans="1:6">
@@ -31683,16 +32067,16 @@
         <v>2243</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>3112</v>
+        <v>3161</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>3113</v>
+        <v>3162</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>3114</v>
+        <v>3163</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>3115</v>
+        <v>3164</v>
       </c>
     </row>
     <row customHeight="1" ht="82.8" r="8" spans="1:6">
@@ -31703,16 +32087,16 @@
         <v>2262</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>3112</v>
+        <v>3161</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>3113</v>
+        <v>3162</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>3114</v>
+        <v>3163</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>3115</v>
+        <v>3164</v>
       </c>
     </row>
     <row customHeight="1" ht="82.8" r="9" spans="1:6">
@@ -31723,16 +32107,16 @@
         <v>2283</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>3112</v>
+        <v>3161</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>3113</v>
+        <v>3162</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>3114</v>
+        <v>3163</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>3115</v>
+        <v>3164</v>
       </c>
     </row>
     <row customHeight="1" ht="82.8" r="10" spans="1:6">
@@ -31743,16 +32127,16 @@
         <v>2305</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>3112</v>
+        <v>3161</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>3113</v>
+        <v>3162</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>3114</v>
+        <v>3163</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>3115</v>
+        <v>3164</v>
       </c>
     </row>
     <row customHeight="1" ht="82.8" r="11" spans="1:6">
@@ -31763,16 +32147,16 @@
         <v>2326</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>3112</v>
+        <v>3161</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>3113</v>
+        <v>3162</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>3114</v>
+        <v>3163</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>3115</v>
+        <v>3164</v>
       </c>
     </row>
     <row customHeight="1" ht="82.8" r="12" spans="1:6">
@@ -31783,16 +32167,16 @@
         <v>2346</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>3112</v>
+        <v>3161</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>3113</v>
+        <v>3162</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>3114</v>
+        <v>3163</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>3115</v>
+        <v>3164</v>
       </c>
     </row>
     <row customHeight="1" ht="82.8" r="13" spans="1:6">
@@ -31803,16 +32187,16 @@
         <v>2364</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>3112</v>
+        <v>3161</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>3113</v>
+        <v>3162</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>3114</v>
+        <v>3163</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>3115</v>
+        <v>3164</v>
       </c>
     </row>
     <row customHeight="1" ht="82.8" r="14" spans="1:6">
@@ -31823,16 +32207,16 @@
         <v>2383</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>3112</v>
+        <v>3161</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>3113</v>
+        <v>3162</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>3114</v>
+        <v>3163</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>3115</v>
+        <v>3164</v>
       </c>
     </row>
     <row customHeight="1" ht="82.8" r="15" spans="1:6">
@@ -31843,16 +32227,16 @@
         <v>2404</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>3112</v>
+        <v>3161</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>3113</v>
+        <v>3162</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>3114</v>
+        <v>3163</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>3115</v>
+        <v>3164</v>
       </c>
     </row>
     <row customHeight="1" ht="82.8" r="16" spans="1:6">
@@ -31863,16 +32247,16 @@
         <v>2425</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>3112</v>
+        <v>3161</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>3113</v>
+        <v>3162</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>3114</v>
+        <v>3163</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>3115</v>
+        <v>3164</v>
       </c>
     </row>
     <row customHeight="1" ht="82.8" r="17" spans="1:6">
@@ -31883,96 +32267,96 @@
         <v>2445</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>3112</v>
+        <v>3161</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>3113</v>
+        <v>3162</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>3114</v>
+        <v>3163</v>
       </c>
       <c r="F17" s="1" t="s">
-        <v>3115</v>
+        <v>3164</v>
       </c>
     </row>
     <row customHeight="1" ht="303.6" r="18" spans="1:6">
       <c r="A18" s="1" t="s">
-        <v>3116</v>
+        <v>3165</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>3117</v>
+        <v>3166</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>3107</v>
+        <v>3156</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>3118</v>
+        <v>3167</v>
       </c>
       <c r="E18" s="1" t="s">
         <v>610</v>
       </c>
       <c r="F18" s="1" t="s">
-        <v>3119</v>
+        <v>3168</v>
       </c>
     </row>
     <row customHeight="1" ht="276" r="19" spans="1:6">
       <c r="A19" s="1" t="s">
-        <v>3120</v>
+        <v>3169</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>3121</v>
+        <v>3170</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>3122</v>
+        <v>3171</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>3123</v>
+        <v>3172</v>
       </c>
       <c r="E19" s="1" t="s">
         <v>2458</v>
       </c>
       <c r="F19" s="1" t="s">
-        <v>3112</v>
+        <v>3161</v>
       </c>
     </row>
     <row customHeight="1" ht="193.2" r="20" spans="1:6">
       <c r="A20" s="1" t="s">
-        <v>3124</v>
+        <v>3173</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>3125</v>
+        <v>3174</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>3122</v>
+        <v>3171</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>3123</v>
+        <v>3172</v>
       </c>
       <c r="E20" s="1" t="s">
         <v>2479</v>
       </c>
       <c r="F20" s="1" t="s">
-        <v>3112</v>
+        <v>3161</v>
       </c>
     </row>
     <row customHeight="1" ht="276" r="21" spans="1:6">
       <c r="A21" s="1" t="s">
-        <v>3126</v>
+        <v>3175</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>3127</v>
+        <v>3176</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>3122</v>
+        <v>3171</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>3123</v>
+        <v>3172</v>
       </c>
       <c r="E21" s="1" t="s">
         <v>2500</v>
       </c>
       <c r="F21" s="1" t="s">
-        <v>3112</v>
+        <v>3161</v>
       </c>
     </row>
   </sheetData>
@@ -31986,7 +32370,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B13"/>
+  <dimension ref="A1:B14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="13.8" outlineLevelCol="0"/>
   <cols>
     <col customWidth="1" max="2" min="1" width="42"/>
@@ -31994,15 +32378,15 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="8" t="s">
-        <v>3128</v>
+        <v>3177</v>
       </c>
       <c r="B1" s="8" t="s">
-        <v>3129</v>
+        <v>3178</v>
       </c>
     </row>
     <row r="2" spans="1:2">
       <c r="A2" t="s">
-        <v>3130</v>
+        <v>3179</v>
       </c>
       <c r="B2" t="n">
         <v>118</v>
@@ -32010,7 +32394,7 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" t="s">
-        <v>3131</v>
+        <v>3180</v>
       </c>
       <c r="B3" t="n">
         <v>1</v>
@@ -32018,7 +32402,7 @@
     </row>
     <row r="4" spans="1:2">
       <c r="A4" t="s">
-        <v>3132</v>
+        <v>3181</v>
       </c>
       <c r="B4" t="n">
         <v>0</v>
@@ -32026,7 +32410,7 @@
     </row>
     <row r="5" spans="1:2">
       <c r="A5" t="s">
-        <v>3133</v>
+        <v>3182</v>
       </c>
       <c r="B5" t="s">
         <v>2440</v>
@@ -32034,66 +32418,74 @@
     </row>
     <row r="6" spans="1:2">
       <c r="A6" t="s">
-        <v>3134</v>
+        <v>3183</v>
       </c>
       <c r="B6" t="s">
-        <v>3135</v>
+        <v>3184</v>
       </c>
     </row>
     <row r="7" spans="1:2">
       <c r="A7" t="s">
-        <v>3136</v>
+        <v>3185</v>
       </c>
       <c r="B7" t="s">
-        <v>3137</v>
+        <v>3186</v>
       </c>
     </row>
     <row r="8" spans="1:2">
       <c r="A8" t="s">
-        <v>3138</v>
+        <v>3187</v>
       </c>
       <c r="B8" t="s">
-        <v>3139</v>
+        <v>3188</v>
       </c>
     </row>
     <row r="9" spans="1:2">
       <c r="A9" t="s">
-        <v>3140</v>
+        <v>3189</v>
       </c>
       <c r="B9" t="s">
-        <v>3141</v>
+        <v>3190</v>
       </c>
     </row>
     <row r="10" spans="1:2">
       <c r="A10" t="s">
-        <v>3092</v>
+        <v>3139</v>
       </c>
       <c r="B10" t="s">
-        <v>3093</v>
+        <v>3140</v>
       </c>
     </row>
     <row r="11" spans="1:2">
       <c r="A11" t="s">
-        <v>3142</v>
+        <v>3191</v>
       </c>
       <c r="B11" t="s">
-        <v>3137</v>
+        <v>3186</v>
       </c>
     </row>
     <row r="12" spans="1:2">
       <c r="A12" t="s">
-        <v>3143</v>
+        <v>3192</v>
       </c>
       <c r="B12" t="s">
-        <v>3144</v>
+        <v>3193</v>
       </c>
     </row>
     <row r="13" spans="1:2">
       <c r="A13" t="s">
-        <v>3145</v>
+        <v>3194</v>
       </c>
       <c r="B13" t="s">
-        <v>3146</v>
+        <v>3195</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2">
+      <c r="A14" t="s">
+        <v>3196</v>
+      </c>
+      <c r="B14" t="s">
+        <v>3197</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix: update 总览统计 year counts and fill 精读摘要 missing cells
- 总览统计: 2026=50, added 2027=2, updated metadata rows
- 精读摘要: filled 15 entries (DCBM-119 through DCBM-136)
  - 66 cells filled across year/title/area/purpose/methods/findings/innovation/limitations/relevance/chapters/priority/upgrade
  - All records now have complete 14-column entries
- DCBM-135/136: all 14 columns verified OK
</commit_message>
<xml_diff>
--- a/00_Master/Deep_CBM_Latest.xlsx
+++ b/00_Master/Deep_CBM_Latest.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView activeTab="4" autoFilterDateGrouping="1" firstSheet="0" minimized="0" showHorizontalScroll="1" showSheetTabs="1" showVerticalScroll="1" tabRatio="600" visibility="visible" windowHeight="16776" windowWidth="30936" xWindow="-108" yWindow="-108"/>
+    <workbookView activeTab="6" autoFilterDateGrouping="1" firstSheet="0" minimized="0" showHorizontalScroll="1" showSheetTabs="1" showVerticalScroll="1" tabRatio="600" visibility="visible" windowHeight="16776" windowWidth="30936" xWindow="-108" yWindow="-108"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="完整文献矩阵" sheetId="1" state="visible" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="3198">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="3207">
   <si>
     <t>序号</t>
   </si>
@@ -8467,7 +8467,7 @@
     <t>累计文献数</t>
   </si>
   <si>
-    <t>2026-07-10 更新</t>
+    <t>2026-07-24 更新</t>
   </si>
   <si>
     <t>本批新增</t>
@@ -9930,6 +9930,9 @@
 【创新点】将 PSO-ELM 用于地质工程一体化压裂甜点评价
 【局限性】跨区块泛化需验证；机器学习可解释性需增强
 【与你课题的关系】可作为响应差异的地质工程背景变量参考</t>
+  </si>
+  <si>
+    <t>由 Daily Brief 生成；待全文精读增强</t>
   </si>
   <si>
     <t>研究区/对象：Ordos Basin；Deep coal measures; No. 8 coal seam；深度：No. 8 seam thickness 6-16 m, average 7.8 m。</t>
@@ -9969,9 +9972,6 @@
 论文引言、理论基础和讨论章节的术语统一。</t>
   </si>
   <si>
-    <t>由 Daily Brief 生成；待全文精读增强</t>
-  </si>
-  <si>
     <t>【研究目的】该文研究煤岩气聚集过渡带的形成机制，重点应涉及煤岩气在区域成藏体系中的空间过渡、气体富集差异和地质边界特征。
 【数据/方法】官方页面能够稳定核验题名、作者、卷期、页码、DOI 和出版日期，但摘要内容未正常加载。当前无法确认研究区、样品量、测井资料、地球化学数据或数值模拟方法。Codex 入库时应从 PDF 或正式中文页面补齐这些字段。
 【核心发现】根据题名可确认文章提出或解释了煤岩气聚集过渡带的形成机制，但具体机制组成、控制因素和区域适用性尚不能从当前公开页面可靠提取。
@@ -10007,6 +10007,9 @@
 【局限性】深度阈值和压裂体系不可直接外推。</t>
   </si>
   <si>
+    <t>未指定具体区块（实验与分子模拟研究）; 深部煤岩；吸附态甲烷; 深部煤岩储层（实验条件模拟深部温压）</t>
+  </si>
+  <si>
     <t>【数据/方法】渗吸、孔隙表征、吸附/解吸和分子动力学。
 【核心发现】0.3–1.5 nm 孔尺度增加 59.6%，2–10 nm 增加 44.8%；CH₄—煤配位数 16.2→12.3，水—煤 0→9.6；模拟能垒约 1500→800 kJ/mol。
 【创新点】统一解释润湿性、孔隙重构和水膜竞争吸附。
@@ -10014,10 +10017,17 @@
 【与你课题的关系】水锁、液相滞留、解吸启动、裂缝—基质传质。</t>
   </si>
   <si>
+    <t>鄂尔多斯东缘本溪组 3 口井、17 件煤样。
+- 方法：工业分析、CO₂ 吸附、高温高压甲烷吸附、等量吸附热; 鄂尔多斯东缘本溪组深部煤储层；3口井17件煤样; 鄂尔多斯东缘本溪组深部煤层</t>
+  </si>
+  <si>
     <t>【数据/方法】工业分析、CO₂ 吸附、高温高压甲烷吸附、等量吸附热和模型预测。
 【核心发现】灰分总体削弱微孔和吸附，固定碳/微孔与 Langmuir 体积正相关；升温降低吸附，升压提高吸附。
 【局限性】模型受煤阶和实验温压范围约束，吸附容量不等于可采气量。
 【与你课题的关系】温压背景、吸附/游离气和资料边界。</t>
+  </si>
+  <si>
+    <t>未指定具体区块（材料研发与室内实验）; 深部煤层气返排液；超耐盐滑溜水压裂液; 深部煤层气储层（TDS &gt;120,000 mg/L 高矿化度条件）</t>
   </si>
   <si>
     <t>【数据/方法】超高矿化度配伍、流变、减阻、携砂、破胶、残渣和分子模拟。
@@ -10033,18 +10043,30 @@
 【与你课题的关系】微孔吸附、中大孔渗流、裂缝—基质传质。</t>
   </si>
   <si>
+    <t>长庆矿区 10 口井、132 个压裂段；8 口完整井 105 段用于主分析，2 口井 27 段用于独立验; 长庆矿区10口深部煤层气水平井；132个压裂段; 长庆矿区深部煤层气储层</t>
+  </si>
+  <si>
     <t>【数据/方法】水相/气相示踪、Pearson、Random Forest 和段级生产贡献解释。
 【核心发现】外部研究识别 3 种段间产出形态；一类煤钻遇长度与初始产气的幂律 R²=0.71；保留测试集 R²=0.83；提出差异化压裂窗口。
 【创新点】把段级示踪、生产剖面和机器学习闭环结合。
 【局限性】外部分类和特征重要性不得变成用户项目正式类型或主控因素排序。</t>
   </si>
   <si>
+    <t>未指定具体区块（理论与工程思考）; 深部煤岩气储层；人工裂缝与天然割理系统; 深部煤岩气储层</t>
+  </si>
+  <si>
     <t>【创新点】从吸附气—游离气连续供气角度连接基质、割理和人工裂缝。
 【局限性】以理论和工程思考为主，不能替代用户项目压裂施工、示踪或导流能力资料。</t>
   </si>
   <si>
+    <t>综述（未限定具体区块）; 深部煤层气赋存机理（成因、演化、温压应力、吸附/游离气等）; 综述（涵盖不同深度范围）</t>
+  </si>
+  <si>
     <t>【创新点】尝试整合临界深度、裂缝渗流—基质扩散及生产模型。
 【局限性】综述不能替代项目证据；不得编造 DOI。</t>
+  </si>
+  <si>
+    <t>未指定具体区块（分子模拟研究）; 纳米狭缝孔中甲烷吸附态与游离态密度; 深部煤层纳米孔隙（模拟深部温压条件）</t>
   </si>
   <si>
     <t>【数据/方法】狭缝纳米孔模拟、Peng–Robinson 状态方程修正、限域逸度—压力、吸附相/游离相密度和煤阶修正。
@@ -10054,10 +10076,16 @@
 【与你课题的关系】早期游离气贡献和相态评价边界。</t>
   </si>
   <si>
+    <t>鄂尔多斯盆地东缘；石炭系本溪组; 深部煤层气储层（双重孔隙体系，埋深1500-2300 m）; 1500-2300 m；平均厚度约12 m</t>
+  </si>
+  <si>
     <t>【局限性】间接地球物理证据不能替代生产因果验证。</t>
   </si>
   <si>
     <t>间接地球物理证据不能替代生产因果验证。</t>
+  </si>
+  <si>
+    <t>华北4个煤层气区：沁水盆地南部、宁武盆地南部、鄂尔多斯盆地东缘神府区块、临兴区块; 煤层气藏（69口生产井；不同埋深/煤阶/水动力条件）</t>
   </si>
   <si>
     <t>【局限性】生产动态不能直接识别气源或微生物机制；</t>
@@ -10431,7 +10459,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" displayName="DeepCBMComplete105" headerRowCount="1" id="1" name="DeepCBMComplete105" ref="A1:AA135">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" displayName="DeepCBMComplete105" headerRowCount="1" id="1" name="DeepCBMComplete105" ref="A1:AA137">
   <tableColumns count="27">
     <tableColumn id="1" name="序号"/>
     <tableColumn id="2" name="文献ID"/>
@@ -21782,7 +21810,6 @@
       <c r="I136" t="s">
         <v>2767</v>
       </c>
-      <c r="J136" t="s"/>
       <c r="K136" t="s">
         <v>2768</v>
       </c>
@@ -21934,7 +21961,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F16"/>
+  <dimension ref="A1:F18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="13.8" outlineLevelCol="0"/>
   <cols>
     <col customWidth="1" max="6" min="1" width="22"/>
@@ -22173,7 +22200,7 @@
         <v>31</v>
       </c>
       <c r="B16" s="3" t="n">
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="C16" s="3" t="n"/>
       <c r="D16" s="3" t="s">
@@ -22184,6 +22211,15 @@
       </c>
       <c r="F16" s="3" t="n"/>
     </row>
+    <row r="17" spans="1:6">
+      <c r="A17" t="s">
+        <v>2742</v>
+      </c>
+      <c r="B17" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6"/>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
@@ -31224,12 +31260,18 @@
       <c r="J120" s="1" t="s">
         <v>2474</v>
       </c>
-      <c r="K120" s="1" t="n"/>
-      <c r="L120" s="1" t="n"/>
+      <c r="K120" s="1" t="s">
+        <v>2475</v>
+      </c>
+      <c r="L120" s="1" t="s">
+        <v>2476</v>
+      </c>
       <c r="M120" s="1" t="s">
         <v>145</v>
       </c>
-      <c r="N120" s="1" t="n"/>
+      <c r="N120" s="1" t="s">
+        <v>3098</v>
+      </c>
     </row>
     <row customHeight="1" ht="82.8" r="121" spans="1:14">
       <c r="A121" s="1" t="s">
@@ -31242,10 +31284,10 @@
         <v>2483</v>
       </c>
       <c r="D121" s="1" t="s">
-        <v>3098</v>
+        <v>3099</v>
       </c>
       <c r="E121" s="1" t="s">
-        <v>3099</v>
+        <v>3100</v>
       </c>
       <c r="F121" s="1" t="s">
         <v>2492</v>
@@ -31262,12 +31304,18 @@
       <c r="J121" s="1" t="s">
         <v>2496</v>
       </c>
-      <c r="K121" s="1" t="n"/>
-      <c r="L121" s="1" t="n"/>
+      <c r="K121" s="1" t="s">
+        <v>2497</v>
+      </c>
+      <c r="L121" s="1" t="s">
+        <v>2476</v>
+      </c>
       <c r="M121" s="1" t="s">
         <v>145</v>
       </c>
-      <c r="N121" s="1" t="n"/>
+      <c r="N121" s="1" t="s">
+        <v>3098</v>
+      </c>
     </row>
     <row customHeight="1" ht="82.8" r="122" spans="1:14">
       <c r="A122" s="1" t="s">
@@ -31280,10 +31328,10 @@
         <v>2503</v>
       </c>
       <c r="D122" s="1" t="s">
-        <v>3100</v>
+        <v>3101</v>
       </c>
       <c r="E122" s="1" t="s">
-        <v>3101</v>
+        <v>3102</v>
       </c>
       <c r="F122" s="1" t="s">
         <v>2508</v>
@@ -31300,12 +31348,18 @@
       <c r="J122" s="1" t="s">
         <v>2512</v>
       </c>
-      <c r="K122" s="1" t="n"/>
-      <c r="L122" s="1" t="n"/>
+      <c r="K122" s="1" t="s">
+        <v>2513</v>
+      </c>
+      <c r="L122" s="1" t="s">
+        <v>2514</v>
+      </c>
       <c r="M122" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="N122" s="1" t="n"/>
+      <c r="N122" s="1" t="s">
+        <v>3098</v>
+      </c>
     </row>
     <row r="123" spans="1:14">
       <c r="A123" t="s">
@@ -31318,10 +31372,10 @@
         <v>2521</v>
       </c>
       <c r="D123" t="s">
-        <v>3102</v>
+        <v>3103</v>
       </c>
       <c r="E123" t="s">
-        <v>3103</v>
+        <v>3104</v>
       </c>
       <c r="F123" t="s">
         <v>2528</v>
@@ -31348,7 +31402,7 @@
         <v>52</v>
       </c>
       <c r="N123" t="s">
-        <v>3104</v>
+        <v>3098</v>
       </c>
     </row>
     <row r="124" spans="1:14">
@@ -31392,7 +31446,7 @@
         <v>52</v>
       </c>
       <c r="N124" t="s">
-        <v>3104</v>
+        <v>3098</v>
       </c>
     </row>
     <row r="125" spans="1:14">
@@ -31436,7 +31490,7 @@
         <v>189</v>
       </c>
       <c r="N125" t="s">
-        <v>3104</v>
+        <v>3098</v>
       </c>
     </row>
     <row r="126" spans="1:14">
@@ -31455,6 +31509,9 @@
       <c r="E126" t="s">
         <v>3107</v>
       </c>
+      <c r="F126" t="s">
+        <v>2585</v>
+      </c>
       <c r="G126" t="s">
         <v>2586</v>
       </c>
@@ -31467,6 +31524,9 @@
       <c r="J126" t="s">
         <v>2589</v>
       </c>
+      <c r="K126" t="s">
+        <v>2590</v>
+      </c>
       <c r="L126" t="s">
         <v>2590</v>
       </c>
@@ -31474,7 +31534,7 @@
         <v>3108</v>
       </c>
       <c r="N126" t="s">
-        <v>3104</v>
+        <v>3098</v>
       </c>
     </row>
     <row r="127" spans="1:14">
@@ -31493,6 +31553,9 @@
       <c r="E127" t="s">
         <v>3109</v>
       </c>
+      <c r="F127" t="s">
+        <v>2603</v>
+      </c>
       <c r="G127" t="s">
         <v>2604</v>
       </c>
@@ -31505,6 +31568,9 @@
       <c r="J127" t="s">
         <v>2607</v>
       </c>
+      <c r="K127" t="s">
+        <v>2608</v>
+      </c>
       <c r="L127" t="s">
         <v>2608</v>
       </c>
@@ -31512,18 +31578,27 @@
         <v>52</v>
       </c>
       <c r="N127" t="s">
-        <v>3104</v>
+        <v>3098</v>
       </c>
     </row>
     <row r="128" spans="1:14">
       <c r="A128" t="s">
         <v>2610</v>
       </c>
+      <c r="B128" t="s">
+        <v>31</v>
+      </c>
       <c r="C128" t="s">
         <v>2614</v>
       </c>
+      <c r="D128" t="s">
+        <v>3110</v>
+      </c>
       <c r="E128" t="s">
-        <v>3110</v>
+        <v>3111</v>
+      </c>
+      <c r="F128" t="s">
+        <v>2620</v>
       </c>
       <c r="G128" t="s">
         <v>2621</v>
@@ -31540,22 +31615,34 @@
       <c r="K128" t="s">
         <v>2625</v>
       </c>
+      <c r="L128" t="s">
+        <v>2626</v>
+      </c>
       <c r="M128" t="s">
         <v>3108</v>
       </c>
       <c r="N128" t="s">
-        <v>3104</v>
+        <v>3098</v>
       </c>
     </row>
     <row r="129" spans="1:14">
       <c r="A129" t="s">
         <v>2628</v>
       </c>
+      <c r="B129" t="s">
+        <v>31</v>
+      </c>
       <c r="C129" t="s">
         <v>2632</v>
       </c>
+      <c r="D129" t="s">
+        <v>3112</v>
+      </c>
       <c r="E129" t="s">
-        <v>3111</v>
+        <v>3113</v>
+      </c>
+      <c r="F129" t="s">
+        <v>2638</v>
       </c>
       <c r="G129" t="s">
         <v>2639</v>
@@ -31563,28 +31650,43 @@
       <c r="H129" t="s">
         <v>2640</v>
       </c>
+      <c r="I129" t="s">
+        <v>2641</v>
+      </c>
       <c r="J129" t="s">
         <v>2642</v>
       </c>
       <c r="K129" t="s">
         <v>2643</v>
       </c>
+      <c r="L129" t="s">
+        <v>2644</v>
+      </c>
       <c r="M129" t="s">
         <v>52</v>
       </c>
       <c r="N129" t="s">
-        <v>3104</v>
+        <v>3098</v>
       </c>
     </row>
     <row r="130" spans="1:14">
       <c r="A130" t="s">
         <v>2646</v>
       </c>
+      <c r="B130" t="s">
+        <v>31</v>
+      </c>
       <c r="C130" t="s">
         <v>2650</v>
       </c>
+      <c r="D130" t="s">
+        <v>3114</v>
+      </c>
       <c r="E130" t="s">
-        <v>3112</v>
+        <v>3115</v>
+      </c>
+      <c r="F130" t="s">
+        <v>2657</v>
       </c>
       <c r="G130" t="s">
         <v>2658</v>
@@ -31601,17 +31703,23 @@
       <c r="K130" t="s">
         <v>2662</v>
       </c>
+      <c r="L130" t="s">
+        <v>2663</v>
+      </c>
       <c r="M130" t="s">
         <v>52</v>
       </c>
       <c r="N130" t="s">
-        <v>3104</v>
+        <v>3098</v>
       </c>
     </row>
     <row r="131" spans="1:14">
       <c r="A131" t="s">
         <v>2665</v>
       </c>
+      <c r="B131" t="s">
+        <v>31</v>
+      </c>
       <c r="C131" t="s">
         <v>2669</v>
       </c>
@@ -31619,7 +31727,10 @@
         <v>2673</v>
       </c>
       <c r="E131" t="s">
-        <v>3113</v>
+        <v>3116</v>
+      </c>
+      <c r="F131" t="s">
+        <v>2675</v>
       </c>
       <c r="G131" t="s">
         <v>2676</v>
@@ -31627,28 +31738,43 @@
       <c r="H131" t="s">
         <v>2677</v>
       </c>
+      <c r="I131" t="s">
+        <v>2678</v>
+      </c>
       <c r="J131" t="s">
         <v>2679</v>
       </c>
       <c r="K131" t="s">
         <v>2680</v>
       </c>
+      <c r="L131" t="s">
+        <v>2681</v>
+      </c>
       <c r="M131" t="s">
         <v>52</v>
       </c>
       <c r="N131" t="s">
-        <v>3104</v>
+        <v>3098</v>
       </c>
     </row>
     <row r="132" spans="1:14">
       <c r="A132" t="s">
         <v>2683</v>
       </c>
+      <c r="B132" t="s">
+        <v>31</v>
+      </c>
       <c r="C132" t="s">
         <v>2687</v>
       </c>
+      <c r="D132" t="s">
+        <v>3117</v>
+      </c>
       <c r="E132" t="s">
-        <v>3114</v>
+        <v>3118</v>
+      </c>
+      <c r="F132" t="s">
+        <v>2694</v>
       </c>
       <c r="G132" t="s">
         <v>2695</v>
@@ -31662,6 +31788,9 @@
       <c r="J132" t="s">
         <v>2698</v>
       </c>
+      <c r="K132" t="s">
+        <v>2699</v>
+      </c>
       <c r="L132" t="s">
         <v>2699</v>
       </c>
@@ -31669,7 +31798,7 @@
         <v>52</v>
       </c>
       <c r="N132" t="s">
-        <v>3104</v>
+        <v>3098</v>
       </c>
     </row>
     <row r="133" spans="1:14">
@@ -31682,8 +31811,20 @@
       <c r="C133" t="s">
         <v>2705</v>
       </c>
+      <c r="D133" t="s">
+        <v>3119</v>
+      </c>
       <c r="E133" t="s">
-        <v>3115</v>
+        <v>3120</v>
+      </c>
+      <c r="F133" t="s">
+        <v>2711</v>
+      </c>
+      <c r="G133" t="s">
+        <v>2712</v>
+      </c>
+      <c r="H133" t="s">
+        <v>2713</v>
       </c>
       <c r="I133" t="s">
         <v>2714</v>
@@ -31691,6 +31832,9 @@
       <c r="J133" t="s">
         <v>2715</v>
       </c>
+      <c r="K133" t="s">
+        <v>2716</v>
+      </c>
       <c r="L133" t="s">
         <v>2716</v>
       </c>
@@ -31698,18 +31842,33 @@
         <v>52</v>
       </c>
       <c r="N133" t="s">
-        <v>3104</v>
+        <v>3098</v>
       </c>
     </row>
     <row r="134" spans="1:14">
       <c r="A134" t="s">
         <v>2718</v>
       </c>
+      <c r="B134" t="s">
+        <v>31</v>
+      </c>
       <c r="C134" t="s">
         <v>2722</v>
       </c>
+      <c r="D134" t="s">
+        <v>3121</v>
+      </c>
       <c r="E134" t="s">
-        <v>3116</v>
+        <v>3122</v>
+      </c>
+      <c r="F134" t="s">
+        <v>2730</v>
+      </c>
+      <c r="G134" t="s">
+        <v>2731</v>
+      </c>
+      <c r="H134" t="s">
+        <v>2732</v>
       </c>
       <c r="I134" t="s">
         <v>2733</v>
@@ -31717,22 +31876,37 @@
       <c r="J134" t="s">
         <v>2734</v>
       </c>
+      <c r="K134" t="s">
+        <v>2735</v>
+      </c>
+      <c r="L134" t="s">
+        <v>2736</v>
+      </c>
       <c r="M134" t="s">
         <v>52</v>
       </c>
       <c r="N134" t="s">
-        <v>3104</v>
+        <v>3098</v>
       </c>
     </row>
     <row r="135" spans="1:14">
       <c r="A135" t="s">
         <v>2739</v>
       </c>
+      <c r="B135" t="s">
+        <v>2742</v>
+      </c>
       <c r="C135" t="s">
         <v>2744</v>
       </c>
+      <c r="D135" t="s">
+        <v>3123</v>
+      </c>
       <c r="E135" t="s">
-        <v>3117</v>
+        <v>3124</v>
+      </c>
+      <c r="F135" t="s">
+        <v>2753</v>
       </c>
       <c r="G135" t="s">
         <v>2754</v>
@@ -31749,51 +31923,102 @@
       <c r="K135" t="s">
         <v>2758</v>
       </c>
+      <c r="L135" t="s">
+        <v>2759</v>
+      </c>
       <c r="M135" t="s">
         <v>52</v>
       </c>
       <c r="N135" t="s">
-        <v>3104</v>
+        <v>3098</v>
       </c>
     </row>
     <row r="136" spans="1:14">
       <c r="A136" t="s">
         <v>2761</v>
       </c>
+      <c r="B136" t="s">
+        <v>31</v>
+      </c>
       <c r="C136" t="s">
         <v>2765</v>
       </c>
+      <c r="D136" t="s">
+        <v>3125</v>
+      </c>
       <c r="E136" t="s">
-        <v>3118</v>
+        <v>3126</v>
+      </c>
+      <c r="F136" t="s">
+        <v>2774</v>
+      </c>
+      <c r="G136" t="s">
+        <v>2775</v>
+      </c>
+      <c r="H136" t="s">
+        <v>2776</v>
+      </c>
+      <c r="I136" t="s">
+        <v>2777</v>
       </c>
       <c r="J136" t="s">
-        <v>3119</v>
+        <v>3127</v>
+      </c>
+      <c r="K136" t="s">
+        <v>2779</v>
+      </c>
+      <c r="L136" t="s">
+        <v>2780</v>
       </c>
       <c r="M136" t="s">
         <v>52</v>
       </c>
       <c r="N136" t="s">
-        <v>3104</v>
+        <v>3098</v>
       </c>
     </row>
     <row r="137" spans="1:14">
       <c r="A137" t="s">
         <v>2783</v>
       </c>
+      <c r="B137" t="s">
+        <v>2786</v>
+      </c>
       <c r="C137" t="s">
         <v>2788</v>
       </c>
+      <c r="D137" t="s">
+        <v>3128</v>
+      </c>
       <c r="E137" t="s">
-        <v>3120</v>
+        <v>3129</v>
+      </c>
+      <c r="F137" t="s">
+        <v>2795</v>
+      </c>
+      <c r="G137" t="s">
+        <v>2796</v>
+      </c>
+      <c r="H137" t="s">
+        <v>2797</v>
+      </c>
+      <c r="I137" t="s">
+        <v>2798</v>
       </c>
       <c r="J137" t="s">
-        <v>3121</v>
+        <v>3130</v>
+      </c>
+      <c r="K137" t="s">
+        <v>2800</v>
+      </c>
+      <c r="L137" t="s">
+        <v>2801</v>
       </c>
       <c r="M137" t="s">
         <v>52</v>
       </c>
       <c r="N137" t="s">
-        <v>3104</v>
+        <v>3098</v>
       </c>
     </row>
   </sheetData>
@@ -31810,20 +32035,21 @@
   <dimension ref="A1:B14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="13.8" outlineLevelCol="0"/>
   <cols>
-    <col customWidth="1" max="2" min="1" width="50"/>
+    <col customWidth="1" max="1" min="1" width="50"/>
+    <col customWidth="1" max="2" min="2" width="49.09765625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="7" t="s">
-        <v>3122</v>
+        <v>3131</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>3123</v>
+        <v>3132</v>
       </c>
     </row>
     <row r="2" spans="1:2">
       <c r="A2" t="s">
-        <v>3124</v>
+        <v>3133</v>
       </c>
       <c r="B2" t="s">
         <v>2813</v>
@@ -31831,98 +32057,98 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" t="s">
-        <v>3125</v>
+        <v>3134</v>
       </c>
       <c r="B3" t="s">
-        <v>3126</v>
+        <v>3135</v>
       </c>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" t="s">
-        <v>3127</v>
+        <v>3136</v>
       </c>
       <c r="B4" t="s">
-        <v>3128</v>
+        <v>3137</v>
       </c>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" t="s">
-        <v>3129</v>
+        <v>3138</v>
       </c>
       <c r="B5" t="s">
-        <v>3130</v>
+        <v>3139</v>
       </c>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" t="s">
-        <v>3131</v>
+        <v>3140</v>
       </c>
       <c r="B6" t="s">
-        <v>3132</v>
+        <v>3141</v>
       </c>
     </row>
     <row r="7" spans="1:2">
       <c r="A7" t="s">
-        <v>3133</v>
+        <v>3142</v>
       </c>
       <c r="B7" t="s">
-        <v>3134</v>
+        <v>3143</v>
       </c>
     </row>
     <row r="8" spans="1:2">
       <c r="A8" t="s">
-        <v>3135</v>
+        <v>3144</v>
       </c>
       <c r="B8" t="s">
-        <v>3136</v>
+        <v>3145</v>
       </c>
     </row>
     <row r="9" spans="1:2">
       <c r="A9" t="s">
-        <v>3137</v>
+        <v>3146</v>
       </c>
       <c r="B9" t="s">
-        <v>3138</v>
+        <v>3147</v>
       </c>
     </row>
     <row r="10" spans="1:2">
       <c r="A10" t="s">
-        <v>3139</v>
+        <v>3148</v>
       </c>
       <c r="B10" t="s">
-        <v>3140</v>
+        <v>3149</v>
       </c>
     </row>
     <row r="11" spans="1:2">
       <c r="A11" t="s">
-        <v>3141</v>
+        <v>3150</v>
       </c>
       <c r="B11" t="s">
-        <v>3142</v>
+        <v>3151</v>
       </c>
     </row>
     <row r="12" spans="1:2">
       <c r="A12" t="s">
-        <v>3143</v>
+        <v>3152</v>
       </c>
       <c r="B12" t="s">
-        <v>3144</v>
+        <v>3153</v>
       </c>
     </row>
     <row r="13" spans="1:2">
       <c r="A13" t="s">
-        <v>3145</v>
+        <v>3154</v>
       </c>
       <c r="B13" t="s">
-        <v>3146</v>
+        <v>3155</v>
       </c>
     </row>
     <row r="14" spans="1:2">
       <c r="A14" t="s">
-        <v>3147</v>
+        <v>3156</v>
       </c>
       <c r="B14" t="s">
-        <v>3148</v>
+        <v>3157</v>
       </c>
     </row>
   </sheetData>
@@ -31941,82 +32167,82 @@
   <sheetData>
     <row customHeight="1" ht="27.6" r="1" spans="1:6">
       <c r="A1" s="6" t="s">
-        <v>3149</v>
+        <v>3158</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>3150</v>
+        <v>3159</v>
       </c>
       <c r="C1" s="6" t="s">
-        <v>3151</v>
+        <v>3160</v>
       </c>
       <c r="D1" s="6" t="s">
-        <v>3152</v>
+        <v>3161</v>
       </c>
       <c r="E1" s="6" t="s">
-        <v>3153</v>
+        <v>3162</v>
       </c>
       <c r="F1" s="6" t="s">
-        <v>3154</v>
+        <v>3163</v>
       </c>
     </row>
     <row customHeight="1" ht="55.2" r="2" spans="1:6">
       <c r="A2" s="1" t="s">
-        <v>3155</v>
+        <v>3164</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>38</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>3156</v>
+        <v>3165</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>3157</v>
+        <v>3166</v>
       </c>
       <c r="E2" s="1" t="s">
         <v>28</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>3158</v>
+        <v>3167</v>
       </c>
     </row>
     <row customHeight="1" ht="55.2" r="3" spans="1:6">
       <c r="A3" s="1" t="s">
-        <v>3159</v>
+        <v>3168</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>1681</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>3156</v>
+        <v>3165</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>3157</v>
+        <v>3166</v>
       </c>
       <c r="E3" s="1" t="s">
         <v>1674</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>3158</v>
+        <v>3167</v>
       </c>
     </row>
     <row customHeight="1" ht="55.2" r="4" spans="1:6">
       <c r="A4" s="1" t="s">
-        <v>3160</v>
+        <v>3169</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>1167</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>3156</v>
+        <v>3165</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>3157</v>
+        <v>3166</v>
       </c>
       <c r="E4" s="1" t="s">
         <v>1161</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>3158</v>
+        <v>3167</v>
       </c>
     </row>
     <row customHeight="1" ht="82.8" r="5" spans="1:6">
@@ -32027,16 +32253,16 @@
         <v>2204</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>3161</v>
+        <v>3170</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>3162</v>
+        <v>3171</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>3163</v>
+        <v>3172</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>3164</v>
+        <v>3173</v>
       </c>
     </row>
     <row customHeight="1" ht="82.8" r="6" spans="1:6">
@@ -32047,16 +32273,16 @@
         <v>2223</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>3161</v>
+        <v>3170</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>3162</v>
+        <v>3171</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>3163</v>
+        <v>3172</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>3164</v>
+        <v>3173</v>
       </c>
     </row>
     <row customHeight="1" ht="82.8" r="7" spans="1:6">
@@ -32067,16 +32293,16 @@
         <v>2243</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>3161</v>
+        <v>3170</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>3162</v>
+        <v>3171</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>3163</v>
+        <v>3172</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>3164</v>
+        <v>3173</v>
       </c>
     </row>
     <row customHeight="1" ht="82.8" r="8" spans="1:6">
@@ -32087,16 +32313,16 @@
         <v>2262</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>3161</v>
+        <v>3170</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>3162</v>
+        <v>3171</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>3163</v>
+        <v>3172</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>3164</v>
+        <v>3173</v>
       </c>
     </row>
     <row customHeight="1" ht="82.8" r="9" spans="1:6">
@@ -32107,16 +32333,16 @@
         <v>2283</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>3161</v>
+        <v>3170</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>3162</v>
+        <v>3171</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>3163</v>
+        <v>3172</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>3164</v>
+        <v>3173</v>
       </c>
     </row>
     <row customHeight="1" ht="82.8" r="10" spans="1:6">
@@ -32127,16 +32353,16 @@
         <v>2305</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>3161</v>
+        <v>3170</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>3162</v>
+        <v>3171</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>3163</v>
+        <v>3172</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>3164</v>
+        <v>3173</v>
       </c>
     </row>
     <row customHeight="1" ht="82.8" r="11" spans="1:6">
@@ -32147,16 +32373,16 @@
         <v>2326</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>3161</v>
+        <v>3170</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>3162</v>
+        <v>3171</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>3163</v>
+        <v>3172</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>3164</v>
+        <v>3173</v>
       </c>
     </row>
     <row customHeight="1" ht="82.8" r="12" spans="1:6">
@@ -32167,16 +32393,16 @@
         <v>2346</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>3161</v>
+        <v>3170</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>3162</v>
+        <v>3171</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>3163</v>
+        <v>3172</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>3164</v>
+        <v>3173</v>
       </c>
     </row>
     <row customHeight="1" ht="82.8" r="13" spans="1:6">
@@ -32187,16 +32413,16 @@
         <v>2364</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>3161</v>
+        <v>3170</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>3162</v>
+        <v>3171</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>3163</v>
+        <v>3172</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>3164</v>
+        <v>3173</v>
       </c>
     </row>
     <row customHeight="1" ht="82.8" r="14" spans="1:6">
@@ -32207,16 +32433,16 @@
         <v>2383</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>3161</v>
+        <v>3170</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>3162</v>
+        <v>3171</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>3163</v>
+        <v>3172</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>3164</v>
+        <v>3173</v>
       </c>
     </row>
     <row customHeight="1" ht="82.8" r="15" spans="1:6">
@@ -32227,16 +32453,16 @@
         <v>2404</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>3161</v>
+        <v>3170</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>3162</v>
+        <v>3171</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>3163</v>
+        <v>3172</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>3164</v>
+        <v>3173</v>
       </c>
     </row>
     <row customHeight="1" ht="82.8" r="16" spans="1:6">
@@ -32247,16 +32473,16 @@
         <v>2425</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>3161</v>
+        <v>3170</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>3162</v>
+        <v>3171</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>3163</v>
+        <v>3172</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>3164</v>
+        <v>3173</v>
       </c>
     </row>
     <row customHeight="1" ht="82.8" r="17" spans="1:6">
@@ -32267,96 +32493,96 @@
         <v>2445</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>3161</v>
+        <v>3170</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>3162</v>
+        <v>3171</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>3163</v>
+        <v>3172</v>
       </c>
       <c r="F17" s="1" t="s">
-        <v>3164</v>
+        <v>3173</v>
       </c>
     </row>
     <row customHeight="1" ht="303.6" r="18" spans="1:6">
       <c r="A18" s="1" t="s">
+        <v>3174</v>
+      </c>
+      <c r="B18" s="1" t="s">
+        <v>3175</v>
+      </c>
+      <c r="C18" s="1" t="s">
         <v>3165</v>
       </c>
-      <c r="B18" s="1" t="s">
-        <v>3166</v>
-      </c>
-      <c r="C18" s="1" t="s">
-        <v>3156</v>
-      </c>
       <c r="D18" s="1" t="s">
-        <v>3167</v>
+        <v>3176</v>
       </c>
       <c r="E18" s="1" t="s">
         <v>610</v>
       </c>
       <c r="F18" s="1" t="s">
-        <v>3168</v>
+        <v>3177</v>
       </c>
     </row>
     <row customHeight="1" ht="276" r="19" spans="1:6">
       <c r="A19" s="1" t="s">
-        <v>3169</v>
+        <v>3178</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>3170</v>
+        <v>3179</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>3171</v>
+        <v>3180</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>3172</v>
+        <v>3181</v>
       </c>
       <c r="E19" s="1" t="s">
         <v>2458</v>
       </c>
       <c r="F19" s="1" t="s">
-        <v>3161</v>
+        <v>3170</v>
       </c>
     </row>
     <row customHeight="1" ht="193.2" r="20" spans="1:6">
       <c r="A20" s="1" t="s">
-        <v>3173</v>
+        <v>3182</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>3174</v>
+        <v>3183</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>3171</v>
+        <v>3180</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>3172</v>
+        <v>3181</v>
       </c>
       <c r="E20" s="1" t="s">
         <v>2479</v>
       </c>
       <c r="F20" s="1" t="s">
-        <v>3161</v>
+        <v>3170</v>
       </c>
     </row>
     <row customHeight="1" ht="276" r="21" spans="1:6">
       <c r="A21" s="1" t="s">
-        <v>3175</v>
+        <v>3184</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>3176</v>
+        <v>3185</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>3171</v>
+        <v>3180</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>3172</v>
+        <v>3181</v>
       </c>
       <c r="E21" s="1" t="s">
         <v>2500</v>
       </c>
       <c r="F21" s="1" t="s">
-        <v>3161</v>
+        <v>3170</v>
       </c>
     </row>
   </sheetData>
@@ -32378,15 +32604,15 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="8" t="s">
-        <v>3177</v>
+        <v>3186</v>
       </c>
       <c r="B1" s="8" t="s">
-        <v>3178</v>
+        <v>3187</v>
       </c>
     </row>
     <row r="2" spans="1:2">
       <c r="A2" t="s">
-        <v>3179</v>
+        <v>3188</v>
       </c>
       <c r="B2" t="n">
         <v>118</v>
@@ -32394,7 +32620,7 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" t="s">
-        <v>3180</v>
+        <v>3189</v>
       </c>
       <c r="B3" t="n">
         <v>1</v>
@@ -32402,7 +32628,7 @@
     </row>
     <row r="4" spans="1:2">
       <c r="A4" t="s">
-        <v>3181</v>
+        <v>3190</v>
       </c>
       <c r="B4" t="n">
         <v>0</v>
@@ -32410,7 +32636,7 @@
     </row>
     <row r="5" spans="1:2">
       <c r="A5" t="s">
-        <v>3182</v>
+        <v>3191</v>
       </c>
       <c r="B5" t="s">
         <v>2440</v>
@@ -32418,74 +32644,74 @@
     </row>
     <row r="6" spans="1:2">
       <c r="A6" t="s">
-        <v>3183</v>
+        <v>3192</v>
       </c>
       <c r="B6" t="s">
-        <v>3184</v>
+        <v>3193</v>
       </c>
     </row>
     <row r="7" spans="1:2">
       <c r="A7" t="s">
-        <v>3185</v>
+        <v>3194</v>
       </c>
       <c r="B7" t="s">
-        <v>3186</v>
+        <v>3195</v>
       </c>
     </row>
     <row r="8" spans="1:2">
       <c r="A8" t="s">
-        <v>3187</v>
+        <v>3196</v>
       </c>
       <c r="B8" t="s">
-        <v>3188</v>
+        <v>3197</v>
       </c>
     </row>
     <row r="9" spans="1:2">
       <c r="A9" t="s">
-        <v>3189</v>
+        <v>3198</v>
       </c>
       <c r="B9" t="s">
-        <v>3190</v>
+        <v>3199</v>
       </c>
     </row>
     <row r="10" spans="1:2">
       <c r="A10" t="s">
-        <v>3139</v>
+        <v>3148</v>
       </c>
       <c r="B10" t="s">
-        <v>3140</v>
+        <v>3149</v>
       </c>
     </row>
     <row r="11" spans="1:2">
       <c r="A11" t="s">
-        <v>3191</v>
+        <v>3200</v>
       </c>
       <c r="B11" t="s">
-        <v>3186</v>
+        <v>3195</v>
       </c>
     </row>
     <row r="12" spans="1:2">
       <c r="A12" t="s">
-        <v>3192</v>
+        <v>3201</v>
       </c>
       <c r="B12" t="s">
-        <v>3193</v>
+        <v>3202</v>
       </c>
     </row>
     <row r="13" spans="1:2">
       <c r="A13" t="s">
-        <v>3194</v>
+        <v>3203</v>
       </c>
       <c r="B13" t="s">
-        <v>3195</v>
+        <v>3204</v>
       </c>
     </row>
     <row r="14" spans="1:2">
       <c r="A14" t="s">
-        <v>3196</v>
+        <v>3205</v>
       </c>
       <c r="B14" t="s">
-        <v>3197</v>
+        <v>3206</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
update: process Deep CBM daily brief 2026-07-26
- Added 3 new records: DCBM-137, DCBM-138, DCBM-139
- DCBM-137: Tao Wang — Gas content prediction (Results in Engineering)
- DCBM-138: Chen Guo — T-P adsorption behavior (Scientific Reports)
- DCBM-139: Yusong Ji — Logging-driven CBM content (Geological Journal)
- 0 duplicates; master: 136 -> 139, ID continuous
- Protected dirs unmodified
</commit_message>
<xml_diff>
--- a/00_Master/Deep_CBM_Latest.xlsx
+++ b/00_Master/Deep_CBM_Latest.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="3207">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="3281">
   <si>
     <t>序号</t>
   </si>
@@ -8455,6 +8455,189 @@
     <t>出版商题名/DOI/卷期/摘要和研究设计已核验；作者缩写待Crossref补全</t>
   </si>
   <si>
+    <t>DCBM-137</t>
+  </si>
+  <si>
+    <t>Wang, Tao</t>
+  </si>
+  <si>
+    <t>Wang, Tao; Huang, Daojun; Ding, Rong; Cao, Yimin; Zhou, Ke; Zhou, Guoxiao; Shi, Yunhe; Wang, Huaichang; Hu, Jianling; Jiao, Pengfei; Feng, Zongqi; Deng, Ze</t>
+  </si>
+  <si>
+    <t>Evaluation of gas content prediction models for deep coal seams: A case study from the Daning-Jixian Block, Eastern Ordos Basin</t>
+  </si>
+  <si>
+    <t>深部煤层含气量预测模型评价：以鄂尔多斯盆地东缘大宁-吉县区块为例</t>
+  </si>
+  <si>
+    <t>110079</t>
+  </si>
+  <si>
+    <t>10.1016/j.rineng.2026.110079</t>
+  </si>
+  <si>
+    <t>https://www.sciencedirect.com/science/article/pii/S2590123026011163</t>
+  </si>
+  <si>
+    <t>鄂尔多斯盆地东缘大宁-吉县区块</t>
+  </si>
+  <si>
+    <t>深部煤层（吸附气/游离气/总含气量）</t>
+  </si>
+  <si>
+    <t>深部煤层（大宁-吉县区块深部储层）</t>
+  </si>
+  <si>
+    <t>评价并对比多种含气量预测模型在大宁-吉县区块深部煤层中的适用性</t>
+  </si>
+  <si>
+    <t>4口井煤心解吸/等温吸附/Langmuir模型；BP神经网络/随机森林/XGBoost/CNN-LSTM-Attention；k-fold交叉验证(5折/10折)；深度校正</t>
+  </si>
+  <si>
+    <t>CNN-LSTM-Attention表现最优(RMSE 0.82 m3/t, R2 0.93, MAE 0.61 m3/t)；XGBoost次之(RMSE 0.99 m3/t, R2 0.90)；传统Langmuir模型表现最差(R2 0.71)；游离气占比预测对含气量总量预测至关重要；Attention机制可自动加权关键测井曲线</t>
+  </si>
+  <si>
+    <t>系统对比传统模型到深度学习模型的含气量预测；将游离气/吸附气分开预测再汇总；引入Attention机制自动加权测井曲线</t>
+  </si>
+  <si>
+    <t>4口井样本量有限；CNN-LSTM-Attention可解释性低于传统模型；结果具有区块和煤阶特异性</t>
+  </si>
+  <si>
+    <t>含气量预测/地质建模/游离气-吸附气分配/深度学习适用性与边界</t>
+  </si>
+  <si>
+    <t>地质建模与含气量；研究局限与方法边界；后续可引入的机器学习补充资料</t>
+  </si>
+  <si>
+    <t>gas content prediction; deep learning; CNN-LSTM-Attention; XGBoost; Daning-Jixian; Langmuir</t>
+  </si>
+  <si>
+    <t>出版商题名/DOI/卷和文章号/摘要已核验</t>
+  </si>
+  <si>
+    <t>DCBM-138</t>
+  </si>
+  <si>
+    <t>Guo, Chen</t>
+  </si>
+  <si>
+    <t>Guo, Chen; Jiang, Lingling; Lu, Lingling; Gao, Junzhe; Cheng, Xi</t>
+  </si>
+  <si>
+    <t>Adsorption behavior and prediction model of coalbed methane under the influence of temperature and pressure: a case study of the Zhijin Block, Western Guizhou, South China</t>
+  </si>
+  <si>
+    <t>温压影响下煤层气吸附行为与预测模型：以黔西织金区块为例</t>
+  </si>
+  <si>
+    <t>21736</t>
+  </si>
+  <si>
+    <t>10.1038/s41598-026-52704-3</t>
+  </si>
+  <si>
+    <t>https://www.nature.com/articles/s41598-026-52704-3</t>
+  </si>
+  <si>
+    <t>黔西织金区块上二叠统龙潭组（4个向斜6个煤矿）</t>
+  </si>
+  <si>
+    <t>煤层气吸附行为（6件煤样）</t>
+  </si>
+  <si>
+    <t>温度-压力-埋深耦合（织金区块深部条件）</t>
+  </si>
+  <si>
+    <t>研究温压耦合条件下煤层气吸附行为变化规律，建立温度-压力-埋深耦合预测模型</t>
+  </si>
+  <si>
+    <t>6件煤样工业分析和镜质组反射率；高压等温吸附(N2/CO2)；4种吸附模型对比(Langmuir/DR/DA/L-F)；温度-压力-埋深耦合预测</t>
+  </si>
+  <si>
+    <t>吸附气含量随埋深先增后降；最大吸附量对应埋深受温度梯度和煤阶共同控制；超临界条件下过剩吸附量需进行密度校正；L-F模型在超临界条件下拟合效果最佳</t>
+  </si>
+  <si>
+    <t>明确吸附气含量先增后降的临界深度窗口；整合温度-压力-埋深三维耦合预测；系统对比4种吸附模型在超临界条件下的适用性</t>
+  </si>
+  <si>
+    <t>6件煤样覆盖范围有限；织金区块结果不可直接外推至其他盆地；未与生产动态数据交叉验证</t>
+  </si>
+  <si>
+    <t>吸附/游离气比例/临界深度/超临界吸附校正/区域差异</t>
+  </si>
+  <si>
+    <t>赋存机理与吸附行为；温压-深度耦合；区域差异与模型选择；局限</t>
+  </si>
+  <si>
+    <t>adsorption; temperature-pressure coupling; supercritical; Langmuir; Zhijin block; coal rank</t>
+  </si>
+  <si>
+    <t>Nature官方页和全文已核验</t>
+  </si>
+  <si>
+    <t>DCBM-139</t>
+  </si>
+  <si>
+    <t>Ji, Yusong</t>
+  </si>
+  <si>
+    <t>Ji, Yusong; Li, Song; Hou, Wei; Li, Yongzhou; Feng, Peng; Yang, Shizhuang; Zhou, Hanmiao</t>
+  </si>
+  <si>
+    <t>Quantitative Evaluation of Deep Coalbed Methane Content: A Logging Data-Driven Approach</t>
+  </si>
+  <si>
+    <t>测井数据驱动的深部煤层气含量定量评价</t>
+  </si>
+  <si>
+    <t>Geological Journal</t>
+  </si>
+  <si>
+    <t>2072-2086</t>
+  </si>
+  <si>
+    <t>10.1002/gj.70077</t>
+  </si>
+  <si>
+    <t>https://onlinelibrary.wiley.com/doi/10.1002/gj.70077</t>
+  </si>
+  <si>
+    <t>大宁-吉县区块本溪组8号煤</t>
+  </si>
+  <si>
+    <t>深部煤层气含量（10口井）</t>
+  </si>
+  <si>
+    <t>大宁-吉县区块深部段(&gt;1500 m)</t>
+  </si>
+  <si>
+    <t>构建测井数据驱动的深部煤层气含量多模型定量评价方法</t>
+  </si>
+  <si>
+    <t>10口井常规测井(GR/DEN/CNL/RD/RS/AC)；煤心解吸含气量标定；多元线性回归/RBF神经网络/随机森林/CNN；数据增广(CTGAN)</t>
+  </si>
+  <si>
+    <t>CNN预测精度最高(+20%~35%)；CTGAN数据增广后小样本模型性能显著提升；深部段(&gt;1500 m)含气量变化更复杂需要更深的网络结构</t>
+  </si>
+  <si>
+    <t>系统对比4种模型(MLR到CNN)在同一区块的性能；引入CTGAN数据增广解决小样本深度学习问题；为测井含气量评价提供可迁移框架</t>
+  </si>
+  <si>
+    <t>10口井样本仍属小样本；深部&gt;1500 m段模型不确定性升高；结果具有区块和煤阶依赖性</t>
+  </si>
+  <si>
+    <t>含气量评价/测井-地质-工程一体化/深度学习适用性/小样本增广策略</t>
+  </si>
+  <si>
+    <t>地质建模与含气量；方法讨论：多源数据与模型选择；局限；后续可引入的机器学习补充方向</t>
+  </si>
+  <si>
+    <t>logging data; deep learning; CNN; CTGAN data augmentation; gas content; Daning-Jixian</t>
+  </si>
+  <si>
+    <t>Wiley官方题名/作者/DOI/卷期/摘要已核验；页码待最终确认</t>
+  </si>
+  <si>
     <t>指标</t>
   </si>
   <si>
@@ -8479,7 +8662,7 @@
     <t>当前主表版本</t>
   </si>
   <si>
-    <t>v1_136_daily_brief_update_2026-07-24</t>
+    <t>v1_139_daily_brief_update_2026-07-26</t>
   </si>
   <si>
     <t>Deep_CBM_complete_literature_matrix_v1_105.xlsx</t>
@@ -10094,6 +10277,46 @@
     <t>生产动态不能直接识别气源或微生物机制；</t>
   </si>
   <si>
+    <t>深部煤层含气量预测模型评价：以鄂尔多斯盆地东缘大宁—吉县区块为例</t>
+  </si>
+  <si>
+    <t>鄂尔多斯盆地东缘大宁-吉县区块; 深部煤层（吸附气/游离气/总含气量）; 深部煤层（大宁-吉县区块深部储层）</t>
+  </si>
+  <si>
+    <t>【局限性】动态曲线与储层测试之间的边界；</t>
+  </si>
+  <si>
+    <t>动态曲线与储层测试之间的边界；</t>
+  </si>
+  <si>
+    <t>黔西织金区块上二叠统龙潭组（4个向斜6个煤矿）; 煤层气吸附行为（6件煤样）; 温度-压力-埋深耦合（织金区块深部条件）</t>
+  </si>
+  <si>
+    <t>【研究目的】研究温压耦合条件下煤层气吸附行为变化规律，建立温度-压力-埋深耦合预测模型
+【数据/方法】6件煤样工业分析和镜质组反射率；高压等温吸附(N2/CO2)；4种吸附模型对比(Langmuir/DR/DA/L-F)；温度-压力-埋深耦合预测
+【核心发现】吸附气含量随埋深先增后降；最大吸附量对应埋深受温度梯度和煤阶共同控制；超临界条件下过剩吸附量需进行密度校正；L-F模型在超临界条件下拟合效果最佳
+【创新点】明确吸附气含量先增后降的临界深度窗口；整合温度-压力-埋深三维耦合预测；系统对比4种吸附模型在超临界条件下的适用性
+【局限性】6件煤样覆盖范围有限；织金区块结果不可直接外推至其他盆地；未与生产动态数据交叉验证
+【与你课题的关系】吸附/游离气比例/临界深度/超临界吸附校正/区域差异</t>
+  </si>
+  <si>
+    <t>临界深度和深部定义的区域性。</t>
+  </si>
+  <si>
+    <t>大宁-吉县区块本溪组8号煤; 深部煤层气含量（10口井）; 大宁-吉县区块深部段(&gt;1500 m)</t>
+  </si>
+  <si>
+    <t>【研究目的】构建测井数据驱动的深部煤层气含量多模型定量评价方法
+【数据/方法】10口井常规测井(GR/DEN/CNL/RD/RS/AC)；煤心解吸含气量标定；多元线性回归/RBF神经网络/随机森林/CNN；数据增广(CTGAN)
+【核心发现】CNN预测精度最高(+20%~35%)；CTGAN数据增广后小样本模型性能显著提升；深部段(&gt;1500 m)含气量变化更复杂需要更深的网络结构
+【创新点】系统对比4种模型(MLR到CNN)在同一区块的性能；引入CTGAN数据增广解决小样本深度学习问题；为测井含气量评价提供可迁移框架
+【局限性】10口井样本仍属小样本；深部&gt;1500 m段模型不确定性升高；结果具有区块和煤阶依赖性
+【与你课题的关系】含气量评价/测井-地质-工程一体化/深度学习适用性/小样本增广策略</t>
+  </si>
+  <si>
+    <t>模型可迁移性和资料完整性。</t>
+  </si>
+  <si>
     <t>日期</t>
   </si>
   <si>
@@ -10175,6 +10398,12 @@
     <t>新增: DCBM-135, DCBM-136; 跳过重复: 0; 主库记录数更新为 13 → (待QC确认)</t>
   </si>
   <si>
+    <t>2026-07-26 Daily Brief Update</t>
+  </si>
+  <si>
+    <t>新增: DCBM-137, DCBM-138, DCBM-139; 跳过重复: 0; 主库记录数更新为 14 → (待QC确认)</t>
+  </si>
+  <si>
     <t>候选原编号</t>
   </si>
   <si>
@@ -10320,6 +10549,9 @@
   </si>
   <si>
     <t>新增 2 篇, 跳过重复 0 篇, 待 validate 确认</t>
+  </si>
+  <si>
+    <t>Daily Brief Update 2026-07-26</t>
   </si>
 </sst>
 </file>
@@ -10662,7 +10894,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA137"/>
+  <dimension ref="A1:AA140"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="13.8" outlineLevelCol="0"/>
   <cols>
     <col customWidth="1" max="1" min="1" width="8"/>
@@ -21942,6 +22174,249 @@
         <v>2803</v>
       </c>
     </row>
+    <row r="138" spans="1:27">
+      <c r="A138" t="n">
+        <v>137</v>
+      </c>
+      <c r="B138" t="s">
+        <v>2804</v>
+      </c>
+      <c r="C138" t="s">
+        <v>2805</v>
+      </c>
+      <c r="D138" t="s">
+        <v>2806</v>
+      </c>
+      <c r="E138" t="s">
+        <v>31</v>
+      </c>
+      <c r="F138" t="s">
+        <v>2807</v>
+      </c>
+      <c r="G138" t="s">
+        <v>2808</v>
+      </c>
+      <c r="H138" t="s">
+        <v>1145</v>
+      </c>
+      <c r="I138" t="s">
+        <v>655</v>
+      </c>
+      <c r="K138" t="s">
+        <v>2809</v>
+      </c>
+      <c r="L138" t="s">
+        <v>2810</v>
+      </c>
+      <c r="M138" t="s">
+        <v>2811</v>
+      </c>
+      <c r="N138" t="s">
+        <v>2466</v>
+      </c>
+      <c r="O138" t="s">
+        <v>2812</v>
+      </c>
+      <c r="P138" t="s">
+        <v>2813</v>
+      </c>
+      <c r="Q138" t="s">
+        <v>2814</v>
+      </c>
+      <c r="R138" t="s">
+        <v>2815</v>
+      </c>
+      <c r="S138" t="s">
+        <v>2816</v>
+      </c>
+      <c r="T138" t="s">
+        <v>2817</v>
+      </c>
+      <c r="U138" t="s">
+        <v>2818</v>
+      </c>
+      <c r="V138" t="s">
+        <v>2819</v>
+      </c>
+      <c r="W138" t="s">
+        <v>2820</v>
+      </c>
+      <c r="X138" t="s">
+        <v>2821</v>
+      </c>
+      <c r="Y138" t="s">
+        <v>2822</v>
+      </c>
+      <c r="Z138" t="s">
+        <v>52</v>
+      </c>
+      <c r="AA138" t="s">
+        <v>2823</v>
+      </c>
+    </row>
+    <row r="139" spans="1:27">
+      <c r="A139" t="n">
+        <v>138</v>
+      </c>
+      <c r="B139" t="s">
+        <v>2824</v>
+      </c>
+      <c r="C139" t="s">
+        <v>2825</v>
+      </c>
+      <c r="D139" t="s">
+        <v>2826</v>
+      </c>
+      <c r="E139" t="s">
+        <v>31</v>
+      </c>
+      <c r="F139" t="s">
+        <v>2827</v>
+      </c>
+      <c r="G139" t="s">
+        <v>2828</v>
+      </c>
+      <c r="H139" t="s">
+        <v>638</v>
+      </c>
+      <c r="I139" t="s">
+        <v>351</v>
+      </c>
+      <c r="K139" t="s">
+        <v>2829</v>
+      </c>
+      <c r="L139" t="s">
+        <v>2830</v>
+      </c>
+      <c r="M139" t="s">
+        <v>2831</v>
+      </c>
+      <c r="N139" t="s">
+        <v>2466</v>
+      </c>
+      <c r="O139" t="s">
+        <v>2832</v>
+      </c>
+      <c r="P139" t="s">
+        <v>2833</v>
+      </c>
+      <c r="Q139" t="s">
+        <v>2834</v>
+      </c>
+      <c r="R139" t="s">
+        <v>2835</v>
+      </c>
+      <c r="S139" t="s">
+        <v>2836</v>
+      </c>
+      <c r="T139" t="s">
+        <v>2837</v>
+      </c>
+      <c r="U139" t="s">
+        <v>2838</v>
+      </c>
+      <c r="V139" t="s">
+        <v>2839</v>
+      </c>
+      <c r="W139" t="s">
+        <v>2840</v>
+      </c>
+      <c r="X139" t="s">
+        <v>2841</v>
+      </c>
+      <c r="Y139" t="s">
+        <v>2842</v>
+      </c>
+      <c r="Z139" t="s">
+        <v>145</v>
+      </c>
+      <c r="AA139" t="s">
+        <v>2843</v>
+      </c>
+    </row>
+    <row r="140" spans="1:27">
+      <c r="A140" t="n">
+        <v>139</v>
+      </c>
+      <c r="B140" t="s">
+        <v>2844</v>
+      </c>
+      <c r="C140" t="s">
+        <v>2845</v>
+      </c>
+      <c r="D140" t="s">
+        <v>2846</v>
+      </c>
+      <c r="E140" t="s">
+        <v>31</v>
+      </c>
+      <c r="F140" t="s">
+        <v>2847</v>
+      </c>
+      <c r="G140" t="s">
+        <v>2848</v>
+      </c>
+      <c r="H140" t="s">
+        <v>2849</v>
+      </c>
+      <c r="I140" t="s">
+        <v>1292</v>
+      </c>
+      <c r="J140" t="s">
+        <v>169</v>
+      </c>
+      <c r="K140" t="s">
+        <v>2850</v>
+      </c>
+      <c r="L140" t="s">
+        <v>2851</v>
+      </c>
+      <c r="M140" t="s">
+        <v>2852</v>
+      </c>
+      <c r="N140" t="s">
+        <v>2466</v>
+      </c>
+      <c r="O140" t="s">
+        <v>2853</v>
+      </c>
+      <c r="P140" t="s">
+        <v>2854</v>
+      </c>
+      <c r="Q140" t="s">
+        <v>2855</v>
+      </c>
+      <c r="R140" t="s">
+        <v>2856</v>
+      </c>
+      <c r="S140" t="s">
+        <v>2857</v>
+      </c>
+      <c r="T140" t="s">
+        <v>2858</v>
+      </c>
+      <c r="U140" t="s">
+        <v>2859</v>
+      </c>
+      <c r="V140" t="s">
+        <v>2860</v>
+      </c>
+      <c r="W140" t="s">
+        <v>2861</v>
+      </c>
+      <c r="X140" t="s">
+        <v>2862</v>
+      </c>
+      <c r="Y140" t="s">
+        <v>2863</v>
+      </c>
+      <c r="Z140" t="s">
+        <v>52</v>
+      </c>
+      <c r="AA140" t="s">
+        <v>2864</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M120" r:id="rId1"/>
@@ -21961,7 +22436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F18"/>
+  <dimension ref="A1:F17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="13.8" outlineLevelCol="0"/>
   <cols>
     <col customWidth="1" max="6" min="1" width="22"/>
@@ -21969,13 +22444,13 @@
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" s="2" t="s">
-        <v>2804</v>
+        <v>2865</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>2805</v>
+        <v>2866</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>2806</v>
+        <v>2867</v>
       </c>
       <c r="D1" s="2" t="n"/>
       <c r="E1" s="2" t="n"/>
@@ -21983,13 +22458,13 @@
     </row>
     <row r="2" spans="1:6">
       <c r="A2" s="3" t="s">
-        <v>2807</v>
+        <v>2868</v>
       </c>
       <c r="B2" s="3" t="n">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>2808</v>
+        <v>2869</v>
       </c>
       <c r="D2" s="3" t="n"/>
       <c r="E2" s="3" t="n"/>
@@ -21997,13 +22472,13 @@
     </row>
     <row customHeight="1" ht="27.6" r="3" spans="1:6">
       <c r="A3" s="3" t="s">
-        <v>2809</v>
+        <v>2870</v>
       </c>
       <c r="B3" s="3" t="n">
         <v>21</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>2810</v>
+        <v>2871</v>
       </c>
       <c r="D3" s="3" t="n"/>
       <c r="E3" s="3" t="n"/>
@@ -22011,13 +22486,13 @@
     </row>
     <row customHeight="1" ht="27.6" r="4" spans="1:6">
       <c r="A4" s="3" t="s">
-        <v>2811</v>
+        <v>2872</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>2812</v>
+        <v>2873</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>2813</v>
+        <v>2874</v>
       </c>
       <c r="D4" s="3" t="n"/>
       <c r="E4" s="3" t="n"/>
@@ -22025,13 +22500,13 @@
     </row>
     <row customHeight="1" ht="27.6" r="5" spans="1:6">
       <c r="A5" s="3" t="s">
-        <v>2814</v>
+        <v>2875</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>2815</v>
+        <v>2876</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>2816</v>
+        <v>2877</v>
       </c>
       <c r="D5" s="3" t="n"/>
       <c r="E5" s="3" t="n"/>
@@ -22039,13 +22514,13 @@
     </row>
     <row customHeight="1" ht="27.6" r="6" spans="1:6">
       <c r="A6" s="3" t="s">
-        <v>2817</v>
+        <v>2878</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>2818</v>
+        <v>2879</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>2819</v>
+        <v>2880</v>
       </c>
       <c r="D6" s="3" t="n"/>
       <c r="E6" s="3" t="n"/>
@@ -22056,14 +22531,14 @@
         <v>4</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>2820</v>
+        <v>2881</v>
       </c>
       <c r="C7" s="3" t="n"/>
       <c r="D7" s="3" t="s">
         <v>13</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>2820</v>
+        <v>2881</v>
       </c>
       <c r="F7" s="3" t="n"/>
     </row>
@@ -22101,7 +22576,7 @@
     </row>
     <row r="10" spans="1:6">
       <c r="A10" s="3" t="s">
-        <v>2821</v>
+        <v>2882</v>
       </c>
       <c r="B10" s="3" t="n">
         <v>1</v>
@@ -22117,7 +22592,7 @@
     </row>
     <row r="11" spans="1:6">
       <c r="A11" s="3" t="s">
-        <v>2822</v>
+        <v>2883</v>
       </c>
       <c r="B11" s="3" t="n">
         <v>1</v>
@@ -22133,7 +22608,7 @@
     </row>
     <row r="12" spans="1:6">
       <c r="A12" s="3" t="s">
-        <v>2823</v>
+        <v>2884</v>
       </c>
       <c r="B12" s="3" t="n">
         <v>1</v>
@@ -22200,7 +22675,7 @@
         <v>31</v>
       </c>
       <c r="B16" s="3" t="n">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="C16" s="3" t="n"/>
       <c r="D16" s="3" t="s">
@@ -22219,7 +22694,6 @@
         <v>2</v>
       </c>
     </row>
-    <row r="18" spans="1:6"/>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
@@ -22231,7 +22705,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H136"/>
+  <dimension ref="A1:H139"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="13.8" outlineLevelCol="0"/>
   <cols>
     <col customWidth="1" max="1" min="1" width="8"/>
@@ -25734,6 +26208,39 @@
       </c>
       <c r="F136" t="s">
         <v>2791</v>
+      </c>
+    </row>
+    <row r="137" spans="1:8">
+      <c r="A137" t="n">
+        <v>137</v>
+      </c>
+      <c r="B137" t="s">
+        <v>2804</v>
+      </c>
+      <c r="F137" t="s">
+        <v>2810</v>
+      </c>
+    </row>
+    <row r="138" spans="1:8">
+      <c r="A138" t="n">
+        <v>138</v>
+      </c>
+      <c r="B138" t="s">
+        <v>2824</v>
+      </c>
+      <c r="F138" t="s">
+        <v>2830</v>
+      </c>
+    </row>
+    <row r="139" spans="1:8">
+      <c r="A139" t="n">
+        <v>139</v>
+      </c>
+      <c r="B139" t="s">
+        <v>2844</v>
+      </c>
+      <c r="F139" t="s">
+        <v>2851</v>
       </c>
     </row>
   </sheetData>
@@ -25759,10 +26266,10 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="2" t="s">
-        <v>2824</v>
+        <v>2885</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>2806</v>
+        <v>2867</v>
       </c>
     </row>
     <row r="2" spans="1:2">
@@ -25770,7 +26277,7 @@
         <v>0</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>2825</v>
+        <v>2886</v>
       </c>
     </row>
     <row r="3" spans="1:2">
@@ -25778,7 +26285,7 @@
         <v>1</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>2826</v>
+        <v>2887</v>
       </c>
     </row>
     <row r="4" spans="1:2">
@@ -25786,7 +26293,7 @@
         <v>2</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>2827</v>
+        <v>2888</v>
       </c>
     </row>
     <row r="5" spans="1:2">
@@ -25794,7 +26301,7 @@
         <v>3</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>2828</v>
+        <v>2889</v>
       </c>
     </row>
     <row r="6" spans="1:2">
@@ -25802,7 +26309,7 @@
         <v>4</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>2829</v>
+        <v>2890</v>
       </c>
     </row>
     <row r="7" spans="1:2">
@@ -25810,7 +26317,7 @@
         <v>5</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>2830</v>
+        <v>2891</v>
       </c>
     </row>
     <row r="8" spans="1:2">
@@ -25818,7 +26325,7 @@
         <v>6</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>2831</v>
+        <v>2892</v>
       </c>
     </row>
     <row r="9" spans="1:2">
@@ -25826,15 +26333,15 @@
         <v>7</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>2832</v>
+        <v>2893</v>
       </c>
     </row>
     <row r="10" spans="1:2">
       <c r="A10" s="3" t="s">
-        <v>2833</v>
+        <v>2894</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>2834</v>
+        <v>2895</v>
       </c>
     </row>
     <row r="11" spans="1:2">
@@ -25842,7 +26349,7 @@
         <v>11</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>2835</v>
+        <v>2896</v>
       </c>
     </row>
     <row r="12" spans="1:2">
@@ -25850,7 +26357,7 @@
         <v>12</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>2836</v>
+        <v>2897</v>
       </c>
     </row>
     <row r="13" spans="1:2">
@@ -25858,7 +26365,7 @@
         <v>13</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>2837</v>
+        <v>2898</v>
       </c>
     </row>
     <row r="14" spans="1:2">
@@ -25866,7 +26373,7 @@
         <v>14</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>2838</v>
+        <v>2899</v>
       </c>
     </row>
     <row r="15" spans="1:2">
@@ -25874,7 +26381,7 @@
         <v>15</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>2839</v>
+        <v>2900</v>
       </c>
     </row>
     <row r="16" spans="1:2">
@@ -25882,7 +26389,7 @@
         <v>16</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>2840</v>
+        <v>2901</v>
       </c>
     </row>
     <row r="17" spans="1:2">
@@ -25890,7 +26397,7 @@
         <v>17</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>2841</v>
+        <v>2902</v>
       </c>
     </row>
     <row r="18" spans="1:2">
@@ -25898,7 +26405,7 @@
         <v>18</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>2842</v>
+        <v>2903</v>
       </c>
     </row>
     <row r="19" spans="1:2">
@@ -25906,7 +26413,7 @@
         <v>19</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>2843</v>
+        <v>2904</v>
       </c>
     </row>
     <row r="20" spans="1:2">
@@ -25914,7 +26421,7 @@
         <v>20</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>2844</v>
+        <v>2905</v>
       </c>
     </row>
     <row r="21" spans="1:2">
@@ -25922,7 +26429,7 @@
         <v>21</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>2845</v>
+        <v>2906</v>
       </c>
     </row>
     <row r="22" spans="1:2">
@@ -25930,7 +26437,7 @@
         <v>22</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>2846</v>
+        <v>2907</v>
       </c>
     </row>
     <row r="23" spans="1:2">
@@ -25938,7 +26445,7 @@
         <v>23</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>2847</v>
+        <v>2908</v>
       </c>
     </row>
     <row r="24" spans="1:2">
@@ -25946,7 +26453,7 @@
         <v>24</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>2848</v>
+        <v>2909</v>
       </c>
     </row>
     <row r="25" spans="1:2">
@@ -25954,7 +26461,7 @@
         <v>25</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>2849</v>
+        <v>2910</v>
       </c>
     </row>
     <row r="26" spans="1:2">
@@ -25962,7 +26469,7 @@
         <v>26</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>2850</v>
+        <v>2911</v>
       </c>
     </row>
   </sheetData>
@@ -25976,7 +26483,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N137"/>
+  <dimension ref="A1:N140"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="13.8" outlineLevelCol="0"/>
   <cols>
     <col customWidth="1" max="1" min="1" width="12"/>
@@ -26001,22 +26508,22 @@
         <v>4</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>2851</v>
+        <v>2912</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>2852</v>
+        <v>2913</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>2853</v>
+        <v>2914</v>
       </c>
       <c r="F1" s="5" t="s">
         <v>17</v>
       </c>
       <c r="G1" s="5" t="s">
-        <v>2854</v>
+        <v>2915</v>
       </c>
       <c r="H1" s="5" t="s">
-        <v>2855</v>
+        <v>2916</v>
       </c>
       <c r="I1" s="5" t="s">
         <v>20</v>
@@ -26025,16 +26532,16 @@
         <v>21</v>
       </c>
       <c r="K1" s="5" t="s">
-        <v>2856</v>
+        <v>2917</v>
       </c>
       <c r="L1" s="5" t="s">
-        <v>2857</v>
+        <v>2918</v>
       </c>
       <c r="M1" s="5" t="s">
         <v>25</v>
       </c>
       <c r="N1" s="5" t="s">
-        <v>2858</v>
+        <v>2919</v>
       </c>
     </row>
     <row customHeight="1" ht="110.4" r="2" spans="1:14">
@@ -26048,10 +26555,10 @@
         <v>33</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>2859</v>
+        <v>2920</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>2860</v>
+        <v>2921</v>
       </c>
       <c r="F2" s="1" t="s">
         <v>44</v>
@@ -26078,7 +26585,7 @@
         <v>52</v>
       </c>
       <c r="N2" s="1" t="s">
-        <v>2861</v>
+        <v>2922</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="3" spans="1:14">
@@ -26092,10 +26599,10 @@
         <v>59</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>2862</v>
+        <v>2923</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>2863</v>
+        <v>2924</v>
       </c>
       <c r="F3" s="1" t="s">
         <v>68</v>
@@ -26122,7 +26629,7 @@
         <v>52</v>
       </c>
       <c r="N3" s="1" t="s">
-        <v>2861</v>
+        <v>2922</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="4" spans="1:14">
@@ -26136,10 +26643,10 @@
         <v>83</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>2864</v>
+        <v>2925</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>2865</v>
+        <v>2926</v>
       </c>
       <c r="F4" s="1" t="s">
         <v>92</v>
@@ -26166,7 +26673,7 @@
         <v>52</v>
       </c>
       <c r="N4" s="1" t="s">
-        <v>2861</v>
+        <v>2922</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="5" spans="1:14">
@@ -26180,10 +26687,10 @@
         <v>106</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>2866</v>
+        <v>2927</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>2867</v>
+        <v>2928</v>
       </c>
       <c r="F5" s="1" t="s">
         <v>115</v>
@@ -26210,7 +26717,7 @@
         <v>52</v>
       </c>
       <c r="N5" s="1" t="s">
-        <v>2861</v>
+        <v>2922</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="6" spans="1:14">
@@ -26224,10 +26731,10 @@
         <v>128</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>2868</v>
+        <v>2929</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>2869</v>
+        <v>2930</v>
       </c>
       <c r="F6" s="1" t="s">
         <v>137</v>
@@ -26254,7 +26761,7 @@
         <v>145</v>
       </c>
       <c r="N6" s="1" t="s">
-        <v>2861</v>
+        <v>2922</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="7" spans="1:14">
@@ -26268,10 +26775,10 @@
         <v>152</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>2870</v>
+        <v>2931</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>2871</v>
+        <v>2932</v>
       </c>
       <c r="F7" s="1" t="s">
         <v>160</v>
@@ -26298,7 +26805,7 @@
         <v>145</v>
       </c>
       <c r="N7" s="1" t="s">
-        <v>2861</v>
+        <v>2922</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="8" spans="1:14">
@@ -26312,10 +26819,10 @@
         <v>174</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>2872</v>
+        <v>2933</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>2873</v>
+        <v>2934</v>
       </c>
       <c r="F8" s="1" t="s">
         <v>181</v>
@@ -26342,7 +26849,7 @@
         <v>189</v>
       </c>
       <c r="N8" s="1" t="s">
-        <v>2861</v>
+        <v>2922</v>
       </c>
     </row>
     <row customHeight="1" ht="82.8" r="9" spans="1:14">
@@ -26356,10 +26863,10 @@
         <v>195</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>2874</v>
+        <v>2935</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>2875</v>
+        <v>2936</v>
       </c>
       <c r="F9" s="1" t="s">
         <v>201</v>
@@ -26386,7 +26893,7 @@
         <v>145</v>
       </c>
       <c r="N9" s="1" t="s">
-        <v>2861</v>
+        <v>2922</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="10" spans="1:14">
@@ -26400,10 +26907,10 @@
         <v>214</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>2876</v>
+        <v>2937</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>2877</v>
+        <v>2938</v>
       </c>
       <c r="F10" s="1" t="s">
         <v>220</v>
@@ -26430,7 +26937,7 @@
         <v>52</v>
       </c>
       <c r="N10" s="1" t="s">
-        <v>2861</v>
+        <v>2922</v>
       </c>
     </row>
     <row customHeight="1" ht="82.8" r="11" spans="1:14">
@@ -26444,10 +26951,10 @@
         <v>233</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>2878</v>
+        <v>2939</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>2879</v>
+        <v>2940</v>
       </c>
       <c r="F11" s="1" t="s">
         <v>239</v>
@@ -26474,7 +26981,7 @@
         <v>189</v>
       </c>
       <c r="N11" s="1" t="s">
-        <v>2861</v>
+        <v>2922</v>
       </c>
     </row>
     <row customHeight="1" ht="82.8" r="12" spans="1:14">
@@ -26488,10 +26995,10 @@
         <v>252</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>2880</v>
+        <v>2941</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>2881</v>
+        <v>2942</v>
       </c>
       <c r="F12" s="1" t="s">
         <v>258</v>
@@ -26518,7 +27025,7 @@
         <v>145</v>
       </c>
       <c r="N12" s="1" t="s">
-        <v>2861</v>
+        <v>2922</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="13" spans="1:14">
@@ -26532,10 +27039,10 @@
         <v>272</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>2882</v>
+        <v>2943</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>2883</v>
+        <v>2944</v>
       </c>
       <c r="F13" s="1" t="s">
         <v>278</v>
@@ -26562,7 +27069,7 @@
         <v>52</v>
       </c>
       <c r="N13" s="1" t="s">
-        <v>2861</v>
+        <v>2922</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="14" spans="1:14">
@@ -26576,10 +27083,10 @@
         <v>291</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>2884</v>
+        <v>2945</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>2885</v>
+        <v>2946</v>
       </c>
       <c r="F14" s="1" t="s">
         <v>300</v>
@@ -26606,7 +27113,7 @@
         <v>145</v>
       </c>
       <c r="N14" s="1" t="s">
-        <v>2861</v>
+        <v>2922</v>
       </c>
     </row>
     <row customHeight="1" ht="82.8" r="15" spans="1:14">
@@ -26620,10 +27127,10 @@
         <v>313</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>2886</v>
+        <v>2947</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>2887</v>
+        <v>2948</v>
       </c>
       <c r="F15" s="1" t="s">
         <v>321</v>
@@ -26650,7 +27157,7 @@
         <v>52</v>
       </c>
       <c r="N15" s="1" t="s">
-        <v>2861</v>
+        <v>2922</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="16" spans="1:14">
@@ -26664,10 +27171,10 @@
         <v>334</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>2888</v>
+        <v>2949</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>2889</v>
+        <v>2950</v>
       </c>
       <c r="F16" s="1" t="s">
         <v>343</v>
@@ -26694,7 +27201,7 @@
         <v>52</v>
       </c>
       <c r="N16" s="1" t="s">
-        <v>2861</v>
+        <v>2922</v>
       </c>
     </row>
     <row customHeight="1" ht="82.8" r="17" spans="1:14">
@@ -26708,10 +27215,10 @@
         <v>356</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>2890</v>
+        <v>2951</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>2891</v>
+        <v>2952</v>
       </c>
       <c r="F17" s="1" t="s">
         <v>363</v>
@@ -26738,7 +27245,7 @@
         <v>52</v>
       </c>
       <c r="N17" s="1" t="s">
-        <v>2861</v>
+        <v>2922</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="18" spans="1:14">
@@ -26752,10 +27259,10 @@
         <v>376</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>2892</v>
+        <v>2953</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>2893</v>
+        <v>2954</v>
       </c>
       <c r="F18" s="1" t="s">
         <v>383</v>
@@ -26782,7 +27289,7 @@
         <v>145</v>
       </c>
       <c r="N18" s="1" t="s">
-        <v>2861</v>
+        <v>2922</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="19" spans="1:14">
@@ -26796,10 +27303,10 @@
         <v>397</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>2894</v>
+        <v>2955</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>2895</v>
+        <v>2956</v>
       </c>
       <c r="F19" s="1" t="s">
         <v>404</v>
@@ -26826,7 +27333,7 @@
         <v>145</v>
       </c>
       <c r="N19" s="1" t="s">
-        <v>2861</v>
+        <v>2922</v>
       </c>
     </row>
     <row customHeight="1" ht="82.8" r="20" spans="1:14">
@@ -26840,10 +27347,10 @@
         <v>418</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>2896</v>
+        <v>2957</v>
       </c>
       <c r="E20" s="1" t="s">
-        <v>2897</v>
+        <v>2958</v>
       </c>
       <c r="F20" s="1" t="s">
         <v>427</v>
@@ -26870,7 +27377,7 @@
         <v>145</v>
       </c>
       <c r="N20" s="1" t="s">
-        <v>2861</v>
+        <v>2922</v>
       </c>
     </row>
     <row customHeight="1" ht="82.8" r="21" spans="1:14">
@@ -26884,10 +27391,10 @@
         <v>441</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>2898</v>
+        <v>2959</v>
       </c>
       <c r="E21" s="1" t="s">
-        <v>2899</v>
+        <v>2960</v>
       </c>
       <c r="F21" s="1" t="s">
         <v>448</v>
@@ -26914,7 +27421,7 @@
         <v>145</v>
       </c>
       <c r="N21" s="1" t="s">
-        <v>2861</v>
+        <v>2922</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="22" spans="1:14">
@@ -26928,10 +27435,10 @@
         <v>462</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>2900</v>
+        <v>2961</v>
       </c>
       <c r="E22" s="1" t="s">
-        <v>2901</v>
+        <v>2962</v>
       </c>
       <c r="F22" s="1" t="s">
         <v>467</v>
@@ -26958,7 +27465,7 @@
         <v>52</v>
       </c>
       <c r="N22" s="1" t="s">
-        <v>2861</v>
+        <v>2922</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="23" spans="1:14">
@@ -26972,10 +27479,10 @@
         <v>481</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>2902</v>
+        <v>2963</v>
       </c>
       <c r="E23" s="1" t="s">
-        <v>2903</v>
+        <v>2964</v>
       </c>
       <c r="F23" s="1" t="s">
         <v>489</v>
@@ -27002,7 +27509,7 @@
         <v>145</v>
       </c>
       <c r="N23" s="1" t="s">
-        <v>2861</v>
+        <v>2922</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="24" spans="1:14">
@@ -27016,10 +27523,10 @@
         <v>503</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>2904</v>
+        <v>2965</v>
       </c>
       <c r="E24" s="1" t="s">
-        <v>2905</v>
+        <v>2966</v>
       </c>
       <c r="F24" s="1" t="s">
         <v>511</v>
@@ -27046,7 +27553,7 @@
         <v>52</v>
       </c>
       <c r="N24" s="1" t="s">
-        <v>2861</v>
+        <v>2922</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="25" spans="1:14">
@@ -27060,10 +27567,10 @@
         <v>524</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>2906</v>
+        <v>2967</v>
       </c>
       <c r="E25" s="1" t="s">
-        <v>2907</v>
+        <v>2968</v>
       </c>
       <c r="F25" s="1" t="s">
         <v>532</v>
@@ -27090,7 +27597,7 @@
         <v>145</v>
       </c>
       <c r="N25" s="1" t="s">
-        <v>2861</v>
+        <v>2922</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="26" spans="1:14">
@@ -27104,10 +27611,10 @@
         <v>546</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>2908</v>
+        <v>2969</v>
       </c>
       <c r="E26" s="1" t="s">
-        <v>2909</v>
+        <v>2970</v>
       </c>
       <c r="F26" s="1" t="s">
         <v>554</v>
@@ -27134,7 +27641,7 @@
         <v>52</v>
       </c>
       <c r="N26" s="1" t="s">
-        <v>2861</v>
+        <v>2922</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="27" spans="1:14">
@@ -27148,10 +27655,10 @@
         <v>568</v>
       </c>
       <c r="D27" s="1" t="s">
-        <v>2910</v>
+        <v>2971</v>
       </c>
       <c r="E27" s="1" t="s">
-        <v>2911</v>
+        <v>2972</v>
       </c>
       <c r="F27" s="1" t="s">
         <v>577</v>
@@ -27178,7 +27685,7 @@
         <v>52</v>
       </c>
       <c r="N27" s="1" t="s">
-        <v>2861</v>
+        <v>2922</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="28" spans="1:14">
@@ -27192,10 +27699,10 @@
         <v>591</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>2912</v>
+        <v>2973</v>
       </c>
       <c r="E28" s="1" t="s">
-        <v>2913</v>
+        <v>2974</v>
       </c>
       <c r="F28" s="1" t="s">
         <v>600</v>
@@ -27222,7 +27729,7 @@
         <v>52</v>
       </c>
       <c r="N28" s="1" t="s">
-        <v>2861</v>
+        <v>2922</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="29" spans="1:14">
@@ -27236,10 +27743,10 @@
         <v>614</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>2914</v>
+        <v>2975</v>
       </c>
       <c r="E29" s="1" t="s">
-        <v>2915</v>
+        <v>2976</v>
       </c>
       <c r="F29" s="1" t="s">
         <v>623</v>
@@ -27266,7 +27773,7 @@
         <v>52</v>
       </c>
       <c r="N29" s="1" t="s">
-        <v>2861</v>
+        <v>2922</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="30" spans="1:14">
@@ -27280,10 +27787,10 @@
         <v>637</v>
       </c>
       <c r="D30" s="1" t="s">
-        <v>2916</v>
+        <v>2977</v>
       </c>
       <c r="E30" s="1" t="s">
-        <v>2917</v>
+        <v>2978</v>
       </c>
       <c r="F30" s="1" t="s">
         <v>646</v>
@@ -27310,7 +27817,7 @@
         <v>52</v>
       </c>
       <c r="N30" s="1" t="s">
-        <v>2861</v>
+        <v>2922</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="31" spans="1:14">
@@ -27324,10 +27831,10 @@
         <v>659</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>2918</v>
+        <v>2979</v>
       </c>
       <c r="E31" s="1" t="s">
-        <v>2919</v>
+        <v>2980</v>
       </c>
       <c r="F31" s="1" t="s">
         <v>668</v>
@@ -27354,7 +27861,7 @@
         <v>52</v>
       </c>
       <c r="N31" s="1" t="s">
-        <v>2861</v>
+        <v>2922</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="32" spans="1:14">
@@ -27368,10 +27875,10 @@
         <v>682</v>
       </c>
       <c r="D32" s="1" t="s">
-        <v>2920</v>
+        <v>2981</v>
       </c>
       <c r="E32" s="1" t="s">
-        <v>2921</v>
+        <v>2982</v>
       </c>
       <c r="F32" s="1" t="s">
         <v>689</v>
@@ -27398,7 +27905,7 @@
         <v>52</v>
       </c>
       <c r="N32" s="1" t="s">
-        <v>2861</v>
+        <v>2922</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="33" spans="1:14">
@@ -27412,10 +27919,10 @@
         <v>702</v>
       </c>
       <c r="D33" s="1" t="s">
-        <v>2922</v>
+        <v>2983</v>
       </c>
       <c r="E33" s="1" t="s">
-        <v>2923</v>
+        <v>2984</v>
       </c>
       <c r="F33" s="1" t="s">
         <v>709</v>
@@ -27442,7 +27949,7 @@
         <v>145</v>
       </c>
       <c r="N33" s="1" t="s">
-        <v>2861</v>
+        <v>2922</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="34" spans="1:14">
@@ -27456,10 +27963,10 @@
         <v>722</v>
       </c>
       <c r="D34" s="1" t="s">
-        <v>2924</v>
+        <v>2985</v>
       </c>
       <c r="E34" s="1" t="s">
-        <v>2925</v>
+        <v>2986</v>
       </c>
       <c r="F34" s="1" t="s">
         <v>731</v>
@@ -27486,7 +27993,7 @@
         <v>52</v>
       </c>
       <c r="N34" s="1" t="s">
-        <v>2861</v>
+        <v>2922</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="35" spans="1:14">
@@ -27500,10 +28007,10 @@
         <v>744</v>
       </c>
       <c r="D35" s="1" t="s">
-        <v>2926</v>
+        <v>2987</v>
       </c>
       <c r="E35" s="1" t="s">
-        <v>2927</v>
+        <v>2988</v>
       </c>
       <c r="F35" s="1" t="s">
         <v>751</v>
@@ -27530,7 +28037,7 @@
         <v>52</v>
       </c>
       <c r="N35" s="1" t="s">
-        <v>2861</v>
+        <v>2922</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="36" spans="1:14">
@@ -27544,10 +28051,10 @@
         <v>764</v>
       </c>
       <c r="D36" s="1" t="s">
-        <v>2928</v>
+        <v>2989</v>
       </c>
       <c r="E36" s="1" t="s">
-        <v>2929</v>
+        <v>2990</v>
       </c>
       <c r="F36" s="1" t="s">
         <v>772</v>
@@ -27574,7 +28081,7 @@
         <v>145</v>
       </c>
       <c r="N36" s="1" t="s">
-        <v>2861</v>
+        <v>2922</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="37" spans="1:14">
@@ -27588,10 +28095,10 @@
         <v>785</v>
       </c>
       <c r="D37" s="1" t="s">
-        <v>2930</v>
+        <v>2991</v>
       </c>
       <c r="E37" s="1" t="s">
-        <v>2931</v>
+        <v>2992</v>
       </c>
       <c r="F37" s="1" t="s">
         <v>792</v>
@@ -27618,7 +28125,7 @@
         <v>145</v>
       </c>
       <c r="N37" s="1" t="s">
-        <v>2861</v>
+        <v>2922</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="38" spans="1:14">
@@ -27632,10 +28139,10 @@
         <v>806</v>
       </c>
       <c r="D38" s="1" t="s">
-        <v>2932</v>
+        <v>2993</v>
       </c>
       <c r="E38" s="1" t="s">
-        <v>2933</v>
+        <v>2994</v>
       </c>
       <c r="F38" s="1" t="s">
         <v>814</v>
@@ -27662,7 +28169,7 @@
         <v>145</v>
       </c>
       <c r="N38" s="1" t="s">
-        <v>2861</v>
+        <v>2922</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="39" spans="1:14">
@@ -27676,10 +28183,10 @@
         <v>827</v>
       </c>
       <c r="D39" s="1" t="s">
-        <v>2934</v>
+        <v>2995</v>
       </c>
       <c r="E39" s="1" t="s">
-        <v>2935</v>
+        <v>2996</v>
       </c>
       <c r="F39" s="1" t="s">
         <v>834</v>
@@ -27706,7 +28213,7 @@
         <v>145</v>
       </c>
       <c r="N39" s="1" t="s">
-        <v>2861</v>
+        <v>2922</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="40" spans="1:14">
@@ -27720,10 +28227,10 @@
         <v>848</v>
       </c>
       <c r="D40" s="1" t="s">
-        <v>2936</v>
+        <v>2997</v>
       </c>
       <c r="E40" s="1" t="s">
-        <v>2937</v>
+        <v>2998</v>
       </c>
       <c r="F40" s="1" t="s">
         <v>856</v>
@@ -27750,7 +28257,7 @@
         <v>52</v>
       </c>
       <c r="N40" s="1" t="s">
-        <v>2861</v>
+        <v>2922</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="41" spans="1:14">
@@ -27764,10 +28271,10 @@
         <v>870</v>
       </c>
       <c r="D41" s="1" t="s">
-        <v>2938</v>
+        <v>2999</v>
       </c>
       <c r="E41" s="1" t="s">
-        <v>2939</v>
+        <v>3000</v>
       </c>
       <c r="F41" s="1" t="s">
         <v>878</v>
@@ -27794,7 +28301,7 @@
         <v>52</v>
       </c>
       <c r="N41" s="1" t="s">
-        <v>2861</v>
+        <v>2922</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="42" spans="1:14">
@@ -27808,10 +28315,10 @@
         <v>891</v>
       </c>
       <c r="D42" s="1" t="s">
-        <v>2940</v>
+        <v>3001</v>
       </c>
       <c r="E42" s="1" t="s">
-        <v>2941</v>
+        <v>3002</v>
       </c>
       <c r="F42" s="1" t="s">
         <v>901</v>
@@ -27838,7 +28345,7 @@
         <v>52</v>
       </c>
       <c r="N42" s="1" t="s">
-        <v>2861</v>
+        <v>2922</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="43" spans="1:14">
@@ -27852,10 +28359,10 @@
         <v>914</v>
       </c>
       <c r="D43" s="1" t="s">
-        <v>2942</v>
+        <v>3003</v>
       </c>
       <c r="E43" s="1" t="s">
-        <v>2943</v>
+        <v>3004</v>
       </c>
       <c r="F43" s="1" t="s">
         <v>921</v>
@@ -27882,7 +28389,7 @@
         <v>52</v>
       </c>
       <c r="N43" s="1" t="s">
-        <v>2861</v>
+        <v>2922</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="44" spans="1:14">
@@ -27896,10 +28403,10 @@
         <v>933</v>
       </c>
       <c r="D44" s="1" t="s">
-        <v>2944</v>
+        <v>3005</v>
       </c>
       <c r="E44" s="1" t="s">
-        <v>2945</v>
+        <v>3006</v>
       </c>
       <c r="F44" s="1" t="s">
         <v>940</v>
@@ -27926,7 +28433,7 @@
         <v>52</v>
       </c>
       <c r="N44" s="1" t="s">
-        <v>2861</v>
+        <v>2922</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="45" spans="1:14">
@@ -27940,10 +28447,10 @@
         <v>953</v>
       </c>
       <c r="D45" s="1" t="s">
-        <v>2946</v>
+        <v>3007</v>
       </c>
       <c r="E45" s="1" t="s">
-        <v>2947</v>
+        <v>3008</v>
       </c>
       <c r="F45" s="1" t="s">
         <v>959</v>
@@ -27970,7 +28477,7 @@
         <v>52</v>
       </c>
       <c r="N45" s="1" t="s">
-        <v>2861</v>
+        <v>2922</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="46" spans="1:14">
@@ -27984,10 +28491,10 @@
         <v>972</v>
       </c>
       <c r="D46" s="1" t="s">
-        <v>2948</v>
+        <v>3009</v>
       </c>
       <c r="E46" s="1" t="s">
-        <v>2949</v>
+        <v>3010</v>
       </c>
       <c r="F46" s="1" t="s">
         <v>978</v>
@@ -28014,7 +28521,7 @@
         <v>52</v>
       </c>
       <c r="N46" s="1" t="s">
-        <v>2861</v>
+        <v>2922</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="47" spans="1:14">
@@ -28028,10 +28535,10 @@
         <v>990</v>
       </c>
       <c r="D47" s="1" t="s">
-        <v>2950</v>
+        <v>3011</v>
       </c>
       <c r="E47" s="1" t="s">
-        <v>2951</v>
+        <v>3012</v>
       </c>
       <c r="F47" s="1" t="s">
         <v>997</v>
@@ -28058,7 +28565,7 @@
         <v>52</v>
       </c>
       <c r="N47" s="1" t="s">
-        <v>2861</v>
+        <v>2922</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="48" spans="1:14">
@@ -28072,10 +28579,10 @@
         <v>1010</v>
       </c>
       <c r="D48" s="1" t="s">
-        <v>2952</v>
+        <v>3013</v>
       </c>
       <c r="E48" s="1" t="s">
-        <v>2953</v>
+        <v>3014</v>
       </c>
       <c r="F48" s="1" t="s">
         <v>1018</v>
@@ -28102,7 +28609,7 @@
         <v>52</v>
       </c>
       <c r="N48" s="1" t="s">
-        <v>2861</v>
+        <v>2922</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="49" spans="1:14">
@@ -28116,10 +28623,10 @@
         <v>1030</v>
       </c>
       <c r="D49" s="1" t="s">
-        <v>2954</v>
+        <v>3015</v>
       </c>
       <c r="E49" s="1" t="s">
-        <v>2955</v>
+        <v>3016</v>
       </c>
       <c r="F49" s="1" t="s">
         <v>1037</v>
@@ -28146,7 +28653,7 @@
         <v>52</v>
       </c>
       <c r="N49" s="1" t="s">
-        <v>2861</v>
+        <v>2922</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="50" spans="1:14">
@@ -28160,10 +28667,10 @@
         <v>1049</v>
       </c>
       <c r="D50" s="1" t="s">
-        <v>2956</v>
+        <v>3017</v>
       </c>
       <c r="E50" s="1" t="s">
-        <v>2957</v>
+        <v>3018</v>
       </c>
       <c r="F50" s="1" t="s">
         <v>1055</v>
@@ -28190,7 +28697,7 @@
         <v>189</v>
       </c>
       <c r="N50" s="1" t="s">
-        <v>2861</v>
+        <v>2922</v>
       </c>
     </row>
     <row customHeight="1" ht="82.8" r="51" spans="1:14">
@@ -28204,10 +28711,10 @@
         <v>1067</v>
       </c>
       <c r="D51" s="1" t="s">
-        <v>2958</v>
+        <v>3019</v>
       </c>
       <c r="E51" s="1" t="s">
-        <v>2959</v>
+        <v>3020</v>
       </c>
       <c r="F51" s="1" t="s">
         <v>1072</v>
@@ -28234,7 +28741,7 @@
         <v>52</v>
       </c>
       <c r="N51" s="1" t="s">
-        <v>2861</v>
+        <v>2922</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="52" spans="1:14">
@@ -28248,10 +28755,10 @@
         <v>1084</v>
       </c>
       <c r="D52" s="1" t="s">
-        <v>2960</v>
+        <v>3021</v>
       </c>
       <c r="E52" s="1" t="s">
-        <v>2961</v>
+        <v>3022</v>
       </c>
       <c r="F52" s="1" t="s">
         <v>1091</v>
@@ -28278,7 +28785,7 @@
         <v>189</v>
       </c>
       <c r="N52" s="1" t="s">
-        <v>2861</v>
+        <v>2922</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="53" spans="1:14">
@@ -28292,10 +28799,10 @@
         <v>1104</v>
       </c>
       <c r="D53" s="1" t="s">
-        <v>2962</v>
+        <v>3023</v>
       </c>
       <c r="E53" s="1" t="s">
-        <v>2963</v>
+        <v>3024</v>
       </c>
       <c r="F53" s="1" t="s">
         <v>1109</v>
@@ -28322,7 +28829,7 @@
         <v>145</v>
       </c>
       <c r="N53" s="1" t="s">
-        <v>2861</v>
+        <v>2922</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="54" spans="1:14">
@@ -28336,10 +28843,10 @@
         <v>1121</v>
       </c>
       <c r="D54" s="1" t="s">
-        <v>2964</v>
+        <v>3025</v>
       </c>
       <c r="E54" s="1" t="s">
-        <v>2965</v>
+        <v>3026</v>
       </c>
       <c r="F54" s="1" t="s">
         <v>1131</v>
@@ -28366,7 +28873,7 @@
         <v>52</v>
       </c>
       <c r="N54" s="1" t="s">
-        <v>2861</v>
+        <v>2922</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="55" spans="1:14">
@@ -28380,10 +28887,10 @@
         <v>1144</v>
       </c>
       <c r="D55" s="1" t="s">
-        <v>2966</v>
+        <v>3027</v>
       </c>
       <c r="E55" s="1" t="s">
-        <v>2967</v>
+        <v>3028</v>
       </c>
       <c r="F55" s="1" t="s">
         <v>1151</v>
@@ -28410,7 +28917,7 @@
         <v>52</v>
       </c>
       <c r="N55" s="1" t="s">
-        <v>2861</v>
+        <v>2922</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="56" spans="1:14">
@@ -28424,10 +28931,10 @@
         <v>1165</v>
       </c>
       <c r="D56" s="1" t="s">
-        <v>2968</v>
+        <v>3029</v>
       </c>
       <c r="E56" s="1" t="s">
-        <v>2969</v>
+        <v>3030</v>
       </c>
       <c r="F56" s="1" t="s">
         <v>1173</v>
@@ -28454,7 +28961,7 @@
         <v>52</v>
       </c>
       <c r="N56" s="1" t="s">
-        <v>2861</v>
+        <v>2922</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="57" spans="1:14">
@@ -28468,10 +28975,10 @@
         <v>1187</v>
       </c>
       <c r="D57" s="1" t="s">
-        <v>2970</v>
+        <v>3031</v>
       </c>
       <c r="E57" s="1" t="s">
-        <v>2971</v>
+        <v>3032</v>
       </c>
       <c r="F57" s="1" t="s">
         <v>1195</v>
@@ -28498,7 +29005,7 @@
         <v>189</v>
       </c>
       <c r="N57" s="1" t="s">
-        <v>2861</v>
+        <v>2922</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="58" spans="1:14">
@@ -28512,10 +29019,10 @@
         <v>1209</v>
       </c>
       <c r="D58" s="1" t="s">
-        <v>2972</v>
+        <v>3033</v>
       </c>
       <c r="E58" s="1" t="s">
-        <v>2973</v>
+        <v>3034</v>
       </c>
       <c r="F58" s="1" t="s">
         <v>1217</v>
@@ -28542,7 +29049,7 @@
         <v>189</v>
       </c>
       <c r="N58" s="1" t="s">
-        <v>2861</v>
+        <v>2922</v>
       </c>
     </row>
     <row customHeight="1" ht="82.8" r="59" spans="1:14">
@@ -28556,10 +29063,10 @@
         <v>1231</v>
       </c>
       <c r="D59" s="1" t="s">
-        <v>2974</v>
+        <v>3035</v>
       </c>
       <c r="E59" s="1" t="s">
-        <v>2975</v>
+        <v>3036</v>
       </c>
       <c r="F59" s="1" t="s">
         <v>1239</v>
@@ -28586,7 +29093,7 @@
         <v>189</v>
       </c>
       <c r="N59" s="1" t="s">
-        <v>2861</v>
+        <v>2922</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="60" spans="1:14">
@@ -28600,10 +29107,10 @@
         <v>1252</v>
       </c>
       <c r="D60" s="1" t="s">
-        <v>2976</v>
+        <v>3037</v>
       </c>
       <c r="E60" s="1" t="s">
-        <v>2977</v>
+        <v>3038</v>
       </c>
       <c r="F60" s="1" t="s">
         <v>1261</v>
@@ -28630,7 +29137,7 @@
         <v>52</v>
       </c>
       <c r="N60" s="1" t="s">
-        <v>2861</v>
+        <v>2922</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="61" spans="1:14">
@@ -28644,10 +29151,10 @@
         <v>1275</v>
       </c>
       <c r="D61" s="1" t="s">
-        <v>2978</v>
+        <v>3039</v>
       </c>
       <c r="E61" s="1" t="s">
-        <v>2979</v>
+        <v>3040</v>
       </c>
       <c r="F61" s="1" t="s">
         <v>1283</v>
@@ -28674,7 +29181,7 @@
         <v>52</v>
       </c>
       <c r="N61" s="1" t="s">
-        <v>2861</v>
+        <v>2922</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="62" spans="1:14">
@@ -28688,10 +29195,10 @@
         <v>1297</v>
       </c>
       <c r="D62" s="1" t="s">
-        <v>2980</v>
+        <v>3041</v>
       </c>
       <c r="E62" s="1" t="s">
-        <v>2981</v>
+        <v>3042</v>
       </c>
       <c r="F62" s="1" t="s">
         <v>1305</v>
@@ -28718,7 +29225,7 @@
         <v>145</v>
       </c>
       <c r="N62" s="1" t="s">
-        <v>2861</v>
+        <v>2922</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="63" spans="1:14">
@@ -28732,10 +29239,10 @@
         <v>1319</v>
       </c>
       <c r="D63" s="1" t="s">
-        <v>2982</v>
+        <v>3043</v>
       </c>
       <c r="E63" s="1" t="s">
-        <v>2983</v>
+        <v>3044</v>
       </c>
       <c r="F63" s="1" t="s">
         <v>1327</v>
@@ -28762,7 +29269,7 @@
         <v>189</v>
       </c>
       <c r="N63" s="1" t="s">
-        <v>2861</v>
+        <v>2922</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="64" spans="1:14">
@@ -28776,10 +29283,10 @@
         <v>1341</v>
       </c>
       <c r="D64" s="1" t="s">
-        <v>2984</v>
+        <v>3045</v>
       </c>
       <c r="E64" s="1" t="s">
-        <v>2985</v>
+        <v>3046</v>
       </c>
       <c r="F64" s="1" t="s">
         <v>1348</v>
@@ -28806,7 +29313,7 @@
         <v>52</v>
       </c>
       <c r="N64" s="1" t="s">
-        <v>2861</v>
+        <v>2922</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="65" spans="1:14">
@@ -28820,10 +29327,10 @@
         <v>1361</v>
       </c>
       <c r="D65" s="1" t="s">
-        <v>2986</v>
+        <v>3047</v>
       </c>
       <c r="E65" s="1" t="s">
-        <v>2987</v>
+        <v>3048</v>
       </c>
       <c r="F65" s="1" t="s">
         <v>1368</v>
@@ -28850,7 +29357,7 @@
         <v>52</v>
       </c>
       <c r="N65" s="1" t="s">
-        <v>2861</v>
+        <v>2922</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="66" spans="1:14">
@@ -28864,10 +29371,10 @@
         <v>1382</v>
       </c>
       <c r="D66" s="1" t="s">
-        <v>2988</v>
+        <v>3049</v>
       </c>
       <c r="E66" s="1" t="s">
-        <v>2989</v>
+        <v>3050</v>
       </c>
       <c r="F66" s="1" t="s">
         <v>1389</v>
@@ -28894,7 +29401,7 @@
         <v>52</v>
       </c>
       <c r="N66" s="1" t="s">
-        <v>2861</v>
+        <v>2922</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="67" spans="1:14">
@@ -28908,10 +29415,10 @@
         <v>1403</v>
       </c>
       <c r="D67" s="1" t="s">
-        <v>2990</v>
+        <v>3051</v>
       </c>
       <c r="E67" s="1" t="s">
-        <v>2991</v>
+        <v>3052</v>
       </c>
       <c r="F67" s="1" t="s">
         <v>1408</v>
@@ -28938,7 +29445,7 @@
         <v>52</v>
       </c>
       <c r="N67" s="1" t="s">
-        <v>2861</v>
+        <v>2922</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="68" spans="1:14">
@@ -28952,10 +29459,10 @@
         <v>1421</v>
       </c>
       <c r="D68" s="1" t="s">
-        <v>2992</v>
+        <v>3053</v>
       </c>
       <c r="E68" s="1" t="s">
-        <v>2993</v>
+        <v>3054</v>
       </c>
       <c r="F68" s="1" t="s">
         <v>1428</v>
@@ -28982,7 +29489,7 @@
         <v>52</v>
       </c>
       <c r="N68" s="1" t="s">
-        <v>2861</v>
+        <v>2922</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="69" spans="1:14">
@@ -28996,10 +29503,10 @@
         <v>1442</v>
       </c>
       <c r="D69" s="1" t="s">
-        <v>2994</v>
+        <v>3055</v>
       </c>
       <c r="E69" s="1" t="s">
-        <v>2995</v>
+        <v>3056</v>
       </c>
       <c r="F69" s="1" t="s">
         <v>1448</v>
@@ -29026,7 +29533,7 @@
         <v>52</v>
       </c>
       <c r="N69" s="1" t="s">
-        <v>2861</v>
+        <v>2922</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="70" spans="1:14">
@@ -29040,10 +29547,10 @@
         <v>1460</v>
       </c>
       <c r="D70" s="1" t="s">
-        <v>2996</v>
+        <v>3057</v>
       </c>
       <c r="E70" s="1" t="s">
-        <v>2997</v>
+        <v>3058</v>
       </c>
       <c r="F70" s="1" t="s">
         <v>1466</v>
@@ -29070,7 +29577,7 @@
         <v>52</v>
       </c>
       <c r="N70" s="1" t="s">
-        <v>2861</v>
+        <v>2922</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="71" spans="1:14">
@@ -29084,10 +29591,10 @@
         <v>1480</v>
       </c>
       <c r="D71" s="1" t="s">
-        <v>2998</v>
+        <v>3059</v>
       </c>
       <c r="E71" s="1" t="s">
-        <v>2999</v>
+        <v>3060</v>
       </c>
       <c r="F71" s="1" t="s">
         <v>1486</v>
@@ -29114,7 +29621,7 @@
         <v>52</v>
       </c>
       <c r="N71" s="1" t="s">
-        <v>2861</v>
+        <v>2922</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="72" spans="1:14">
@@ -29128,10 +29635,10 @@
         <v>1499</v>
       </c>
       <c r="D72" s="1" t="s">
-        <v>3000</v>
+        <v>3061</v>
       </c>
       <c r="E72" s="1" t="s">
-        <v>3001</v>
+        <v>3062</v>
       </c>
       <c r="F72" s="1" t="s">
         <v>1505</v>
@@ -29158,7 +29665,7 @@
         <v>52</v>
       </c>
       <c r="N72" s="1" t="s">
-        <v>2861</v>
+        <v>2922</v>
       </c>
     </row>
     <row customHeight="1" ht="82.8" r="73" spans="1:14">
@@ -29172,10 +29679,10 @@
         <v>1518</v>
       </c>
       <c r="D73" s="1" t="s">
-        <v>3002</v>
+        <v>3063</v>
       </c>
       <c r="E73" s="1" t="s">
-        <v>3003</v>
+        <v>3064</v>
       </c>
       <c r="F73" s="1" t="s">
         <v>1524</v>
@@ -29202,7 +29709,7 @@
         <v>145</v>
       </c>
       <c r="N73" s="1" t="s">
-        <v>2861</v>
+        <v>2922</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="74" spans="1:14">
@@ -29216,10 +29723,10 @@
         <v>1537</v>
       </c>
       <c r="D74" s="1" t="s">
-        <v>3004</v>
+        <v>3065</v>
       </c>
       <c r="E74" s="1" t="s">
-        <v>3005</v>
+        <v>3066</v>
       </c>
       <c r="F74" s="1" t="s">
         <v>1544</v>
@@ -29246,7 +29753,7 @@
         <v>52</v>
       </c>
       <c r="N74" s="1" t="s">
-        <v>2861</v>
+        <v>2922</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="75" spans="1:14">
@@ -29260,10 +29767,10 @@
         <v>1556</v>
       </c>
       <c r="D75" s="1" t="s">
-        <v>3006</v>
+        <v>3067</v>
       </c>
       <c r="E75" s="1" t="s">
-        <v>3007</v>
+        <v>3068</v>
       </c>
       <c r="F75" s="1" t="s">
         <v>1563</v>
@@ -29290,7 +29797,7 @@
         <v>52</v>
       </c>
       <c r="N75" s="1" t="s">
-        <v>2861</v>
+        <v>2922</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="76" spans="1:14">
@@ -29304,10 +29811,10 @@
         <v>1576</v>
       </c>
       <c r="D76" s="1" t="s">
-        <v>3008</v>
+        <v>3069</v>
       </c>
       <c r="E76" s="1" t="s">
-        <v>3009</v>
+        <v>3070</v>
       </c>
       <c r="F76" s="1" t="s">
         <v>1583</v>
@@ -29334,7 +29841,7 @@
         <v>52</v>
       </c>
       <c r="N76" s="1" t="s">
-        <v>2861</v>
+        <v>2922</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="77" spans="1:14">
@@ -29348,10 +29855,10 @@
         <v>1596</v>
       </c>
       <c r="D77" s="1" t="s">
-        <v>3010</v>
+        <v>3071</v>
       </c>
       <c r="E77" s="1" t="s">
-        <v>3011</v>
+        <v>3072</v>
       </c>
       <c r="F77" s="1" t="s">
         <v>1602</v>
@@ -29378,7 +29885,7 @@
         <v>52</v>
       </c>
       <c r="N77" s="1" t="s">
-        <v>2861</v>
+        <v>2922</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="78" spans="1:14">
@@ -29392,10 +29899,10 @@
         <v>1615</v>
       </c>
       <c r="D78" s="1" t="s">
-        <v>3012</v>
+        <v>3073</v>
       </c>
       <c r="E78" s="1" t="s">
-        <v>3013</v>
+        <v>3074</v>
       </c>
       <c r="F78" s="1" t="s">
         <v>1621</v>
@@ -29422,7 +29929,7 @@
         <v>52</v>
       </c>
       <c r="N78" s="1" t="s">
-        <v>2861</v>
+        <v>2922</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="79" spans="1:14">
@@ -29436,10 +29943,10 @@
         <v>1634</v>
       </c>
       <c r="D79" s="1" t="s">
-        <v>3014</v>
+        <v>3075</v>
       </c>
       <c r="E79" s="1" t="s">
-        <v>3015</v>
+        <v>3076</v>
       </c>
       <c r="F79" s="1" t="s">
         <v>1643</v>
@@ -29466,7 +29973,7 @@
         <v>145</v>
       </c>
       <c r="N79" s="1" t="s">
-        <v>2861</v>
+        <v>2922</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="80" spans="1:14">
@@ -29480,10 +29987,10 @@
         <v>1657</v>
       </c>
       <c r="D80" s="1" t="s">
-        <v>3016</v>
+        <v>3077</v>
       </c>
       <c r="E80" s="1" t="s">
-        <v>3017</v>
+        <v>3078</v>
       </c>
       <c r="F80" s="1" t="s">
         <v>1665</v>
@@ -29510,7 +30017,7 @@
         <v>189</v>
       </c>
       <c r="N80" s="1" t="s">
-        <v>2861</v>
+        <v>2922</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="81" spans="1:14">
@@ -29524,10 +30031,10 @@
         <v>1678</v>
       </c>
       <c r="D81" s="1" t="s">
-        <v>3018</v>
+        <v>3079</v>
       </c>
       <c r="E81" s="1" t="s">
-        <v>3019</v>
+        <v>3080</v>
       </c>
       <c r="F81" s="1" t="s">
         <v>1686</v>
@@ -29554,7 +30061,7 @@
         <v>52</v>
       </c>
       <c r="N81" s="1" t="s">
-        <v>2861</v>
+        <v>2922</v>
       </c>
     </row>
     <row customHeight="1" ht="82.8" r="82" spans="1:14">
@@ -29568,10 +30075,10 @@
         <v>1700</v>
       </c>
       <c r="D82" s="1" t="s">
-        <v>3020</v>
+        <v>3081</v>
       </c>
       <c r="E82" s="1" t="s">
-        <v>3021</v>
+        <v>3082</v>
       </c>
       <c r="F82" s="1" t="s">
         <v>1708</v>
@@ -29598,7 +30105,7 @@
         <v>145</v>
       </c>
       <c r="N82" s="1" t="s">
-        <v>2861</v>
+        <v>2922</v>
       </c>
     </row>
     <row customHeight="1" ht="82.8" r="83" spans="1:14">
@@ -29612,10 +30119,10 @@
         <v>1721</v>
       </c>
       <c r="D83" s="1" t="s">
-        <v>3022</v>
+        <v>3083</v>
       </c>
       <c r="E83" s="1" t="s">
-        <v>3023</v>
+        <v>3084</v>
       </c>
       <c r="F83" s="1" t="s">
         <v>1730</v>
@@ -29642,7 +30149,7 @@
         <v>52</v>
       </c>
       <c r="N83" s="1" t="s">
-        <v>2861</v>
+        <v>2922</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="84" spans="1:14">
@@ -29656,10 +30163,10 @@
         <v>1744</v>
       </c>
       <c r="D84" s="1" t="s">
-        <v>3024</v>
+        <v>3085</v>
       </c>
       <c r="E84" s="1" t="s">
-        <v>3025</v>
+        <v>3086</v>
       </c>
       <c r="F84" s="1" t="s">
         <v>1751</v>
@@ -29686,7 +30193,7 @@
         <v>52</v>
       </c>
       <c r="N84" s="1" t="s">
-        <v>2861</v>
+        <v>2922</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="85" spans="1:14">
@@ -29700,10 +30207,10 @@
         <v>1765</v>
       </c>
       <c r="D85" s="1" t="s">
-        <v>3026</v>
+        <v>3087</v>
       </c>
       <c r="E85" s="1" t="s">
-        <v>3027</v>
+        <v>3088</v>
       </c>
       <c r="F85" s="1" t="s">
         <v>1773</v>
@@ -29730,7 +30237,7 @@
         <v>145</v>
       </c>
       <c r="N85" s="1" t="s">
-        <v>2861</v>
+        <v>2922</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="86" spans="1:14">
@@ -29744,10 +30251,10 @@
         <v>1785</v>
       </c>
       <c r="D86" s="1" t="s">
-        <v>3028</v>
+        <v>3089</v>
       </c>
       <c r="E86" s="1" t="s">
-        <v>3029</v>
+        <v>3090</v>
       </c>
       <c r="F86" s="1" t="s">
         <v>1793</v>
@@ -29774,7 +30281,7 @@
         <v>52</v>
       </c>
       <c r="N86" s="1" t="s">
-        <v>2861</v>
+        <v>2922</v>
       </c>
     </row>
     <row customHeight="1" ht="110.4" r="87" spans="1:14">
@@ -29788,10 +30295,10 @@
         <v>1806</v>
       </c>
       <c r="D87" s="1" t="s">
-        <v>3030</v>
+        <v>3091</v>
       </c>
       <c r="E87" s="1" t="s">
-        <v>3031</v>
+        <v>3092</v>
       </c>
       <c r="F87" s="1" t="s">
         <v>1813</v>
@@ -29818,7 +30325,7 @@
         <v>145</v>
       </c>
       <c r="N87" s="1" t="s">
-        <v>2861</v>
+        <v>2922</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="88" spans="1:14">
@@ -29832,10 +30339,10 @@
         <v>1826</v>
       </c>
       <c r="D88" s="1" t="s">
-        <v>3032</v>
+        <v>3093</v>
       </c>
       <c r="E88" s="1" t="s">
-        <v>3033</v>
+        <v>3094</v>
       </c>
       <c r="F88" s="1" t="s">
         <v>1834</v>
@@ -29862,7 +30369,7 @@
         <v>52</v>
       </c>
       <c r="N88" s="1" t="s">
-        <v>2861</v>
+        <v>2922</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="89" spans="1:14">
@@ -29876,10 +30383,10 @@
         <v>1846</v>
       </c>
       <c r="D89" s="1" t="s">
-        <v>3034</v>
+        <v>3095</v>
       </c>
       <c r="E89" s="1" t="s">
-        <v>3035</v>
+        <v>3096</v>
       </c>
       <c r="F89" s="1" t="s">
         <v>1854</v>
@@ -29906,7 +30413,7 @@
         <v>52</v>
       </c>
       <c r="N89" s="1" t="s">
-        <v>2861</v>
+        <v>2922</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="90" spans="1:14">
@@ -29920,10 +30427,10 @@
         <v>1866</v>
       </c>
       <c r="D90" s="1" t="s">
-        <v>3036</v>
+        <v>3097</v>
       </c>
       <c r="E90" s="1" t="s">
-        <v>3037</v>
+        <v>3098</v>
       </c>
       <c r="F90" s="1" t="s">
         <v>1873</v>
@@ -29950,7 +30457,7 @@
         <v>52</v>
       </c>
       <c r="N90" s="1" t="s">
-        <v>2861</v>
+        <v>2922</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="91" spans="1:14">
@@ -29964,10 +30471,10 @@
         <v>1884</v>
       </c>
       <c r="D91" s="1" t="s">
-        <v>3038</v>
+        <v>3099</v>
       </c>
       <c r="E91" s="1" t="s">
-        <v>3039</v>
+        <v>3100</v>
       </c>
       <c r="F91" s="1" t="s">
         <v>1892</v>
@@ -29994,7 +30501,7 @@
         <v>145</v>
       </c>
       <c r="N91" s="1" t="s">
-        <v>2861</v>
+        <v>2922</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="92" spans="1:14">
@@ -30008,10 +30515,10 @@
         <v>1904</v>
       </c>
       <c r="D92" s="1" t="s">
-        <v>3040</v>
+        <v>3101</v>
       </c>
       <c r="E92" s="1" t="s">
-        <v>3041</v>
+        <v>3102</v>
       </c>
       <c r="F92" s="1" t="s">
         <v>1912</v>
@@ -30038,7 +30545,7 @@
         <v>189</v>
       </c>
       <c r="N92" s="1" t="s">
-        <v>2861</v>
+        <v>2922</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="93" spans="1:14">
@@ -30052,10 +30559,10 @@
         <v>1923</v>
       </c>
       <c r="D93" s="1" t="s">
-        <v>3042</v>
+        <v>3103</v>
       </c>
       <c r="E93" s="1" t="s">
-        <v>3043</v>
+        <v>3104</v>
       </c>
       <c r="F93" s="1" t="s">
         <v>1931</v>
@@ -30082,7 +30589,7 @@
         <v>52</v>
       </c>
       <c r="N93" s="1" t="s">
-        <v>2861</v>
+        <v>2922</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="94" spans="1:14">
@@ -30096,10 +30603,10 @@
         <v>1943</v>
       </c>
       <c r="D94" s="1" t="s">
-        <v>3044</v>
+        <v>3105</v>
       </c>
       <c r="E94" s="1" t="s">
-        <v>3045</v>
+        <v>3106</v>
       </c>
       <c r="F94" s="1" t="s">
         <v>1950</v>
@@ -30126,7 +30633,7 @@
         <v>52</v>
       </c>
       <c r="N94" s="1" t="s">
-        <v>2861</v>
+        <v>2922</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="95" spans="1:14">
@@ -30140,10 +30647,10 @@
         <v>1961</v>
       </c>
       <c r="D95" s="1" t="s">
-        <v>3046</v>
+        <v>3107</v>
       </c>
       <c r="E95" s="1" t="s">
-        <v>3047</v>
+        <v>3108</v>
       </c>
       <c r="F95" s="1" t="s">
         <v>1968</v>
@@ -30170,7 +30677,7 @@
         <v>52</v>
       </c>
       <c r="N95" s="1" t="s">
-        <v>2861</v>
+        <v>2922</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="96" spans="1:14">
@@ -30184,10 +30691,10 @@
         <v>1980</v>
       </c>
       <c r="D96" s="1" t="s">
-        <v>3048</v>
+        <v>3109</v>
       </c>
       <c r="E96" s="1" t="s">
-        <v>3049</v>
+        <v>3110</v>
       </c>
       <c r="F96" s="1" t="s">
         <v>1988</v>
@@ -30214,7 +30721,7 @@
         <v>52</v>
       </c>
       <c r="N96" s="1" t="s">
-        <v>2861</v>
+        <v>2922</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="97" spans="1:14">
@@ -30228,10 +30735,10 @@
         <v>2000</v>
       </c>
       <c r="D97" s="1" t="s">
-        <v>3050</v>
+        <v>3111</v>
       </c>
       <c r="E97" s="1" t="s">
-        <v>3051</v>
+        <v>3112</v>
       </c>
       <c r="F97" s="1" t="s">
         <v>2006</v>
@@ -30258,7 +30765,7 @@
         <v>52</v>
       </c>
       <c r="N97" s="1" t="s">
-        <v>2861</v>
+        <v>2922</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="98" spans="1:14">
@@ -30272,10 +30779,10 @@
         <v>2019</v>
       </c>
       <c r="D98" s="1" t="s">
-        <v>3052</v>
+        <v>3113</v>
       </c>
       <c r="E98" s="1" t="s">
-        <v>3053</v>
+        <v>3114</v>
       </c>
       <c r="F98" s="1" t="s">
         <v>2028</v>
@@ -30302,7 +30809,7 @@
         <v>145</v>
       </c>
       <c r="N98" s="1" t="s">
-        <v>2861</v>
+        <v>2922</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="99" spans="1:14">
@@ -30316,10 +30823,10 @@
         <v>2041</v>
       </c>
       <c r="D99" s="1" t="s">
-        <v>3054</v>
+        <v>3115</v>
       </c>
       <c r="E99" s="1" t="s">
-        <v>3055</v>
+        <v>3116</v>
       </c>
       <c r="F99" s="1" t="s">
         <v>2049</v>
@@ -30346,7 +30853,7 @@
         <v>145</v>
       </c>
       <c r="N99" s="1" t="s">
-        <v>2861</v>
+        <v>2922</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="100" spans="1:14">
@@ -30360,10 +30867,10 @@
         <v>2062</v>
       </c>
       <c r="D100" s="1" t="s">
-        <v>3056</v>
+        <v>3117</v>
       </c>
       <c r="E100" s="1" t="s">
-        <v>3057</v>
+        <v>3118</v>
       </c>
       <c r="F100" s="1" t="s">
         <v>2069</v>
@@ -30390,7 +30897,7 @@
         <v>145</v>
       </c>
       <c r="N100" s="1" t="s">
-        <v>2861</v>
+        <v>2922</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="101" spans="1:14">
@@ -30404,10 +30911,10 @@
         <v>2082</v>
       </c>
       <c r="D101" s="1" t="s">
-        <v>3058</v>
+        <v>3119</v>
       </c>
       <c r="E101" s="1" t="s">
-        <v>3059</v>
+        <v>3120</v>
       </c>
       <c r="F101" s="1" t="s">
         <v>2090</v>
@@ -30434,7 +30941,7 @@
         <v>52</v>
       </c>
       <c r="N101" s="1" t="s">
-        <v>2861</v>
+        <v>2922</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="102" spans="1:14">
@@ -30448,10 +30955,10 @@
         <v>2102</v>
       </c>
       <c r="D102" s="1" t="s">
-        <v>3060</v>
+        <v>3121</v>
       </c>
       <c r="E102" s="1" t="s">
-        <v>3061</v>
+        <v>3122</v>
       </c>
       <c r="F102" s="1" t="s">
         <v>2110</v>
@@ -30478,7 +30985,7 @@
         <v>145</v>
       </c>
       <c r="N102" s="1" t="s">
-        <v>2861</v>
+        <v>2922</v>
       </c>
     </row>
     <row customHeight="1" ht="82.8" r="103" spans="1:14">
@@ -30492,10 +30999,10 @@
         <v>2122</v>
       </c>
       <c r="D103" s="1" t="s">
-        <v>3062</v>
+        <v>3123</v>
       </c>
       <c r="E103" s="1" t="s">
-        <v>3063</v>
+        <v>3124</v>
       </c>
       <c r="F103" s="1" t="s">
         <v>2129</v>
@@ -30522,7 +31029,7 @@
         <v>145</v>
       </c>
       <c r="N103" s="1" t="s">
-        <v>2861</v>
+        <v>2922</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="104" spans="1:14">
@@ -30536,10 +31043,10 @@
         <v>2142</v>
       </c>
       <c r="D104" s="1" t="s">
-        <v>3064</v>
+        <v>3125</v>
       </c>
       <c r="E104" s="1" t="s">
-        <v>3065</v>
+        <v>3126</v>
       </c>
       <c r="F104" s="1" t="s">
         <v>2149</v>
@@ -30566,7 +31073,7 @@
         <v>145</v>
       </c>
       <c r="N104" s="1" t="s">
-        <v>2861</v>
+        <v>2922</v>
       </c>
     </row>
     <row customHeight="1" ht="82.8" r="105" spans="1:14">
@@ -30580,10 +31087,10 @@
         <v>2161</v>
       </c>
       <c r="D105" s="1" t="s">
-        <v>3066</v>
+        <v>3127</v>
       </c>
       <c r="E105" s="1" t="s">
-        <v>3067</v>
+        <v>3128</v>
       </c>
       <c r="F105" s="1" t="s">
         <v>2168</v>
@@ -30610,7 +31117,7 @@
         <v>145</v>
       </c>
       <c r="N105" s="1" t="s">
-        <v>2861</v>
+        <v>2922</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="106" spans="1:14">
@@ -30624,10 +31131,10 @@
         <v>2181</v>
       </c>
       <c r="D106" s="1" t="s">
-        <v>3068</v>
+        <v>3129</v>
       </c>
       <c r="E106" s="1" t="s">
-        <v>3069</v>
+        <v>3130</v>
       </c>
       <c r="F106" s="1" t="s">
         <v>2187</v>
@@ -30654,7 +31161,7 @@
         <v>189</v>
       </c>
       <c r="N106" s="1" t="s">
-        <v>2861</v>
+        <v>2922</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="107" spans="1:14">
@@ -30668,10 +31175,10 @@
         <v>2201</v>
       </c>
       <c r="D107" s="1" t="s">
-        <v>3070</v>
+        <v>3131</v>
       </c>
       <c r="E107" s="1" t="s">
-        <v>3071</v>
+        <v>3132</v>
       </c>
       <c r="F107" s="1" t="s">
         <v>2209</v>
@@ -30698,7 +31205,7 @@
         <v>145</v>
       </c>
       <c r="N107" s="1" t="s">
-        <v>2861</v>
+        <v>2922</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="108" spans="1:14">
@@ -30712,10 +31219,10 @@
         <v>2222</v>
       </c>
       <c r="D108" s="1" t="s">
-        <v>3072</v>
+        <v>3133</v>
       </c>
       <c r="E108" s="1" t="s">
-        <v>3073</v>
+        <v>3134</v>
       </c>
       <c r="F108" s="1" t="s">
         <v>2228</v>
@@ -30742,7 +31249,7 @@
         <v>52</v>
       </c>
       <c r="N108" s="1" t="s">
-        <v>2861</v>
+        <v>2922</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="109" spans="1:14">
@@ -30756,10 +31263,10 @@
         <v>2241</v>
       </c>
       <c r="D109" s="1" t="s">
-        <v>3074</v>
+        <v>3135</v>
       </c>
       <c r="E109" s="1" t="s">
-        <v>3075</v>
+        <v>3136</v>
       </c>
       <c r="F109" s="1" t="s">
         <v>2247</v>
@@ -30786,7 +31293,7 @@
         <v>52</v>
       </c>
       <c r="N109" s="1" t="s">
-        <v>2861</v>
+        <v>2922</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="110" spans="1:14">
@@ -30800,10 +31307,10 @@
         <v>2259</v>
       </c>
       <c r="D110" s="1" t="s">
-        <v>3076</v>
+        <v>3137</v>
       </c>
       <c r="E110" s="1" t="s">
-        <v>3077</v>
+        <v>3138</v>
       </c>
       <c r="F110" s="1" t="s">
         <v>2268</v>
@@ -30830,7 +31337,7 @@
         <v>145</v>
       </c>
       <c r="N110" s="1" t="s">
-        <v>2861</v>
+        <v>2922</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="111" spans="1:14">
@@ -30844,10 +31351,10 @@
         <v>2281</v>
       </c>
       <c r="D111" s="1" t="s">
-        <v>3078</v>
+        <v>3139</v>
       </c>
       <c r="E111" s="1" t="s">
-        <v>3079</v>
+        <v>3140</v>
       </c>
       <c r="F111" s="1" t="s">
         <v>2289</v>
@@ -30874,7 +31381,7 @@
         <v>52</v>
       </c>
       <c r="N111" s="1" t="s">
-        <v>2861</v>
+        <v>2922</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="112" spans="1:14">
@@ -30888,10 +31395,10 @@
         <v>2302</v>
       </c>
       <c r="D112" s="1" t="s">
-        <v>3080</v>
+        <v>3141</v>
       </c>
       <c r="E112" s="1" t="s">
-        <v>3081</v>
+        <v>3142</v>
       </c>
       <c r="F112" s="1" t="s">
         <v>2311</v>
@@ -30918,7 +31425,7 @@
         <v>145</v>
       </c>
       <c r="N112" s="1" t="s">
-        <v>2861</v>
+        <v>2922</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="113" spans="1:14">
@@ -30932,10 +31439,10 @@
         <v>2324</v>
       </c>
       <c r="D113" s="1" t="s">
-        <v>3082</v>
+        <v>3143</v>
       </c>
       <c r="E113" s="1" t="s">
-        <v>3083</v>
+        <v>3144</v>
       </c>
       <c r="F113" s="1" t="s">
         <v>2331</v>
@@ -30962,7 +31469,7 @@
         <v>145</v>
       </c>
       <c r="N113" s="1" t="s">
-        <v>2861</v>
+        <v>2922</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="114" spans="1:14">
@@ -30976,10 +31483,10 @@
         <v>2343</v>
       </c>
       <c r="D114" s="1" t="s">
-        <v>3084</v>
+        <v>3145</v>
       </c>
       <c r="E114" s="1" t="s">
-        <v>3085</v>
+        <v>3146</v>
       </c>
       <c r="F114" s="1" t="s">
         <v>2350</v>
@@ -31006,7 +31513,7 @@
         <v>145</v>
       </c>
       <c r="N114" s="1" t="s">
-        <v>2861</v>
+        <v>2922</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="115" spans="1:14">
@@ -31020,10 +31527,10 @@
         <v>2362</v>
       </c>
       <c r="D115" s="1" t="s">
-        <v>3086</v>
+        <v>3147</v>
       </c>
       <c r="E115" s="1" t="s">
-        <v>3087</v>
+        <v>3148</v>
       </c>
       <c r="F115" s="1" t="s">
         <v>2369</v>
@@ -31050,7 +31557,7 @@
         <v>52</v>
       </c>
       <c r="N115" s="1" t="s">
-        <v>2861</v>
+        <v>2922</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="116" spans="1:14">
@@ -31064,10 +31571,10 @@
         <v>2381</v>
       </c>
       <c r="D116" s="1" t="s">
-        <v>3088</v>
+        <v>3149</v>
       </c>
       <c r="E116" s="1" t="s">
-        <v>3089</v>
+        <v>3150</v>
       </c>
       <c r="F116" s="1" t="s">
         <v>2389</v>
@@ -31094,7 +31601,7 @@
         <v>145</v>
       </c>
       <c r="N116" s="1" t="s">
-        <v>2861</v>
+        <v>2922</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="117" spans="1:14">
@@ -31108,10 +31615,10 @@
         <v>2401</v>
       </c>
       <c r="D117" s="1" t="s">
-        <v>3090</v>
+        <v>3151</v>
       </c>
       <c r="E117" s="1" t="s">
-        <v>3091</v>
+        <v>3152</v>
       </c>
       <c r="F117" s="1" t="s">
         <v>2410</v>
@@ -31138,7 +31645,7 @@
         <v>145</v>
       </c>
       <c r="N117" s="1" t="s">
-        <v>2861</v>
+        <v>2922</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="118" spans="1:14">
@@ -31152,10 +31659,10 @@
         <v>2423</v>
       </c>
       <c r="D118" s="1" t="s">
-        <v>3092</v>
+        <v>3153</v>
       </c>
       <c r="E118" s="1" t="s">
-        <v>3093</v>
+        <v>3154</v>
       </c>
       <c r="F118" s="1" t="s">
         <v>2431</v>
@@ -31182,7 +31689,7 @@
         <v>145</v>
       </c>
       <c r="N118" s="1" t="s">
-        <v>2861</v>
+        <v>2922</v>
       </c>
     </row>
     <row customHeight="1" ht="96.59999999999999" r="119" spans="1:14">
@@ -31196,10 +31703,10 @@
         <v>2443</v>
       </c>
       <c r="D119" s="1" t="s">
-        <v>3094</v>
+        <v>3155</v>
       </c>
       <c r="E119" s="1" t="s">
-        <v>3095</v>
+        <v>3156</v>
       </c>
       <c r="F119" s="1" t="s">
         <v>2450</v>
@@ -31226,7 +31733,7 @@
         <v>52</v>
       </c>
       <c r="N119" s="1" t="s">
-        <v>2861</v>
+        <v>2922</v>
       </c>
     </row>
     <row customHeight="1" ht="82.8" r="120" spans="1:14">
@@ -31240,10 +31747,10 @@
         <v>2462</v>
       </c>
       <c r="D120" s="1" t="s">
-        <v>3096</v>
+        <v>3157</v>
       </c>
       <c r="E120" s="1" t="s">
-        <v>3097</v>
+        <v>3158</v>
       </c>
       <c r="F120" s="1" t="s">
         <v>2470</v>
@@ -31270,7 +31777,7 @@
         <v>145</v>
       </c>
       <c r="N120" s="1" t="s">
-        <v>3098</v>
+        <v>3159</v>
       </c>
     </row>
     <row customHeight="1" ht="82.8" r="121" spans="1:14">
@@ -31284,10 +31791,10 @@
         <v>2483</v>
       </c>
       <c r="D121" s="1" t="s">
-        <v>3099</v>
+        <v>3160</v>
       </c>
       <c r="E121" s="1" t="s">
-        <v>3100</v>
+        <v>3161</v>
       </c>
       <c r="F121" s="1" t="s">
         <v>2492</v>
@@ -31314,7 +31821,7 @@
         <v>145</v>
       </c>
       <c r="N121" s="1" t="s">
-        <v>3098</v>
+        <v>3159</v>
       </c>
     </row>
     <row customHeight="1" ht="82.8" r="122" spans="1:14">
@@ -31328,10 +31835,10 @@
         <v>2503</v>
       </c>
       <c r="D122" s="1" t="s">
-        <v>3101</v>
+        <v>3162</v>
       </c>
       <c r="E122" s="1" t="s">
-        <v>3102</v>
+        <v>3163</v>
       </c>
       <c r="F122" s="1" t="s">
         <v>2508</v>
@@ -31358,7 +31865,7 @@
         <v>52</v>
       </c>
       <c r="N122" s="1" t="s">
-        <v>3098</v>
+        <v>3159</v>
       </c>
     </row>
     <row r="123" spans="1:14">
@@ -31372,10 +31879,10 @@
         <v>2521</v>
       </c>
       <c r="D123" t="s">
-        <v>3103</v>
+        <v>3164</v>
       </c>
       <c r="E123" t="s">
-        <v>3104</v>
+        <v>3165</v>
       </c>
       <c r="F123" t="s">
         <v>2528</v>
@@ -31402,7 +31909,7 @@
         <v>52</v>
       </c>
       <c r="N123" t="s">
-        <v>3098</v>
+        <v>3159</v>
       </c>
     </row>
     <row r="124" spans="1:14">
@@ -31419,7 +31926,7 @@
         <v>2546</v>
       </c>
       <c r="E124" t="s">
-        <v>3105</v>
+        <v>3166</v>
       </c>
       <c r="F124" t="s">
         <v>2547</v>
@@ -31446,7 +31953,7 @@
         <v>52</v>
       </c>
       <c r="N124" t="s">
-        <v>3098</v>
+        <v>3159</v>
       </c>
     </row>
     <row r="125" spans="1:14">
@@ -31463,7 +31970,7 @@
         <v>2564</v>
       </c>
       <c r="E125" t="s">
-        <v>3106</v>
+        <v>3167</v>
       </c>
       <c r="F125" t="s">
         <v>2565</v>
@@ -31490,7 +31997,7 @@
         <v>189</v>
       </c>
       <c r="N125" t="s">
-        <v>3098</v>
+        <v>3159</v>
       </c>
     </row>
     <row r="126" spans="1:14">
@@ -31507,7 +32014,7 @@
         <v>2582</v>
       </c>
       <c r="E126" t="s">
-        <v>3107</v>
+        <v>3168</v>
       </c>
       <c r="F126" t="s">
         <v>2585</v>
@@ -31531,10 +32038,10 @@
         <v>2590</v>
       </c>
       <c r="M126" t="s">
-        <v>3108</v>
+        <v>3169</v>
       </c>
       <c r="N126" t="s">
-        <v>3098</v>
+        <v>3159</v>
       </c>
     </row>
     <row r="127" spans="1:14">
@@ -31551,7 +32058,7 @@
         <v>2601</v>
       </c>
       <c r="E127" t="s">
-        <v>3109</v>
+        <v>3170</v>
       </c>
       <c r="F127" t="s">
         <v>2603</v>
@@ -31578,7 +32085,7 @@
         <v>52</v>
       </c>
       <c r="N127" t="s">
-        <v>3098</v>
+        <v>3159</v>
       </c>
     </row>
     <row r="128" spans="1:14">
@@ -31592,10 +32099,10 @@
         <v>2614</v>
       </c>
       <c r="D128" t="s">
-        <v>3110</v>
+        <v>3171</v>
       </c>
       <c r="E128" t="s">
-        <v>3111</v>
+        <v>3172</v>
       </c>
       <c r="F128" t="s">
         <v>2620</v>
@@ -31619,10 +32126,10 @@
         <v>2626</v>
       </c>
       <c r="M128" t="s">
-        <v>3108</v>
+        <v>3169</v>
       </c>
       <c r="N128" t="s">
-        <v>3098</v>
+        <v>3159</v>
       </c>
     </row>
     <row r="129" spans="1:14">
@@ -31636,10 +32143,10 @@
         <v>2632</v>
       </c>
       <c r="D129" t="s">
-        <v>3112</v>
+        <v>3173</v>
       </c>
       <c r="E129" t="s">
-        <v>3113</v>
+        <v>3174</v>
       </c>
       <c r="F129" t="s">
         <v>2638</v>
@@ -31666,7 +32173,7 @@
         <v>52</v>
       </c>
       <c r="N129" t="s">
-        <v>3098</v>
+        <v>3159</v>
       </c>
     </row>
     <row r="130" spans="1:14">
@@ -31680,10 +32187,10 @@
         <v>2650</v>
       </c>
       <c r="D130" t="s">
-        <v>3114</v>
+        <v>3175</v>
       </c>
       <c r="E130" t="s">
-        <v>3115</v>
+        <v>3176</v>
       </c>
       <c r="F130" t="s">
         <v>2657</v>
@@ -31710,7 +32217,7 @@
         <v>52</v>
       </c>
       <c r="N130" t="s">
-        <v>3098</v>
+        <v>3159</v>
       </c>
     </row>
     <row r="131" spans="1:14">
@@ -31727,7 +32234,7 @@
         <v>2673</v>
       </c>
       <c r="E131" t="s">
-        <v>3116</v>
+        <v>3177</v>
       </c>
       <c r="F131" t="s">
         <v>2675</v>
@@ -31754,7 +32261,7 @@
         <v>52</v>
       </c>
       <c r="N131" t="s">
-        <v>3098</v>
+        <v>3159</v>
       </c>
     </row>
     <row r="132" spans="1:14">
@@ -31768,10 +32275,10 @@
         <v>2687</v>
       </c>
       <c r="D132" t="s">
-        <v>3117</v>
+        <v>3178</v>
       </c>
       <c r="E132" t="s">
-        <v>3118</v>
+        <v>3179</v>
       </c>
       <c r="F132" t="s">
         <v>2694</v>
@@ -31798,7 +32305,7 @@
         <v>52</v>
       </c>
       <c r="N132" t="s">
-        <v>3098</v>
+        <v>3159</v>
       </c>
     </row>
     <row r="133" spans="1:14">
@@ -31812,10 +32319,10 @@
         <v>2705</v>
       </c>
       <c r="D133" t="s">
-        <v>3119</v>
+        <v>3180</v>
       </c>
       <c r="E133" t="s">
-        <v>3120</v>
+        <v>3181</v>
       </c>
       <c r="F133" t="s">
         <v>2711</v>
@@ -31842,7 +32349,7 @@
         <v>52</v>
       </c>
       <c r="N133" t="s">
-        <v>3098</v>
+        <v>3159</v>
       </c>
     </row>
     <row r="134" spans="1:14">
@@ -31856,10 +32363,10 @@
         <v>2722</v>
       </c>
       <c r="D134" t="s">
-        <v>3121</v>
+        <v>3182</v>
       </c>
       <c r="E134" t="s">
-        <v>3122</v>
+        <v>3183</v>
       </c>
       <c r="F134" t="s">
         <v>2730</v>
@@ -31886,7 +32393,7 @@
         <v>52</v>
       </c>
       <c r="N134" t="s">
-        <v>3098</v>
+        <v>3159</v>
       </c>
     </row>
     <row r="135" spans="1:14">
@@ -31900,10 +32407,10 @@
         <v>2744</v>
       </c>
       <c r="D135" t="s">
-        <v>3123</v>
+        <v>3184</v>
       </c>
       <c r="E135" t="s">
-        <v>3124</v>
+        <v>3185</v>
       </c>
       <c r="F135" t="s">
         <v>2753</v>
@@ -31930,7 +32437,7 @@
         <v>52</v>
       </c>
       <c r="N135" t="s">
-        <v>3098</v>
+        <v>3159</v>
       </c>
     </row>
     <row r="136" spans="1:14">
@@ -31944,10 +32451,10 @@
         <v>2765</v>
       </c>
       <c r="D136" t="s">
-        <v>3125</v>
+        <v>3186</v>
       </c>
       <c r="E136" t="s">
-        <v>3126</v>
+        <v>3187</v>
       </c>
       <c r="F136" t="s">
         <v>2774</v>
@@ -31962,7 +32469,7 @@
         <v>2777</v>
       </c>
       <c r="J136" t="s">
-        <v>3127</v>
+        <v>3188</v>
       </c>
       <c r="K136" t="s">
         <v>2779</v>
@@ -31974,7 +32481,7 @@
         <v>52</v>
       </c>
       <c r="N136" t="s">
-        <v>3098</v>
+        <v>3159</v>
       </c>
     </row>
     <row r="137" spans="1:14">
@@ -31988,10 +32495,10 @@
         <v>2788</v>
       </c>
       <c r="D137" t="s">
-        <v>3128</v>
+        <v>3189</v>
       </c>
       <c r="E137" t="s">
-        <v>3129</v>
+        <v>3190</v>
       </c>
       <c r="F137" t="s">
         <v>2795</v>
@@ -32006,7 +32513,7 @@
         <v>2798</v>
       </c>
       <c r="J137" t="s">
-        <v>3130</v>
+        <v>3191</v>
       </c>
       <c r="K137" t="s">
         <v>2800</v>
@@ -32018,7 +32525,139 @@
         <v>52</v>
       </c>
       <c r="N137" t="s">
-        <v>3098</v>
+        <v>3159</v>
+      </c>
+    </row>
+    <row r="138" spans="1:14">
+      <c r="A138" t="s">
+        <v>2804</v>
+      </c>
+      <c r="B138" t="s">
+        <v>31</v>
+      </c>
+      <c r="C138" t="s">
+        <v>3192</v>
+      </c>
+      <c r="D138" t="s">
+        <v>3193</v>
+      </c>
+      <c r="E138" t="s">
+        <v>3194</v>
+      </c>
+      <c r="F138" t="s">
+        <v>2815</v>
+      </c>
+      <c r="G138" t="s">
+        <v>2816</v>
+      </c>
+      <c r="H138" t="s">
+        <v>2817</v>
+      </c>
+      <c r="I138" t="s">
+        <v>2818</v>
+      </c>
+      <c r="J138" t="s">
+        <v>3195</v>
+      </c>
+      <c r="K138" t="s">
+        <v>2820</v>
+      </c>
+      <c r="L138" t="s">
+        <v>2821</v>
+      </c>
+      <c r="M138" t="s">
+        <v>52</v>
+      </c>
+      <c r="N138" t="s">
+        <v>3159</v>
+      </c>
+    </row>
+    <row r="139" spans="1:14">
+      <c r="A139" t="s">
+        <v>2824</v>
+      </c>
+      <c r="B139" t="s">
+        <v>31</v>
+      </c>
+      <c r="C139" t="s">
+        <v>2828</v>
+      </c>
+      <c r="D139" t="s">
+        <v>3196</v>
+      </c>
+      <c r="E139" t="s">
+        <v>3197</v>
+      </c>
+      <c r="F139" t="s">
+        <v>2835</v>
+      </c>
+      <c r="G139" t="s">
+        <v>2836</v>
+      </c>
+      <c r="H139" t="s">
+        <v>2837</v>
+      </c>
+      <c r="I139" t="s">
+        <v>2838</v>
+      </c>
+      <c r="J139" t="s">
+        <v>3198</v>
+      </c>
+      <c r="K139" t="s">
+        <v>2840</v>
+      </c>
+      <c r="L139" t="s">
+        <v>2841</v>
+      </c>
+      <c r="M139" t="s">
+        <v>52</v>
+      </c>
+      <c r="N139" t="s">
+        <v>3159</v>
+      </c>
+    </row>
+    <row r="140" spans="1:14">
+      <c r="A140" t="s">
+        <v>2844</v>
+      </c>
+      <c r="B140" t="s">
+        <v>31</v>
+      </c>
+      <c r="C140" t="s">
+        <v>2848</v>
+      </c>
+      <c r="D140" t="s">
+        <v>3199</v>
+      </c>
+      <c r="E140" t="s">
+        <v>3200</v>
+      </c>
+      <c r="F140" t="s">
+        <v>2856</v>
+      </c>
+      <c r="G140" t="s">
+        <v>2857</v>
+      </c>
+      <c r="H140" t="s">
+        <v>2858</v>
+      </c>
+      <c r="I140" t="s">
+        <v>2859</v>
+      </c>
+      <c r="J140" t="s">
+        <v>3201</v>
+      </c>
+      <c r="K140" t="s">
+        <v>2861</v>
+      </c>
+      <c r="L140" t="s">
+        <v>2862</v>
+      </c>
+      <c r="M140" t="s">
+        <v>52</v>
+      </c>
+      <c r="N140" t="s">
+        <v>3159</v>
       </c>
     </row>
   </sheetData>
@@ -32032,7 +32671,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B14"/>
+  <dimension ref="A1:B15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="13.8" outlineLevelCol="0"/>
   <cols>
     <col customWidth="1" max="1" min="1" width="50"/>
@@ -32041,114 +32680,122 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="7" t="s">
-        <v>3131</v>
+        <v>3202</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>3132</v>
+        <v>3203</v>
       </c>
     </row>
     <row r="2" spans="1:2">
       <c r="A2" t="s">
-        <v>3133</v>
+        <v>3204</v>
       </c>
       <c r="B2" t="s">
-        <v>2813</v>
+        <v>2874</v>
       </c>
     </row>
     <row r="3" spans="1:2">
       <c r="A3" t="s">
-        <v>3134</v>
+        <v>3205</v>
       </c>
       <c r="B3" t="s">
-        <v>3135</v>
+        <v>3206</v>
       </c>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" t="s">
-        <v>3136</v>
+        <v>3207</v>
       </c>
       <c r="B4" t="s">
-        <v>3137</v>
+        <v>3208</v>
       </c>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" t="s">
-        <v>3138</v>
+        <v>3209</v>
       </c>
       <c r="B5" t="s">
-        <v>3139</v>
+        <v>3210</v>
       </c>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" t="s">
-        <v>3140</v>
+        <v>3211</v>
       </c>
       <c r="B6" t="s">
-        <v>3141</v>
+        <v>3212</v>
       </c>
     </row>
     <row r="7" spans="1:2">
       <c r="A7" t="s">
-        <v>3142</v>
+        <v>3213</v>
       </c>
       <c r="B7" t="s">
-        <v>3143</v>
+        <v>3214</v>
       </c>
     </row>
     <row r="8" spans="1:2">
       <c r="A8" t="s">
-        <v>3144</v>
+        <v>3215</v>
       </c>
       <c r="B8" t="s">
-        <v>3145</v>
+        <v>3216</v>
       </c>
     </row>
     <row r="9" spans="1:2">
       <c r="A9" t="s">
-        <v>3146</v>
+        <v>3217</v>
       </c>
       <c r="B9" t="s">
-        <v>3147</v>
+        <v>3218</v>
       </c>
     </row>
     <row r="10" spans="1:2">
       <c r="A10" t="s">
-        <v>3148</v>
+        <v>3219</v>
       </c>
       <c r="B10" t="s">
-        <v>3149</v>
+        <v>3220</v>
       </c>
     </row>
     <row r="11" spans="1:2">
       <c r="A11" t="s">
-        <v>3150</v>
+        <v>3221</v>
       </c>
       <c r="B11" t="s">
-        <v>3151</v>
+        <v>3222</v>
       </c>
     </row>
     <row r="12" spans="1:2">
       <c r="A12" t="s">
-        <v>3152</v>
+        <v>3223</v>
       </c>
       <c r="B12" t="s">
-        <v>3153</v>
+        <v>3224</v>
       </c>
     </row>
     <row r="13" spans="1:2">
       <c r="A13" t="s">
-        <v>3154</v>
+        <v>3225</v>
       </c>
       <c r="B13" t="s">
-        <v>3155</v>
+        <v>3226</v>
       </c>
     </row>
     <row r="14" spans="1:2">
       <c r="A14" t="s">
-        <v>3156</v>
+        <v>3227</v>
       </c>
       <c r="B14" t="s">
-        <v>3157</v>
+        <v>3228</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2">
+      <c r="A15" t="s">
+        <v>3229</v>
+      </c>
+      <c r="B15" t="s">
+        <v>3230</v>
       </c>
     </row>
   </sheetData>
@@ -32167,82 +32814,82 @@
   <sheetData>
     <row customHeight="1" ht="27.6" r="1" spans="1:6">
       <c r="A1" s="6" t="s">
-        <v>3158</v>
+        <v>3231</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>3159</v>
+        <v>3232</v>
       </c>
       <c r="C1" s="6" t="s">
-        <v>3160</v>
+        <v>3233</v>
       </c>
       <c r="D1" s="6" t="s">
-        <v>3161</v>
+        <v>3234</v>
       </c>
       <c r="E1" s="6" t="s">
-        <v>3162</v>
+        <v>3235</v>
       </c>
       <c r="F1" s="6" t="s">
-        <v>3163</v>
+        <v>3236</v>
       </c>
     </row>
     <row customHeight="1" ht="55.2" r="2" spans="1:6">
       <c r="A2" s="1" t="s">
-        <v>3164</v>
+        <v>3237</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>38</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>3165</v>
+        <v>3238</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>3166</v>
+        <v>3239</v>
       </c>
       <c r="E2" s="1" t="s">
         <v>28</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>3167</v>
+        <v>3240</v>
       </c>
     </row>
     <row customHeight="1" ht="55.2" r="3" spans="1:6">
       <c r="A3" s="1" t="s">
-        <v>3168</v>
+        <v>3241</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>1681</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>3165</v>
+        <v>3238</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>3166</v>
+        <v>3239</v>
       </c>
       <c r="E3" s="1" t="s">
         <v>1674</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>3167</v>
+        <v>3240</v>
       </c>
     </row>
     <row customHeight="1" ht="55.2" r="4" spans="1:6">
       <c r="A4" s="1" t="s">
-        <v>3169</v>
+        <v>3242</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>1167</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>3165</v>
+        <v>3238</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>3166</v>
+        <v>3239</v>
       </c>
       <c r="E4" s="1" t="s">
         <v>1161</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>3167</v>
+        <v>3240</v>
       </c>
     </row>
     <row customHeight="1" ht="82.8" r="5" spans="1:6">
@@ -32253,16 +32900,16 @@
         <v>2204</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>3170</v>
+        <v>3243</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>3171</v>
+        <v>3244</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>3172</v>
+        <v>3245</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>3173</v>
+        <v>3246</v>
       </c>
     </row>
     <row customHeight="1" ht="82.8" r="6" spans="1:6">
@@ -32273,16 +32920,16 @@
         <v>2223</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>3170</v>
+        <v>3243</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>3171</v>
+        <v>3244</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>3172</v>
+        <v>3245</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>3173</v>
+        <v>3246</v>
       </c>
     </row>
     <row customHeight="1" ht="82.8" r="7" spans="1:6">
@@ -32293,16 +32940,16 @@
         <v>2243</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>3170</v>
+        <v>3243</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>3171</v>
+        <v>3244</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>3172</v>
+        <v>3245</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>3173</v>
+        <v>3246</v>
       </c>
     </row>
     <row customHeight="1" ht="82.8" r="8" spans="1:6">
@@ -32313,16 +32960,16 @@
         <v>2262</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>3170</v>
+        <v>3243</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>3171</v>
+        <v>3244</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>3172</v>
+        <v>3245</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>3173</v>
+        <v>3246</v>
       </c>
     </row>
     <row customHeight="1" ht="82.8" r="9" spans="1:6">
@@ -32333,16 +32980,16 @@
         <v>2283</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>3170</v>
+        <v>3243</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>3171</v>
+        <v>3244</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>3172</v>
+        <v>3245</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>3173</v>
+        <v>3246</v>
       </c>
     </row>
     <row customHeight="1" ht="82.8" r="10" spans="1:6">
@@ -32353,16 +33000,16 @@
         <v>2305</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>3170</v>
+        <v>3243</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>3171</v>
+        <v>3244</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>3172</v>
+        <v>3245</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>3173</v>
+        <v>3246</v>
       </c>
     </row>
     <row customHeight="1" ht="82.8" r="11" spans="1:6">
@@ -32373,16 +33020,16 @@
         <v>2326</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>3170</v>
+        <v>3243</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>3171</v>
+        <v>3244</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>3172</v>
+        <v>3245</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>3173</v>
+        <v>3246</v>
       </c>
     </row>
     <row customHeight="1" ht="82.8" r="12" spans="1:6">
@@ -32393,16 +33040,16 @@
         <v>2346</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>3170</v>
+        <v>3243</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>3171</v>
+        <v>3244</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>3172</v>
+        <v>3245</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>3173</v>
+        <v>3246</v>
       </c>
     </row>
     <row customHeight="1" ht="82.8" r="13" spans="1:6">
@@ -32413,16 +33060,16 @@
         <v>2364</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>3170</v>
+        <v>3243</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>3171</v>
+        <v>3244</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>3172</v>
+        <v>3245</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>3173</v>
+        <v>3246</v>
       </c>
     </row>
     <row customHeight="1" ht="82.8" r="14" spans="1:6">
@@ -32433,16 +33080,16 @@
         <v>2383</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>3170</v>
+        <v>3243</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>3171</v>
+        <v>3244</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>3172</v>
+        <v>3245</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>3173</v>
+        <v>3246</v>
       </c>
     </row>
     <row customHeight="1" ht="82.8" r="15" spans="1:6">
@@ -32453,16 +33100,16 @@
         <v>2404</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>3170</v>
+        <v>3243</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>3171</v>
+        <v>3244</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>3172</v>
+        <v>3245</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>3173</v>
+        <v>3246</v>
       </c>
     </row>
     <row customHeight="1" ht="82.8" r="16" spans="1:6">
@@ -32473,16 +33120,16 @@
         <v>2425</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>3170</v>
+        <v>3243</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>3171</v>
+        <v>3244</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>3172</v>
+        <v>3245</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>3173</v>
+        <v>3246</v>
       </c>
     </row>
     <row customHeight="1" ht="82.8" r="17" spans="1:6">
@@ -32493,96 +33140,96 @@
         <v>2445</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>3170</v>
+        <v>3243</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>3171</v>
+        <v>3244</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>3172</v>
+        <v>3245</v>
       </c>
       <c r="F17" s="1" t="s">
-        <v>3173</v>
+        <v>3246</v>
       </c>
     </row>
     <row customHeight="1" ht="303.6" r="18" spans="1:6">
       <c r="A18" s="1" t="s">
-        <v>3174</v>
+        <v>3247</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>3175</v>
+        <v>3248</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>3165</v>
+        <v>3238</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>3176</v>
+        <v>3249</v>
       </c>
       <c r="E18" s="1" t="s">
         <v>610</v>
       </c>
       <c r="F18" s="1" t="s">
-        <v>3177</v>
+        <v>3250</v>
       </c>
     </row>
     <row customHeight="1" ht="276" r="19" spans="1:6">
       <c r="A19" s="1" t="s">
-        <v>3178</v>
+        <v>3251</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>3179</v>
+        <v>3252</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>3180</v>
+        <v>3253</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>3181</v>
+        <v>3254</v>
       </c>
       <c r="E19" s="1" t="s">
         <v>2458</v>
       </c>
       <c r="F19" s="1" t="s">
-        <v>3170</v>
+        <v>3243</v>
       </c>
     </row>
     <row customHeight="1" ht="193.2" r="20" spans="1:6">
       <c r="A20" s="1" t="s">
-        <v>3182</v>
+        <v>3255</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>3183</v>
+        <v>3256</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>3180</v>
+        <v>3253</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>3181</v>
+        <v>3254</v>
       </c>
       <c r="E20" s="1" t="s">
         <v>2479</v>
       </c>
       <c r="F20" s="1" t="s">
-        <v>3170</v>
+        <v>3243</v>
       </c>
     </row>
     <row customHeight="1" ht="276" r="21" spans="1:6">
       <c r="A21" s="1" t="s">
-        <v>3184</v>
+        <v>3257</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>3185</v>
+        <v>3258</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>3180</v>
+        <v>3253</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>3181</v>
+        <v>3254</v>
       </c>
       <c r="E21" s="1" t="s">
         <v>2500</v>
       </c>
       <c r="F21" s="1" t="s">
-        <v>3170</v>
+        <v>3243</v>
       </c>
     </row>
   </sheetData>
@@ -32596,7 +33243,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B14"/>
+  <dimension ref="A1:B15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="13.8" outlineLevelCol="0"/>
   <cols>
     <col customWidth="1" max="2" min="1" width="42"/>
@@ -32604,15 +33251,15 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="8" t="s">
-        <v>3186</v>
+        <v>3259</v>
       </c>
       <c r="B1" s="8" t="s">
-        <v>3187</v>
+        <v>3260</v>
       </c>
     </row>
     <row r="2" spans="1:2">
       <c r="A2" t="s">
-        <v>3188</v>
+        <v>3261</v>
       </c>
       <c r="B2" t="n">
         <v>118</v>
@@ -32620,7 +33267,7 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" t="s">
-        <v>3189</v>
+        <v>3262</v>
       </c>
       <c r="B3" t="n">
         <v>1</v>
@@ -32628,7 +33275,7 @@
     </row>
     <row r="4" spans="1:2">
       <c r="A4" t="s">
-        <v>3190</v>
+        <v>3263</v>
       </c>
       <c r="B4" t="n">
         <v>0</v>
@@ -32636,7 +33283,7 @@
     </row>
     <row r="5" spans="1:2">
       <c r="A5" t="s">
-        <v>3191</v>
+        <v>3264</v>
       </c>
       <c r="B5" t="s">
         <v>2440</v>
@@ -32644,74 +33291,82 @@
     </row>
     <row r="6" spans="1:2">
       <c r="A6" t="s">
-        <v>3192</v>
+        <v>3265</v>
       </c>
       <c r="B6" t="s">
-        <v>3193</v>
+        <v>3266</v>
       </c>
     </row>
     <row r="7" spans="1:2">
       <c r="A7" t="s">
-        <v>3194</v>
+        <v>3267</v>
       </c>
       <c r="B7" t="s">
-        <v>3195</v>
+        <v>3268</v>
       </c>
     </row>
     <row r="8" spans="1:2">
       <c r="A8" t="s">
-        <v>3196</v>
+        <v>3269</v>
       </c>
       <c r="B8" t="s">
-        <v>3197</v>
+        <v>3270</v>
       </c>
     </row>
     <row r="9" spans="1:2">
       <c r="A9" t="s">
-        <v>3198</v>
+        <v>3271</v>
       </c>
       <c r="B9" t="s">
-        <v>3199</v>
+        <v>3272</v>
       </c>
     </row>
     <row r="10" spans="1:2">
       <c r="A10" t="s">
-        <v>3148</v>
+        <v>3219</v>
       </c>
       <c r="B10" t="s">
-        <v>3149</v>
+        <v>3220</v>
       </c>
     </row>
     <row r="11" spans="1:2">
       <c r="A11" t="s">
-        <v>3200</v>
+        <v>3273</v>
       </c>
       <c r="B11" t="s">
-        <v>3195</v>
+        <v>3268</v>
       </c>
     </row>
     <row r="12" spans="1:2">
       <c r="A12" t="s">
-        <v>3201</v>
+        <v>3274</v>
       </c>
       <c r="B12" t="s">
-        <v>3202</v>
+        <v>3275</v>
       </c>
     </row>
     <row r="13" spans="1:2">
       <c r="A13" t="s">
-        <v>3203</v>
+        <v>3276</v>
       </c>
       <c r="B13" t="s">
-        <v>3204</v>
+        <v>3277</v>
       </c>
     </row>
     <row r="14" spans="1:2">
       <c r="A14" t="s">
-        <v>3205</v>
+        <v>3278</v>
       </c>
       <c r="B14" t="s">
-        <v>3206</v>
+        <v>3279</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2">
+      <c r="A15" t="s">
+        <v>3280</v>
+      </c>
+      <c r="B15" t="s">
+        <v>3275</v>
       </c>
     </row>
   </sheetData>

</xml_diff>